<commit_message>
Import completed inference results and prepare paired-seed Lightning finals
</commit_message>
<xml_diff>
--- a/results.xlsx
+++ b/results.xlsx
@@ -2,10 +2,13 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Backbones" sheetId="1" r:id="R53346bd5de0c437d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Training" sheetId="2" r:id="R1e36755468fd480c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Inference" sheetId="3" r:id="R448cae5ea50c4a35"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Latency" sheetId="4" r:id="R6bb867979508431f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Backbones" sheetId="1" r:id="R53d35f168295427e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Training" sheetId="2" r:id="Ra9d2e6141fd643eb"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Inference" sheetId="3" r:id="R5c97a44c9374414f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Latency" sheetId="4" r:id="Rb3fe4bd9c7894eed"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="5" r:id="R5e78d8ee7b494b23"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Final" sheetId="6" r:id="R0a8ccc05fdcd4087"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="PerClass" sheetId="7" r:id="R6505d689bf0e4acb"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -55,7 +58,7 @@
       <x:name val="Arial"/>
     </x:font>
   </x:fonts>
-  <x:fills count="8">
+  <x:fills count="10">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -92,6 +95,16 @@
         <x:fgColor rgb="FF243B53"/>
       </x:patternFill>
     </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF243B53"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFE4F0E9"/>
+      </x:patternFill>
+    </x:fill>
   </x:fills>
   <x:borders count="1">
     <x:border/>
@@ -99,7 +112,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="45">
+  <x:cellXfs count="57">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyAlignment="1">
       <x:alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -229,6 +242,55 @@
       <x:alignment vertical="center"/>
     </x:xf>
     <x:xf numFmtId="207" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="8" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="8" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="8" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="8" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
+      <x:extLst>
+        <x:ext uri="{C7286773-470A-42A8-94C5-96B5CB345126}">
+          <xfpb:xfComplement xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" i="0"/>
+        </x:ext>
+      </x:extLst>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1">
+      <x:extLst>
+        <x:ext uri="{C7286773-470A-42A8-94C5-96B5CB345126}">
+          <xfpb:xfComplement xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" i="0"/>
+        </x:ext>
+      </x:extLst>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+      <x:extLst>
+        <x:ext uri="{C7286773-470A-42A8-94C5-96B5CB345126}">
+          <xfpb:xfComplement xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" i="0"/>
+        </x:ext>
+      </x:extLst>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="9" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="9" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="3" fillId="9" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="205" fontId="3" fillId="9" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="164" fontId="3" fillId="9" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="center"/>
     </x:xf>
   </x:cellXfs>
@@ -336,6 +398,23 @@
     </x:indexedColors>
   </x:colors>
 </x:styleSheet>
+</file>
+
+<file path=xl/featurePropertyBag/featurePropertyBag.xml><?xml version="1.0" encoding="utf-8"?>
+<xfpb:FeaturePropertyBags xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag">
+  <xfpb:bag type="Checkbox"/>
+  <xfpb:bag type="XFControls">
+    <xfpb:bagId k="CellControl">0</xfpb:bagId>
+  </xfpb:bag>
+  <xfpb:bag type="XFComplement">
+    <xfpb:bagId k="XFControls">1</xfpb:bagId>
+  </xfpb:bag>
+  <xfpb:bag type="XFComplements" extRef="XFComplementsMapperExtRef">
+    <xfpb:a k="MappedFeaturePropertyBags">
+      <xfpb:bagId>2</xfpb:bagId>
+    </xfpb:a>
+  </xfpb:bag>
+</xfpb:FeaturePropertyBags>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1933,67 +2012,67 @@
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="45" customHeight="1">
-      <x:c r="A1" s="38" t="str">
+      <x:c r="A1" s="48" t="str">
         <x:v>exp_id</x:v>
       </x:c>
-      <x:c r="B1" s="38" t="str">
+      <x:c r="B1" s="48" t="str">
         <x:v>Phương pháp</x:v>
       </x:c>
-      <x:c r="C1" s="38" t="str">
+      <x:c r="C1" s="48" t="str">
         <x:v>Checkpoint</x:v>
       </x:c>
-      <x:c r="D1" s="38" t="str">
+      <x:c r="D1" s="48" t="str">
         <x:v>K</x:v>
       </x:c>
-      <x:c r="E1" s="38" t="str">
+      <x:c r="E1" s="48" t="str">
         <x:v>Crop size</x:v>
       </x:c>
-      <x:c r="F1" s="38" t="str">
+      <x:c r="F1" s="48" t="str">
         <x:v>Input size</x:v>
       </x:c>
-      <x:c r="G1" s="38" t="str">
+      <x:c r="G1" s="48" t="str">
         <x:v>dtype</x:v>
       </x:c>
-      <x:c r="H1" s="38" t="str">
+      <x:c r="H1" s="48" t="str">
         <x:v>Gộp view</x:v>
       </x:c>
-      <x:c r="I1" s="38" t="str">
+      <x:c r="I1" s="48" t="str">
         <x:v>Temperature T</x:v>
       </x:c>
-      <x:c r="J1" s="38" t="str">
+      <x:c r="J1" s="48" t="str">
         <x:v>Macro-F1 val</x:v>
       </x:c>
-      <x:c r="K1" s="38" t="str">
+      <x:c r="K1" s="48" t="str">
         <x:v>Top-1 val</x:v>
       </x:c>
-      <x:c r="L1" s="38" t="str">
+      <x:c r="L1" s="48" t="str">
         <x:v>ECE val</x:v>
       </x:c>
-      <x:c r="M1" s="38" t="str">
+      <x:c r="M1" s="48" t="str">
         <x:v>NLL val</x:v>
       </x:c>
-      <x:c r="N1" s="38" t="str">
+      <x:c r="N1" s="48" t="str">
         <x:v>p50 (ms)</x:v>
       </x:c>
-      <x:c r="O1" s="38" t="str">
+      <x:c r="O1" s="48" t="str">
         <x:v>p95 (ms)</x:v>
       </x:c>
-      <x:c r="P1" s="38" t="str">
+      <x:c r="P1" s="48" t="str">
         <x:v>p99 (ms)</x:v>
       </x:c>
-      <x:c r="Q1" s="38" t="str">
+      <x:c r="Q1" s="48" t="str">
         <x:v>Chi phí × I00</x:v>
       </x:c>
-      <x:c r="R1" s="38" t="str">
+      <x:c r="R1" s="48" t="str">
         <x:v>Ảnh/s batch 32</x:v>
       </x:c>
-      <x:c r="S1" s="38" t="str">
+      <x:c r="S1" s="48" t="str">
         <x:v>p95 ≤ 100 ms</x:v>
       </x:c>
-      <x:c r="T1" s="38" t="str">
+      <x:c r="T1" s="48" t="str">
         <x:v>Trạng thái</x:v>
       </x:c>
-      <x:c r="U1" s="38" t="str">
+      <x:c r="U1" s="48" t="str">
         <x:v>Dự đoán val</x:v>
       </x:c>
     </x:row>
@@ -2037,19 +2116,28 @@
       <x:c r="M2" s="41" t="n">
         <x:v>0.18524871511108398</x:v>
       </x:c>
-      <x:c r="N2" s="42"/>
-      <x:c r="O2" s="42"/>
-      <x:c r="P2" s="42"/>
-      <x:c r="Q2" s="43" t="str">
+      <x:c r="N2" s="42" t="n">
+        <x:v>8.170875500013608</x:v>
+      </x:c>
+      <x:c r="O2" s="42" t="n">
+        <x:v>9.390229150073992</x:v>
+      </x:c>
+      <x:c r="P2" s="42" t="n">
+        <x:v>9.759574999982307</x:v>
+      </x:c>
+      <x:c r="Q2" s="43" t="n">
         <x:f>IF(AND(ISNUMBER(N2),ISNUMBER($N$2),$N$2&gt;0),N2/$N$2,"")</x:f>
-      </x:c>
-      <x:c r="R2" s="44"/>
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="R2" s="44" t="n">
+        <x:v>287.92069640754784</x:v>
+      </x:c>
       <x:c r="S2" s="7" t="str">
         <x:f>IF(ISNUMBER(O2),IF(O2&lt;=100,"Đạt","Không đạt"),"Chờ đo")</x:f>
-        <x:v>Chờ đo</x:v>
+        <x:v>Đạt</x:v>
       </x:c>
       <x:c r="T2" s="12" t="str">
-        <x:v>Chờ latency T4</x:v>
+        <x:v>Đủ kết quả</x:v>
       </x:c>
       <x:c r="U2" s="7" t="str">
         <x:v>predictions/I00_seed0_val.csv</x:v>
@@ -2083,23 +2171,40 @@
       <x:c r="I3" s="39" t="n">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="J3" s="40"/>
-      <x:c r="K3" s="40"/>
-      <x:c r="L3" s="41"/>
-      <x:c r="M3" s="41"/>
-      <x:c r="N3" s="42"/>
-      <x:c r="O3" s="42"/>
-      <x:c r="P3" s="42"/>
-      <x:c r="Q3" s="43" t="str">
+      <x:c r="J3" s="40" t="n">
+        <x:v>0.9642588606265972</x:v>
+      </x:c>
+      <x:c r="K3" s="40" t="n">
+        <x:v>0.9734361610968295</x:v>
+      </x:c>
+      <x:c r="L3" s="41" t="n">
+        <x:v>0.09708798446443855</x:v>
+      </x:c>
+      <x:c r="M3" s="41" t="n">
+        <x:v>0.18367426949220683</x:v>
+      </x:c>
+      <x:c r="N3" s="42" t="n">
+        <x:v>15.592512500006706</x:v>
+      </x:c>
+      <x:c r="O3" s="42" t="n">
+        <x:v>18.862193050108544</x:v>
+      </x:c>
+      <x:c r="P3" s="42" t="n">
+        <x:v>20.782552349951416</x:v>
+      </x:c>
+      <x:c r="Q3" s="43" t="n">
         <x:f>IF(AND(ISNUMBER(N3),ISNUMBER($N$2),$N$2&gt;0),N3/$N$2,"")</x:f>
-      </x:c>
-      <x:c r="R3" s="44"/>
+        <x:v>1.9083037674458188</x:v>
+      </x:c>
+      <x:c r="R3" s="44" t="n">
+        <x:v>141.69541108373554</x:v>
+      </x:c>
       <x:c r="S3" s="7" t="str">
         <x:f>IF(ISNUMBER(O3),IF(O3&lt;=100,"Đạt","Không đạt"),"Chờ đo")</x:f>
-        <x:v>Chờ đo</x:v>
+        <x:v>Đạt</x:v>
       </x:c>
       <x:c r="T3" s="12" t="str">
-        <x:v>Chưa chạy</x:v>
+        <x:v>Đủ kết quả</x:v>
       </x:c>
       <x:c r="U3" s="7" t="str">
         <x:v>predictions/I01_seed0_val.csv</x:v>
@@ -2133,23 +2238,40 @@
       <x:c r="I4" s="39" t="n">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="J4" s="40"/>
-      <x:c r="K4" s="40"/>
-      <x:c r="L4" s="41"/>
-      <x:c r="M4" s="41"/>
-      <x:c r="N4" s="42"/>
-      <x:c r="O4" s="42"/>
-      <x:c r="P4" s="42"/>
-      <x:c r="Q4" s="43" t="str">
+      <x:c r="J4" s="40" t="n">
+        <x:v>0.9661639604452444</x:v>
+      </x:c>
+      <x:c r="K4" s="40" t="n">
+        <x:v>0.9754355898314767</x:v>
+      </x:c>
+      <x:c r="L4" s="41" t="n">
+        <x:v>0.09960301870037136</x:v>
+      </x:c>
+      <x:c r="M4" s="41" t="n">
+        <x:v>0.18408662857902397</x:v>
+      </x:c>
+      <x:c r="N4" s="42" t="n">
+        <x:v>25.5043319999686</x:v>
+      </x:c>
+      <x:c r="O4" s="42" t="n">
+        <x:v>42.252744699828774</x:v>
+      </x:c>
+      <x:c r="P4" s="42" t="n">
+        <x:v>44.45592407001868</x:v>
+      </x:c>
+      <x:c r="Q4" s="43" t="n">
         <x:f>IF(AND(ISNUMBER(N4),ISNUMBER($N$2),$N$2&gt;0),N4/$N$2,"")</x:f>
-      </x:c>
-      <x:c r="R4" s="44"/>
+        <x:v>3.12137077598675</x:v>
+      </x:c>
+      <x:c r="R4" s="44" t="n">
+        <x:v>56.018330212275586</x:v>
+      </x:c>
       <x:c r="S4" s="7" t="str">
         <x:f>IF(ISNUMBER(O4),IF(O4&lt;=100,"Đạt","Không đạt"),"Chờ đo")</x:f>
-        <x:v>Chờ đo</x:v>
+        <x:v>Đạt</x:v>
       </x:c>
       <x:c r="T4" s="12" t="str">
-        <x:v>Chưa chạy</x:v>
+        <x:v>Đủ kết quả</x:v>
       </x:c>
       <x:c r="U4" s="7" t="str">
         <x:v>predictions/I02_seed0_val.csv</x:v>
@@ -2183,23 +2305,40 @@
       <x:c r="I5" s="39" t="n">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="J5" s="40"/>
-      <x:c r="K5" s="40"/>
-      <x:c r="L5" s="41"/>
-      <x:c r="M5" s="41"/>
-      <x:c r="N5" s="42"/>
-      <x:c r="O5" s="42"/>
-      <x:c r="P5" s="42"/>
-      <x:c r="Q5" s="43" t="str">
+      <x:c r="J5" s="40" t="n">
+        <x:v>0.9642724549175057</x:v>
+      </x:c>
+      <x:c r="K5" s="40" t="n">
+        <x:v>0.9734361610968295</x:v>
+      </x:c>
+      <x:c r="L5" s="41" t="n">
+        <x:v>0.09718448681233922</x:v>
+      </x:c>
+      <x:c r="M5" s="41" t="n">
+        <x:v>0.18304255989916554</x:v>
+      </x:c>
+      <x:c r="N5" s="42" t="n">
+        <x:v>14.315858999907505</x:v>
+      </x:c>
+      <x:c r="O5" s="42" t="n">
+        <x:v>16.35914885002876</x:v>
+      </x:c>
+      <x:c r="P5" s="42" t="n">
+        <x:v>17.28591950009104</x:v>
+      </x:c>
+      <x:c r="Q5" s="43" t="n">
         <x:f>IF(AND(ISNUMBER(N5),ISNUMBER($N$2),$N$2&gt;0),N5/$N$2,"")</x:f>
-      </x:c>
-      <x:c r="R5" s="44"/>
+        <x:v>1.752059372325972</x:v>
+      </x:c>
+      <x:c r="R5" s="44" t="n">
+        <x:v>140.00087056477707</x:v>
+      </x:c>
       <x:c r="S5" s="7" t="str">
         <x:f>IF(ISNUMBER(O5),IF(O5&lt;=100,"Đạt","Không đạt"),"Chờ đo")</x:f>
-        <x:v>Chờ đo</x:v>
+        <x:v>Đạt</x:v>
       </x:c>
       <x:c r="T5" s="12" t="str">
-        <x:v>Chưa chạy</x:v>
+        <x:v>Đủ kết quả</x:v>
       </x:c>
       <x:c r="U5" s="7" t="str">
         <x:v>predictions/I03_seed0_val.csv</x:v>
@@ -2233,23 +2372,40 @@
       <x:c r="I6" s="39" t="n">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="J6" s="40"/>
-      <x:c r="K6" s="40"/>
-      <x:c r="L6" s="41"/>
-      <x:c r="M6" s="41"/>
-      <x:c r="N6" s="42"/>
-      <x:c r="O6" s="42"/>
-      <x:c r="P6" s="42"/>
-      <x:c r="Q6" s="43" t="str">
+      <x:c r="J6" s="40" t="n">
+        <x:v>0.9689643072792996</x:v>
+      </x:c>
+      <x:c r="K6" s="40" t="n">
+        <x:v>0.9765781205369894</x:v>
+      </x:c>
+      <x:c r="L6" s="41" t="n">
+        <x:v>0.09549411788631819</x:v>
+      </x:c>
+      <x:c r="M6" s="41" t="n">
+        <x:v>0.17404122427507127</x:v>
+      </x:c>
+      <x:c r="N6" s="42" t="n">
+        <x:v>5.762696499687081</x:v>
+      </x:c>
+      <x:c r="O6" s="42" t="n">
+        <x:v>9.138116349868142</x:v>
+      </x:c>
+      <x:c r="P6" s="42" t="n">
+        <x:v>9.336611160060794</x:v>
+      </x:c>
+      <x:c r="Q6" s="43" t="n">
         <x:f>IF(AND(ISNUMBER(N6),ISNUMBER($N$2),$N$2&gt;0),N6/$N$2,"")</x:f>
-      </x:c>
-      <x:c r="R6" s="44"/>
+        <x:v>0.7052728314949217</x:v>
+      </x:c>
+      <x:c r="R6" s="44" t="n">
+        <x:v>219.4559660541361</x:v>
+      </x:c>
       <x:c r="S6" s="7" t="str">
         <x:f>IF(ISNUMBER(O6),IF(O6&lt;=100,"Đạt","Không đạt"),"Chờ đo")</x:f>
-        <x:v>Chờ đo</x:v>
+        <x:v>Đạt</x:v>
       </x:c>
       <x:c r="T6" s="12" t="str">
-        <x:v>Chưa chạy</x:v>
+        <x:v>Đủ kết quả</x:v>
       </x:c>
       <x:c r="U6" s="7" t="str">
         <x:v>predictions/I04_seed0_val.csv</x:v>
@@ -2283,23 +2439,40 @@
       <x:c r="I7" s="39" t="n">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="J7" s="40"/>
-      <x:c r="K7" s="40"/>
-      <x:c r="L7" s="41"/>
-      <x:c r="M7" s="41"/>
-      <x:c r="N7" s="42"/>
-      <x:c r="O7" s="42"/>
-      <x:c r="P7" s="42"/>
-      <x:c r="Q7" s="43" t="str">
+      <x:c r="J7" s="40" t="n">
+        <x:v>0.9698380941836109</x:v>
+      </x:c>
+      <x:c r="K7" s="40" t="n">
+        <x:v>0.9771493858897458</x:v>
+      </x:c>
+      <x:c r="L7" s="41" t="n">
+        <x:v>0.1038055720536991</x:v>
+      </x:c>
+      <x:c r="M7" s="41" t="n">
+        <x:v>0.1815890148680995</x:v>
+      </x:c>
+      <x:c r="N7" s="42" t="n">
+        <x:v>8.536347499784824</x:v>
+      </x:c>
+      <x:c r="O7" s="42" t="n">
+        <x:v>9.068122750227303</x:v>
+      </x:c>
+      <x:c r="P7" s="42" t="n">
+        <x:v>9.182092810183349</x:v>
+      </x:c>
+      <x:c r="Q7" s="43" t="n">
         <x:f>IF(AND(ISNUMBER(N7),ISNUMBER($N$2),$N$2&gt;0),N7/$N$2,"")</x:f>
-      </x:c>
-      <x:c r="R7" s="44"/>
+        <x:v>1.044728621770165</x:v>
+      </x:c>
+      <x:c r="R7" s="44" t="n">
+        <x:v>168.27520588905628</x:v>
+      </x:c>
       <x:c r="S7" s="7" t="str">
         <x:f>IF(ISNUMBER(O7),IF(O7&lt;=100,"Đạt","Không đạt"),"Chờ đo")</x:f>
-        <x:v>Chờ đo</x:v>
+        <x:v>Đạt</x:v>
       </x:c>
       <x:c r="T7" s="12" t="str">
-        <x:v>Chưa chạy</x:v>
+        <x:v>Đủ kết quả</x:v>
       </x:c>
       <x:c r="U7" s="7" t="str">
         <x:v>predictions/I09_seed0_val.csv</x:v>
@@ -2333,23 +2506,40 @@
       <x:c r="I8" s="39" t="n">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="J8" s="40"/>
-      <x:c r="K8" s="40"/>
-      <x:c r="L8" s="41"/>
-      <x:c r="M8" s="41"/>
-      <x:c r="N8" s="42"/>
-      <x:c r="O8" s="42"/>
-      <x:c r="P8" s="42"/>
-      <x:c r="Q8" s="43" t="str">
+      <x:c r="J8" s="40" t="n">
+        <x:v>0.968106255766696</x:v>
+      </x:c>
+      <x:c r="K8" s="40" t="n">
+        <x:v>0.9762924878606113</x:v>
+      </x:c>
+      <x:c r="L8" s="41" t="n">
+        <x:v>0.11564186553556126</x:v>
+      </x:c>
+      <x:c r="M8" s="41" t="n">
+        <x:v>0.19462154942053786</x:v>
+      </x:c>
+      <x:c r="N8" s="42" t="n">
+        <x:v>8.566771000005247</x:v>
+      </x:c>
+      <x:c r="O8" s="42" t="n">
+        <x:v>9.153301400033342</x:v>
+      </x:c>
+      <x:c r="P8" s="42" t="n">
+        <x:v>9.224600080315213</x:v>
+      </x:c>
+      <x:c r="Q8" s="43" t="n">
         <x:f>IF(AND(ISNUMBER(N8),ISNUMBER($N$2),$N$2&gt;0),N8/$N$2,"")</x:f>
-      </x:c>
-      <x:c r="R8" s="44"/>
+        <x:v>1.0484520294050472</x:v>
+      </x:c>
+      <x:c r="R8" s="44" t="n">
+        <x:v>141.12256767170206</x:v>
+      </x:c>
       <x:c r="S8" s="7" t="str">
         <x:f>IF(ISNUMBER(O8),IF(O8&lt;=100,"Đạt","Không đạt"),"Chờ đo")</x:f>
-        <x:v>Chờ đo</x:v>
+        <x:v>Đạt</x:v>
       </x:c>
       <x:c r="T8" s="12" t="str">
-        <x:v>Chưa chạy</x:v>
+        <x:v>Đủ kết quả</x:v>
       </x:c>
       <x:c r="U8" s="7" t="str">
         <x:v>predictions/I10_seed0_val.csv</x:v>
@@ -2395,19 +2585,28 @@
       <x:c r="M9" s="41" t="n">
         <x:v>0.1060759472757501</x:v>
       </x:c>
-      <x:c r="N9" s="42"/>
-      <x:c r="O9" s="42"/>
-      <x:c r="P9" s="42"/>
-      <x:c r="Q9" s="43" t="str">
+      <x:c r="N9" s="42" t="n">
+        <x:v>5.06399899995813</x:v>
+      </x:c>
+      <x:c r="O9" s="42" t="n">
+        <x:v>7.490706349949504</x:v>
+      </x:c>
+      <x:c r="P9" s="42" t="n">
+        <x:v>8.596570879622051</x:v>
+      </x:c>
+      <x:c r="Q9" s="43" t="n">
         <x:f>IF(AND(ISNUMBER(N9),ISNUMBER($N$2),$N$2&gt;0),N9/$N$2,"")</x:f>
-      </x:c>
-      <x:c r="R9" s="44"/>
+        <x:v>0.6197621050461112</x:v>
+      </x:c>
+      <x:c r="R9" s="44" t="n">
+        <x:v>280.69908767079124</x:v>
+      </x:c>
       <x:c r="S9" s="7" t="str">
         <x:f>IF(ISNUMBER(O9),IF(O9&lt;=100,"Đạt","Không đạt"),"Chờ đo")</x:f>
-        <x:v>Chờ đo</x:v>
+        <x:v>Đạt</x:v>
       </x:c>
       <x:c r="T9" s="12" t="str">
-        <x:v>Chờ latency T4</x:v>
+        <x:v>Đủ kết quả</x:v>
       </x:c>
       <x:c r="U9" s="7" t="str">
         <x:v>predictions/I07_seed0_val.csv</x:v>
@@ -2441,23 +2640,40 @@
       <x:c r="I10" s="39" t="n">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="J10" s="40"/>
-      <x:c r="K10" s="40"/>
-      <x:c r="L10" s="41"/>
-      <x:c r="M10" s="41"/>
-      <x:c r="N10" s="42"/>
-      <x:c r="O10" s="42"/>
-      <x:c r="P10" s="42"/>
-      <x:c r="Q10" s="43" t="str">
+      <x:c r="J10" s="40" t="n">
+        <x:v>0.9641032435221208</x:v>
+      </x:c>
+      <x:c r="K10" s="40" t="n">
+        <x:v>0.9737217937732077</x:v>
+      </x:c>
+      <x:c r="L10" s="41" t="n">
+        <x:v>0.09613235726078252</x:v>
+      </x:c>
+      <x:c r="M10" s="41" t="n">
+        <x:v>0.18524799340559084</x:v>
+      </x:c>
+      <x:c r="N10" s="42" t="n">
+        <x:v>7.083049499897243</x:v>
+      </x:c>
+      <x:c r="O10" s="42" t="n">
+        <x:v>10.559240600014162</x:v>
+      </x:c>
+      <x:c r="P10" s="42" t="n">
+        <x:v>11.857329199942797</x:v>
+      </x:c>
+      <x:c r="Q10" s="43" t="n">
         <x:f>IF(AND(ISNUMBER(N10),ISNUMBER($N$2),$N$2&gt;0),N10/$N$2,"")</x:f>
-      </x:c>
-      <x:c r="R10" s="44"/>
+        <x:v>0.8668654295228763</x:v>
+      </x:c>
+      <x:c r="R10" s="44" t="n">
+        <x:v>720.9511613921644</x:v>
+      </x:c>
       <x:c r="S10" s="7" t="str">
         <x:f>IF(ISNUMBER(O10),IF(O10&lt;=100,"Đạt","Không đạt"),"Chờ đo")</x:f>
-        <x:v>Chờ đo</x:v>
+        <x:v>Đạt</x:v>
       </x:c>
       <x:c r="T10" s="12" t="str">
-        <x:v>Chưa chạy</x:v>
+        <x:v>Đủ kết quả</x:v>
       </x:c>
       <x:c r="U10" s="7" t="str">
         <x:v>predictions/I08_seed0_val.csv</x:v>
@@ -2516,105 +2732,1252 @@
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="45" customHeight="1">
-      <x:c r="A1" s="38" t="str">
+      <x:c r="A1" s="48" t="str">
         <x:v>exp_id</x:v>
       </x:c>
-      <x:c r="B1" s="38" t="str">
+      <x:c r="B1" s="48" t="str">
         <x:v>Phương pháp</x:v>
       </x:c>
-      <x:c r="C1" s="38" t="str">
+      <x:c r="C1" s="48" t="str">
         <x:v>gpu</x:v>
       </x:c>
-      <x:c r="D1" s="38" t="str">
+      <x:c r="D1" s="48" t="str">
         <x:v>dtype</x:v>
       </x:c>
-      <x:c r="E1" s="38" t="str">
+      <x:c r="E1" s="48" t="str">
         <x:v>batch</x:v>
       </x:c>
-      <x:c r="F1" s="38" t="str">
+      <x:c r="F1" s="48" t="str">
         <x:v>Crop size</x:v>
       </x:c>
-      <x:c r="G1" s="38" t="str">
+      <x:c r="G1" s="48" t="str">
         <x:v>Input size</x:v>
       </x:c>
-      <x:c r="H1" s="38" t="str">
+      <x:c r="H1" s="48" t="str">
         <x:v>K</x:v>
       </x:c>
-      <x:c r="I1" s="38" t="str">
+      <x:c r="I1" s="48" t="str">
         <x:v>fused_bn</x:v>
       </x:c>
-      <x:c r="J1" s="38" t="str">
+      <x:c r="J1" s="48" t="str">
         <x:v>p50 (ms)</x:v>
       </x:c>
-      <x:c r="K1" s="38" t="str">
+      <x:c r="K1" s="48" t="str">
         <x:v>p95 (ms)</x:v>
       </x:c>
-      <x:c r="L1" s="38" t="str">
+      <x:c r="L1" s="48" t="str">
         <x:v>p99 (ms)</x:v>
       </x:c>
-      <x:c r="M1" s="38" t="str">
+      <x:c r="M1" s="48" t="str">
         <x:v>Mean (ms)</x:v>
       </x:c>
-      <x:c r="N1" s="38" t="str">
+      <x:c r="N1" s="48" t="str">
         <x:v>Ảnh/s</x:v>
       </x:c>
-      <x:c r="O1" s="38" t="str">
+      <x:c r="O1" s="48" t="str">
         <x:v>warmup</x:v>
       </x:c>
-      <x:c r="P1" s="38" t="str">
+      <x:c r="P1" s="48" t="str">
         <x:v>Lần đo</x:v>
       </x:c>
-      <x:c r="Q1" s="38" t="str">
+      <x:c r="Q1" s="48" t="str">
         <x:v>torch</x:v>
       </x:c>
-      <x:c r="R1" s="38" t="str">
+      <x:c r="R1" s="48" t="str">
         <x:v>Gồm tiền xử lý</x:v>
       </x:c>
-      <x:c r="S1" s="38" t="str">
+      <x:c r="S1" s="48" t="str">
         <x:v>Gồm transfer</x:v>
       </x:c>
-      <x:c r="T1" s="38" t="str">
+      <x:c r="T1" s="48" t="str">
         <x:v>Phạm vi đo</x:v>
       </x:c>
-      <x:c r="U1" s="38" t="str">
+      <x:c r="U1" s="48" t="str">
         <x:v>Nguồn số đo</x:v>
       </x:c>
     </x:row>
     <x:row r="2" ht="36" customHeight="1">
-      <x:c r="A2" s="7"/>
-      <x:c r="B2" s="12"/>
-      <x:c r="C2" s="7"/>
-      <x:c r="D2" s="7"/>
-      <x:c r="E2" s="7"/>
-      <x:c r="F2" s="7"/>
-      <x:c r="G2" s="7"/>
-      <x:c r="H2" s="7"/>
-      <x:c r="I2" s="7"/>
-      <x:c r="J2" s="42"/>
-      <x:c r="K2" s="42"/>
-      <x:c r="L2" s="42"/>
-      <x:c r="M2" s="42"/>
-      <x:c r="N2" s="44"/>
-      <x:c r="O2" s="7"/>
-      <x:c r="P2" s="7"/>
-      <x:c r="Q2" s="7"/>
-      <x:c r="R2" s="7"/>
-      <x:c r="S2" s="7"/>
-      <x:c r="T2" s="12"/>
-      <x:c r="U2" s="7"/>
-    </x:row>
-    <x:row r="5">
-      <x:c r="A5" t="str">
-        <x:v>Chưa có số đo T4. Không thay bằng latency sơ bộ Bước 1 hoặc GPU máy cá nhân.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="6">
-      <x:c r="A6" t="str">
+      <x:c r="A2" s="7" t="str">
+        <x:v>I00</x:v>
+      </x:c>
+      <x:c r="B2" s="12" t="str">
+        <x:v>1 view FP32</x:v>
+      </x:c>
+      <x:c r="C2" s="7" t="str">
+        <x:v>Tesla T4</x:v>
+      </x:c>
+      <x:c r="D2" s="7" t="str">
+        <x:v>fp32</x:v>
+      </x:c>
+      <x:c r="E2" s="7" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="F2" s="7" t="n">
+        <x:v>224</x:v>
+      </x:c>
+      <x:c r="G2" s="7" t="n">
+        <x:v>224</x:v>
+      </x:c>
+      <x:c r="H2" s="7" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="I2" s="51" t="b">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="J2" s="42" t="n">
+        <x:v>8.170875500013608</x:v>
+      </x:c>
+      <x:c r="K2" s="42" t="n">
+        <x:v>9.390229150073992</x:v>
+      </x:c>
+      <x:c r="L2" s="42" t="n">
+        <x:v>9.759574999982307</x:v>
+      </x:c>
+      <x:c r="M2" s="42" t="n">
+        <x:v>8.15660145000038</x:v>
+      </x:c>
+      <x:c r="N2" s="44" t="n">
+        <x:v>122.60008118944604</x:v>
+      </x:c>
+      <x:c r="O2" s="7" t="n">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="P2" s="7" t="n">
+        <x:v>100</x:v>
+      </x:c>
+      <x:c r="Q2" s="7" t="str">
+        <x:v>2.8.0+cu128</x:v>
+      </x:c>
+      <x:c r="R2" s="51" t="b">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="S2" s="51" t="b">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="T2" s="12" t="str">
+        <x:v>normalized GPU input; tensor TTA + model + softmax/aggregation/T</x:v>
+      </x:c>
+      <x:c r="U2" s="7" t="str">
+        <x:v>step3/I00/latency_batch1.json</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="3" ht="36" customHeight="1">
+      <x:c r="A3" s="7" t="str">
+        <x:v>I00</x:v>
+      </x:c>
+      <x:c r="B3" s="12" t="str">
+        <x:v>1 view FP32</x:v>
+      </x:c>
+      <x:c r="C3" s="7" t="str">
+        <x:v>Tesla T4</x:v>
+      </x:c>
+      <x:c r="D3" s="7" t="str">
+        <x:v>fp32</x:v>
+      </x:c>
+      <x:c r="E3" s="7" t="n">
+        <x:v>32</x:v>
+      </x:c>
+      <x:c r="F3" s="7" t="n">
+        <x:v>224</x:v>
+      </x:c>
+      <x:c r="G3" s="7" t="n">
+        <x:v>224</x:v>
+      </x:c>
+      <x:c r="H3" s="7" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="I3" s="51" t="b">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="J3" s="42" t="n">
+        <x:v>111.22459650005112</x:v>
+      </x:c>
+      <x:c r="K3" s="42" t="n">
+        <x:v>112.0663408500377</x:v>
+      </x:c>
+      <x:c r="L3" s="42" t="n">
+        <x:v>112.45865352001147</x:v>
+      </x:c>
+      <x:c r="M3" s="42" t="n">
+        <x:v>111.14171505998456</x:v>
+      </x:c>
+      <x:c r="N3" s="44" t="n">
+        <x:v>287.92069640754784</x:v>
+      </x:c>
+      <x:c r="O3" s="7" t="n">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="P3" s="7" t="n">
+        <x:v>100</x:v>
+      </x:c>
+      <x:c r="Q3" s="7" t="str">
+        <x:v>2.8.0+cu128</x:v>
+      </x:c>
+      <x:c r="R3" s="51" t="b">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="S3" s="51" t="b">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="T3" s="12" t="str">
+        <x:v>normalized GPU input; tensor TTA + model + softmax/aggregation/T</x:v>
+      </x:c>
+      <x:c r="U3" s="7" t="str">
+        <x:v>step3/I00/latency_batch32.json</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="4" ht="36" customHeight="1">
+      <x:c r="A4" s="7" t="str">
+        <x:v>I01</x:v>
+      </x:c>
+      <x:c r="B4" s="12" t="str">
+        <x:v>Hflip TTA / probability</x:v>
+      </x:c>
+      <x:c r="C4" s="7" t="str">
+        <x:v>Tesla T4</x:v>
+      </x:c>
+      <x:c r="D4" s="7" t="str">
+        <x:v>fp32</x:v>
+      </x:c>
+      <x:c r="E4" s="7" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="F4" s="7" t="n">
+        <x:v>224</x:v>
+      </x:c>
+      <x:c r="G4" s="7" t="n">
+        <x:v>224</x:v>
+      </x:c>
+      <x:c r="H4" s="7" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="I4" s="51" t="b">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="J4" s="42" t="n">
+        <x:v>15.592512500006706</x:v>
+      </x:c>
+      <x:c r="K4" s="42" t="n">
+        <x:v>18.862193050108544</x:v>
+      </x:c>
+      <x:c r="L4" s="42" t="n">
+        <x:v>20.782552349951416</x:v>
+      </x:c>
+      <x:c r="M4" s="42" t="n">
+        <x:v>15.899964079999336</x:v>
+      </x:c>
+      <x:c r="N4" s="44" t="n">
+        <x:v>62.89322384431712</x:v>
+      </x:c>
+      <x:c r="O4" s="7" t="n">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="P4" s="7" t="n">
+        <x:v>100</x:v>
+      </x:c>
+      <x:c r="Q4" s="7" t="str">
+        <x:v>2.8.0+cu128</x:v>
+      </x:c>
+      <x:c r="R4" s="51" t="b">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="S4" s="51" t="b">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="T4" s="12" t="str">
+        <x:v>normalized GPU input; tensor TTA + model + softmax/aggregation/T</x:v>
+      </x:c>
+      <x:c r="U4" s="7" t="str">
+        <x:v>step3/I01/latency_batch1.json</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="5" ht="36" customHeight="1">
+      <x:c r="A5" s="7" t="str">
+        <x:v>I01</x:v>
+      </x:c>
+      <x:c r="B5" s="12" t="str">
+        <x:v>Hflip TTA / probability</x:v>
+      </x:c>
+      <x:c r="C5" s="7" t="str">
+        <x:v>Tesla T4</x:v>
+      </x:c>
+      <x:c r="D5" s="7" t="str">
+        <x:v>fp32</x:v>
+      </x:c>
+      <x:c r="E5" s="7" t="n">
+        <x:v>32</x:v>
+      </x:c>
+      <x:c r="F5" s="7" t="n">
+        <x:v>224</x:v>
+      </x:c>
+      <x:c r="G5" s="7" t="n">
+        <x:v>224</x:v>
+      </x:c>
+      <x:c r="H5" s="7" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="I5" s="51" t="b">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="J5" s="42" t="n">
+        <x:v>225.82709200003137</x:v>
+      </x:c>
+      <x:c r="K5" s="42" t="n">
+        <x:v>227.34254434993773</x:v>
+      </x:c>
+      <x:c r="L5" s="42" t="n">
+        <x:v>227.93199235995644</x:v>
+      </x:c>
+      <x:c r="M5" s="42" t="n">
+        <x:v>225.83653031000037</x:v>
+      </x:c>
+      <x:c r="N5" s="44" t="n">
+        <x:v>141.69541108373554</x:v>
+      </x:c>
+      <x:c r="O5" s="7" t="n">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="P5" s="7" t="n">
+        <x:v>100</x:v>
+      </x:c>
+      <x:c r="Q5" s="7" t="str">
+        <x:v>2.8.0+cu128</x:v>
+      </x:c>
+      <x:c r="R5" s="51" t="b">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="S5" s="51" t="b">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="T5" s="12" t="str">
+        <x:v>normalized GPU input; tensor TTA + model + softmax/aggregation/T</x:v>
+      </x:c>
+      <x:c r="U5" s="7" t="str">
+        <x:v>step3/I01/latency_batch32.json</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="6" ht="36" customHeight="1">
+      <x:c r="A6" s="7" t="str">
+        <x:v>I02</x:v>
+      </x:c>
+      <x:c r="B6" s="12" t="str">
+        <x:v>5 crops / probability</x:v>
+      </x:c>
+      <x:c r="C6" s="7" t="str">
+        <x:v>Tesla T4</x:v>
+      </x:c>
+      <x:c r="D6" s="7" t="str">
+        <x:v>fp32</x:v>
+      </x:c>
+      <x:c r="E6" s="7" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="F6" s="7" t="n">
+        <x:v>224</x:v>
+      </x:c>
+      <x:c r="G6" s="7" t="n">
+        <x:v>256</x:v>
+      </x:c>
+      <x:c r="H6" s="7" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="I6" s="51" t="b">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="J6" s="42" t="n">
+        <x:v>25.5043319999686</x:v>
+      </x:c>
+      <x:c r="K6" s="42" t="n">
+        <x:v>42.252744699828774</x:v>
+      </x:c>
+      <x:c r="L6" s="42" t="n">
+        <x:v>44.45592407001868</x:v>
+      </x:c>
+      <x:c r="M6" s="42" t="n">
+        <x:v>29.357443929995952</x:v>
+      </x:c>
+      <x:c r="N6" s="44" t="n">
+        <x:v>34.062911007666116</x:v>
+      </x:c>
+      <x:c r="O6" s="7" t="n">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="P6" s="7" t="n">
+        <x:v>100</x:v>
+      </x:c>
+      <x:c r="Q6" s="7" t="str">
+        <x:v>2.8.0+cu128</x:v>
+      </x:c>
+      <x:c r="R6" s="51" t="b">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="S6" s="51" t="b">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="T6" s="12" t="str">
+        <x:v>normalized GPU input; tensor TTA + model + softmax/aggregation/T</x:v>
+      </x:c>
+      <x:c r="U6" s="7" t="str">
+        <x:v>step3/I02/latency_batch1.json</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="7" ht="36" customHeight="1">
+      <x:c r="A7" s="7" t="str">
+        <x:v>I02</x:v>
+      </x:c>
+      <x:c r="B7" s="12" t="str">
+        <x:v>5 crops / probability</x:v>
+      </x:c>
+      <x:c r="C7" s="7" t="str">
+        <x:v>Tesla T4</x:v>
+      </x:c>
+      <x:c r="D7" s="7" t="str">
+        <x:v>fp32</x:v>
+      </x:c>
+      <x:c r="E7" s="7" t="n">
+        <x:v>32</x:v>
+      </x:c>
+      <x:c r="F7" s="7" t="n">
+        <x:v>224</x:v>
+      </x:c>
+      <x:c r="G7" s="7" t="n">
+        <x:v>256</x:v>
+      </x:c>
+      <x:c r="H7" s="7" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="I7" s="51" t="b">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="J7" s="42" t="n">
+        <x:v>571.2320369998451</x:v>
+      </x:c>
+      <x:c r="K7" s="42" t="n">
+        <x:v>573.4608021998611</x:v>
+      </x:c>
+      <x:c r="L7" s="42" t="n">
+        <x:v>573.6716340500766</x:v>
+      </x:c>
+      <x:c r="M7" s="42" t="n">
+        <x:v>571.2415896500191</x:v>
+      </x:c>
+      <x:c r="N7" s="44" t="n">
+        <x:v>56.018330212275586</x:v>
+      </x:c>
+      <x:c r="O7" s="7" t="n">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="P7" s="7" t="n">
+        <x:v>100</x:v>
+      </x:c>
+      <x:c r="Q7" s="7" t="str">
+        <x:v>2.8.0+cu128</x:v>
+      </x:c>
+      <x:c r="R7" s="51" t="b">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="S7" s="51" t="b">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="T7" s="12" t="str">
+        <x:v>normalized GPU input; tensor TTA + model + softmax/aggregation/T</x:v>
+      </x:c>
+      <x:c r="U7" s="7" t="str">
+        <x:v>step3/I02/latency_batch32.json</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="8" ht="36" customHeight="1">
+      <x:c r="A8" s="7" t="str">
+        <x:v>I03</x:v>
+      </x:c>
+      <x:c r="B8" s="12" t="str">
+        <x:v>Hflip TTA / logits</x:v>
+      </x:c>
+      <x:c r="C8" s="7" t="str">
+        <x:v>Tesla T4</x:v>
+      </x:c>
+      <x:c r="D8" s="7" t="str">
+        <x:v>fp32</x:v>
+      </x:c>
+      <x:c r="E8" s="7" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="F8" s="7" t="n">
+        <x:v>224</x:v>
+      </x:c>
+      <x:c r="G8" s="7" t="n">
+        <x:v>224</x:v>
+      </x:c>
+      <x:c r="H8" s="7" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="I8" s="51" t="b">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="J8" s="42" t="n">
+        <x:v>14.315858999907505</x:v>
+      </x:c>
+      <x:c r="K8" s="42" t="n">
+        <x:v>16.35914885002876</x:v>
+      </x:c>
+      <x:c r="L8" s="42" t="n">
+        <x:v>17.28591950009104</x:v>
+      </x:c>
+      <x:c r="M8" s="42" t="n">
+        <x:v>13.603611519984042</x:v>
+      </x:c>
+      <x:c r="N8" s="44" t="n">
+        <x:v>73.50989099703231</x:v>
+      </x:c>
+      <x:c r="O8" s="7" t="n">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="P8" s="7" t="n">
+        <x:v>100</x:v>
+      </x:c>
+      <x:c r="Q8" s="7" t="str">
+        <x:v>2.8.0+cu128</x:v>
+      </x:c>
+      <x:c r="R8" s="51" t="b">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="S8" s="51" t="b">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="T8" s="12" t="str">
+        <x:v>normalized GPU input; tensor TTA + model + softmax/aggregation/T</x:v>
+      </x:c>
+      <x:c r="U8" s="7" t="str">
+        <x:v>step3/I03/latency_batch1.json</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="9" ht="36" customHeight="1">
+      <x:c r="A9" s="7" t="str">
+        <x:v>I03</x:v>
+      </x:c>
+      <x:c r="B9" s="12" t="str">
+        <x:v>Hflip TTA / logits</x:v>
+      </x:c>
+      <x:c r="C9" s="7" t="str">
+        <x:v>Tesla T4</x:v>
+      </x:c>
+      <x:c r="D9" s="7" t="str">
+        <x:v>fp32</x:v>
+      </x:c>
+      <x:c r="E9" s="7" t="n">
+        <x:v>32</x:v>
+      </x:c>
+      <x:c r="F9" s="7" t="n">
+        <x:v>224</x:v>
+      </x:c>
+      <x:c r="G9" s="7" t="n">
+        <x:v>224</x:v>
+      </x:c>
+      <x:c r="H9" s="7" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="I9" s="51" t="b">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="J9" s="42" t="n">
+        <x:v>228.59176900010425</x:v>
+      </x:c>
+      <x:c r="K9" s="42" t="n">
+        <x:v>230.371583150054</x:v>
+      </x:c>
+      <x:c r="L9" s="42" t="n">
+        <x:v>230.73990807982227</x:v>
+      </x:c>
+      <x:c r="M9" s="42" t="n">
+        <x:v>228.57000725001853</x:v>
+      </x:c>
+      <x:c r="N9" s="44" t="n">
+        <x:v>140.00087056477707</x:v>
+      </x:c>
+      <x:c r="O9" s="7" t="n">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="P9" s="7" t="n">
+        <x:v>100</x:v>
+      </x:c>
+      <x:c r="Q9" s="7" t="str">
+        <x:v>2.8.0+cu128</x:v>
+      </x:c>
+      <x:c r="R9" s="51" t="b">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="S9" s="51" t="b">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="T9" s="12" t="str">
+        <x:v>normalized GPU input; tensor TTA + model + softmax/aggregation/T</x:v>
+      </x:c>
+      <x:c r="U9" s="7" t="str">
+        <x:v>step3/I03/latency_batch32.json</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="10" ht="36" customHeight="1">
+      <x:c r="A10" s="7" t="str">
+        <x:v>I04</x:v>
+      </x:c>
+      <x:c r="B10" s="12" t="str">
+        <x:v>Resolution 256</x:v>
+      </x:c>
+      <x:c r="C10" s="7" t="str">
+        <x:v>Tesla T4</x:v>
+      </x:c>
+      <x:c r="D10" s="7" t="str">
+        <x:v>fp32</x:v>
+      </x:c>
+      <x:c r="E10" s="7" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="F10" s="7" t="n">
+        <x:v>256</x:v>
+      </x:c>
+      <x:c r="G10" s="7" t="n">
+        <x:v>256</x:v>
+      </x:c>
+      <x:c r="H10" s="7" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="I10" s="51" t="b">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="J10" s="42" t="n">
+        <x:v>5.762696499687081</x:v>
+      </x:c>
+      <x:c r="K10" s="42" t="n">
+        <x:v>9.138116349868142</x:v>
+      </x:c>
+      <x:c r="L10" s="42" t="n">
+        <x:v>9.336611160060794</x:v>
+      </x:c>
+      <x:c r="M10" s="42" t="n">
+        <x:v>6.896288039979481</x:v>
+      </x:c>
+      <x:c r="N10" s="44" t="n">
+        <x:v>145.0055441714084</x:v>
+      </x:c>
+      <x:c r="O10" s="7" t="n">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="P10" s="7" t="n">
+        <x:v>100</x:v>
+      </x:c>
+      <x:c r="Q10" s="7" t="str">
+        <x:v>2.8.0+cu128</x:v>
+      </x:c>
+      <x:c r="R10" s="51" t="b">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="S10" s="51" t="b">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="T10" s="12" t="str">
+        <x:v>normalized GPU input; tensor TTA + model + softmax/aggregation/T</x:v>
+      </x:c>
+      <x:c r="U10" s="7" t="str">
+        <x:v>step3/I04/latency_batch1.json</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="11" ht="36" customHeight="1">
+      <x:c r="A11" s="7" t="str">
+        <x:v>I04</x:v>
+      </x:c>
+      <x:c r="B11" s="12" t="str">
+        <x:v>Resolution 256</x:v>
+      </x:c>
+      <x:c r="C11" s="7" t="str">
+        <x:v>Tesla T4</x:v>
+      </x:c>
+      <x:c r="D11" s="7" t="str">
+        <x:v>fp32</x:v>
+      </x:c>
+      <x:c r="E11" s="7" t="n">
+        <x:v>32</x:v>
+      </x:c>
+      <x:c r="F11" s="7" t="n">
+        <x:v>256</x:v>
+      </x:c>
+      <x:c r="G11" s="7" t="n">
+        <x:v>256</x:v>
+      </x:c>
+      <x:c r="H11" s="7" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="I11" s="51" t="b">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="J11" s="42" t="n">
+        <x:v>145.80802249975022</x:v>
+      </x:c>
+      <x:c r="K11" s="42" t="n">
+        <x:v>147.3497600499968</x:v>
+      </x:c>
+      <x:c r="L11" s="42" t="n">
+        <x:v>148.0081490100656</x:v>
+      </x:c>
+      <x:c r="M11" s="42" t="n">
+        <x:v>145.81512899998415</x:v>
+      </x:c>
+      <x:c r="N11" s="44" t="n">
+        <x:v>219.4559660541361</x:v>
+      </x:c>
+      <x:c r="O11" s="7" t="n">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="P11" s="7" t="n">
+        <x:v>100</x:v>
+      </x:c>
+      <x:c r="Q11" s="7" t="str">
+        <x:v>2.8.0+cu128</x:v>
+      </x:c>
+      <x:c r="R11" s="51" t="b">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="S11" s="51" t="b">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="T11" s="12" t="str">
+        <x:v>normalized GPU input; tensor TTA + model + softmax/aggregation/T</x:v>
+      </x:c>
+      <x:c r="U11" s="7" t="str">
+        <x:v>step3/I04/latency_batch32.json</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="12" ht="36" customHeight="1">
+      <x:c r="A12" s="7" t="str">
+        <x:v>I09</x:v>
+      </x:c>
+      <x:c r="B12" s="12" t="str">
+        <x:v>Resolution 288</x:v>
+      </x:c>
+      <x:c r="C12" s="7" t="str">
+        <x:v>Tesla T4</x:v>
+      </x:c>
+      <x:c r="D12" s="7" t="str">
+        <x:v>fp32</x:v>
+      </x:c>
+      <x:c r="E12" s="7" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="F12" s="7" t="n">
+        <x:v>288</x:v>
+      </x:c>
+      <x:c r="G12" s="7" t="n">
+        <x:v>288</x:v>
+      </x:c>
+      <x:c r="H12" s="7" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="I12" s="51" t="b">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="J12" s="42" t="n">
+        <x:v>8.536347499784824</x:v>
+      </x:c>
+      <x:c r="K12" s="42" t="n">
+        <x:v>9.068122750227303</x:v>
+      </x:c>
+      <x:c r="L12" s="42" t="n">
+        <x:v>9.182092810183349</x:v>
+      </x:c>
+      <x:c r="M12" s="42" t="n">
+        <x:v>7.908351769988258</x:v>
+      </x:c>
+      <x:c r="N12" s="44" t="n">
+        <x:v>126.44859878324365</x:v>
+      </x:c>
+      <x:c r="O12" s="7" t="n">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="P12" s="7" t="n">
+        <x:v>100</x:v>
+      </x:c>
+      <x:c r="Q12" s="7" t="str">
+        <x:v>2.8.0+cu128</x:v>
+      </x:c>
+      <x:c r="R12" s="51" t="b">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="S12" s="51" t="b">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="T12" s="12" t="str">
+        <x:v>normalized GPU input; tensor TTA + model + softmax/aggregation/T</x:v>
+      </x:c>
+      <x:c r="U12" s="7" t="str">
+        <x:v>step3/I09/latency_batch1.json</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="13" ht="36" customHeight="1">
+      <x:c r="A13" s="7" t="str">
+        <x:v>I09</x:v>
+      </x:c>
+      <x:c r="B13" s="12" t="str">
+        <x:v>Resolution 288</x:v>
+      </x:c>
+      <x:c r="C13" s="7" t="str">
+        <x:v>Tesla T4</x:v>
+      </x:c>
+      <x:c r="D13" s="7" t="str">
+        <x:v>fp32</x:v>
+      </x:c>
+      <x:c r="E13" s="7" t="n">
+        <x:v>32</x:v>
+      </x:c>
+      <x:c r="F13" s="7" t="n">
+        <x:v>288</x:v>
+      </x:c>
+      <x:c r="G13" s="7" t="n">
+        <x:v>288</x:v>
+      </x:c>
+      <x:c r="H13" s="7" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="I13" s="51" t="b">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="J13" s="42" t="n">
+        <x:v>190.2043625002534</x:v>
+      </x:c>
+      <x:c r="K13" s="42" t="n">
+        <x:v>192.74151690005965</x:v>
+      </x:c>
+      <x:c r="L13" s="42" t="n">
+        <x:v>193.54442563013436</x:v>
+      </x:c>
+      <x:c r="M13" s="42" t="n">
+        <x:v>190.16467596003167</x:v>
+      </x:c>
+      <x:c r="N13" s="44" t="n">
+        <x:v>168.27520588905628</x:v>
+      </x:c>
+      <x:c r="O13" s="7" t="n">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="P13" s="7" t="n">
+        <x:v>100</x:v>
+      </x:c>
+      <x:c r="Q13" s="7" t="str">
+        <x:v>2.8.0+cu128</x:v>
+      </x:c>
+      <x:c r="R13" s="51" t="b">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="S13" s="51" t="b">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="T13" s="12" t="str">
+        <x:v>normalized GPU input; tensor TTA + model + softmax/aggregation/T</x:v>
+      </x:c>
+      <x:c r="U13" s="7" t="str">
+        <x:v>step3/I09/latency_batch32.json</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="14" ht="36" customHeight="1">
+      <x:c r="A14" s="7" t="str">
+        <x:v>I10</x:v>
+      </x:c>
+      <x:c r="B14" s="12" t="str">
+        <x:v>Resolution 320</x:v>
+      </x:c>
+      <x:c r="C14" s="7" t="str">
+        <x:v>Tesla T4</x:v>
+      </x:c>
+      <x:c r="D14" s="7" t="str">
+        <x:v>fp32</x:v>
+      </x:c>
+      <x:c r="E14" s="7" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="F14" s="7" t="n">
+        <x:v>320</x:v>
+      </x:c>
+      <x:c r="G14" s="7" t="n">
+        <x:v>320</x:v>
+      </x:c>
+      <x:c r="H14" s="7" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="I14" s="51" t="b">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="J14" s="42" t="n">
+        <x:v>8.566771000005247</x:v>
+      </x:c>
+      <x:c r="K14" s="42" t="n">
+        <x:v>9.153301400033342</x:v>
+      </x:c>
+      <x:c r="L14" s="42" t="n">
+        <x:v>9.224600080315213</x:v>
+      </x:c>
+      <x:c r="M14" s="42" t="n">
+        <x:v>8.667125530018893</x:v>
+      </x:c>
+      <x:c r="N14" s="44" t="n">
+        <x:v>115.37850658058025</x:v>
+      </x:c>
+      <x:c r="O14" s="7" t="n">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="P14" s="7" t="n">
+        <x:v>100</x:v>
+      </x:c>
+      <x:c r="Q14" s="7" t="str">
+        <x:v>2.8.0+cu128</x:v>
+      </x:c>
+      <x:c r="R14" s="51" t="b">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="S14" s="51" t="b">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="T14" s="12" t="str">
+        <x:v>normalized GPU input; tensor TTA + model + softmax/aggregation/T</x:v>
+      </x:c>
+      <x:c r="U14" s="7" t="str">
+        <x:v>step3/I10/latency_batch1.json</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="15" ht="36" customHeight="1">
+      <x:c r="A15" s="7" t="str">
+        <x:v>I10</x:v>
+      </x:c>
+      <x:c r="B15" s="12" t="str">
+        <x:v>Resolution 320</x:v>
+      </x:c>
+      <x:c r="C15" s="7" t="str">
+        <x:v>Tesla T4</x:v>
+      </x:c>
+      <x:c r="D15" s="7" t="str">
+        <x:v>fp32</x:v>
+      </x:c>
+      <x:c r="E15" s="7" t="n">
+        <x:v>32</x:v>
+      </x:c>
+      <x:c r="F15" s="7" t="n">
+        <x:v>320</x:v>
+      </x:c>
+      <x:c r="G15" s="7" t="n">
+        <x:v>320</x:v>
+      </x:c>
+      <x:c r="H15" s="7" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="I15" s="51" t="b">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="J15" s="42" t="n">
+        <x:v>226.53145599997515</x:v>
+      </x:c>
+      <x:c r="K15" s="42" t="n">
+        <x:v>229.26256739986002</x:v>
+      </x:c>
+      <x:c r="L15" s="42" t="n">
+        <x:v>229.99557527973593</x:v>
+      </x:c>
+      <x:c r="M15" s="42" t="n">
+        <x:v>226.75324385000295</x:v>
+      </x:c>
+      <x:c r="N15" s="44" t="n">
+        <x:v>141.12256767170206</x:v>
+      </x:c>
+      <x:c r="O15" s="7" t="n">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="P15" s="7" t="n">
+        <x:v>100</x:v>
+      </x:c>
+      <x:c r="Q15" s="7" t="str">
+        <x:v>2.8.0+cu128</x:v>
+      </x:c>
+      <x:c r="R15" s="51" t="b">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="S15" s="51" t="b">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="T15" s="12" t="str">
+        <x:v>normalized GPU input; tensor TTA + model + softmax/aggregation/T</x:v>
+      </x:c>
+      <x:c r="U15" s="7" t="str">
+        <x:v>step3/I10/latency_batch32.json</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="16" ht="36" customHeight="1">
+      <x:c r="A16" s="7" t="str">
+        <x:v>I07</x:v>
+      </x:c>
+      <x:c r="B16" s="12" t="str">
+        <x:v>1 view + temperature</x:v>
+      </x:c>
+      <x:c r="C16" s="7" t="str">
+        <x:v>Tesla T4</x:v>
+      </x:c>
+      <x:c r="D16" s="7" t="str">
+        <x:v>fp32</x:v>
+      </x:c>
+      <x:c r="E16" s="7" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="F16" s="7" t="n">
+        <x:v>224</x:v>
+      </x:c>
+      <x:c r="G16" s="7" t="n">
+        <x:v>224</x:v>
+      </x:c>
+      <x:c r="H16" s="7" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="I16" s="51" t="b">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="J16" s="42" t="n">
+        <x:v>5.06399899995813</x:v>
+      </x:c>
+      <x:c r="K16" s="42" t="n">
+        <x:v>7.490706349949504</x:v>
+      </x:c>
+      <x:c r="L16" s="42" t="n">
+        <x:v>8.596570879622051</x:v>
+      </x:c>
+      <x:c r="M16" s="42" t="n">
+        <x:v>5.366366360003667</x:v>
+      </x:c>
+      <x:c r="N16" s="44" t="n">
+        <x:v>186.34583122262205</x:v>
+      </x:c>
+      <x:c r="O16" s="7" t="n">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="P16" s="7" t="n">
+        <x:v>100</x:v>
+      </x:c>
+      <x:c r="Q16" s="7" t="str">
+        <x:v>2.8.0+cu128</x:v>
+      </x:c>
+      <x:c r="R16" s="51" t="b">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="S16" s="51" t="b">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="T16" s="12" t="str">
+        <x:v>normalized GPU input; tensor TTA + model + softmax/aggregation/T</x:v>
+      </x:c>
+      <x:c r="U16" s="7" t="str">
+        <x:v>step3/I07/latency_batch1.json</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="17" ht="36" customHeight="1">
+      <x:c r="A17" s="7" t="str">
+        <x:v>I07</x:v>
+      </x:c>
+      <x:c r="B17" s="12" t="str">
+        <x:v>1 view + temperature</x:v>
+      </x:c>
+      <x:c r="C17" s="7" t="str">
+        <x:v>Tesla T4</x:v>
+      </x:c>
+      <x:c r="D17" s="7" t="str">
+        <x:v>fp32</x:v>
+      </x:c>
+      <x:c r="E17" s="7" t="n">
+        <x:v>32</x:v>
+      </x:c>
+      <x:c r="F17" s="7" t="n">
+        <x:v>224</x:v>
+      </x:c>
+      <x:c r="G17" s="7" t="n">
+        <x:v>224</x:v>
+      </x:c>
+      <x:c r="H17" s="7" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="I17" s="51" t="b">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="J17" s="42" t="n">
+        <x:v>113.99357300001611</x:v>
+      </x:c>
+      <x:c r="K17" s="42" t="n">
+        <x:v>115.24236010031927</x:v>
+      </x:c>
+      <x:c r="L17" s="42" t="n">
+        <x:v>115.59245574032502</x:v>
+      </x:c>
+      <x:c r="M17" s="42" t="n">
+        <x:v>114.00108302998888</x:v>
+      </x:c>
+      <x:c r="N17" s="44" t="n">
+        <x:v>280.69908767079124</x:v>
+      </x:c>
+      <x:c r="O17" s="7" t="n">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="P17" s="7" t="n">
+        <x:v>100</x:v>
+      </x:c>
+      <x:c r="Q17" s="7" t="str">
+        <x:v>2.8.0+cu128</x:v>
+      </x:c>
+      <x:c r="R17" s="51" t="b">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="S17" s="51" t="b">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="T17" s="12" t="str">
+        <x:v>normalized GPU input; tensor TTA + model + softmax/aggregation/T</x:v>
+      </x:c>
+      <x:c r="U17" s="7" t="str">
+        <x:v>step3/I07/latency_batch32.json</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="18" ht="36" customHeight="1">
+      <x:c r="A18" s="7" t="str">
+        <x:v>I08</x:v>
+      </x:c>
+      <x:c r="B18" s="12" t="str">
+        <x:v>1 view AMP FP16</x:v>
+      </x:c>
+      <x:c r="C18" s="7" t="str">
+        <x:v>Tesla T4</x:v>
+      </x:c>
+      <x:c r="D18" s="7" t="str">
+        <x:v>amp</x:v>
+      </x:c>
+      <x:c r="E18" s="7" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="F18" s="7" t="n">
+        <x:v>224</x:v>
+      </x:c>
+      <x:c r="G18" s="7" t="n">
+        <x:v>224</x:v>
+      </x:c>
+      <x:c r="H18" s="7" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="I18" s="51" t="b">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="J18" s="42" t="n">
+        <x:v>7.083049499897243</x:v>
+      </x:c>
+      <x:c r="K18" s="42" t="n">
+        <x:v>10.559240600014162</x:v>
+      </x:c>
+      <x:c r="L18" s="42" t="n">
+        <x:v>11.857329199942797</x:v>
+      </x:c>
+      <x:c r="M18" s="42" t="n">
+        <x:v>7.568062009950154</x:v>
+      </x:c>
+      <x:c r="N18" s="44" t="n">
+        <x:v>132.1342238852224</x:v>
+      </x:c>
+      <x:c r="O18" s="7" t="n">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="P18" s="7" t="n">
+        <x:v>100</x:v>
+      </x:c>
+      <x:c r="Q18" s="7" t="str">
+        <x:v>2.8.0+cu128</x:v>
+      </x:c>
+      <x:c r="R18" s="51" t="b">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="S18" s="51" t="b">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="T18" s="12" t="str">
+        <x:v>normalized GPU input; tensor TTA + model + softmax/aggregation/T</x:v>
+      </x:c>
+      <x:c r="U18" s="7" t="str">
+        <x:v>step3/I08/latency_batch1.json</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="19" ht="36" customHeight="1">
+      <x:c r="A19" s="7" t="str">
+        <x:v>I08</x:v>
+      </x:c>
+      <x:c r="B19" s="12" t="str">
+        <x:v>1 view AMP FP16</x:v>
+      </x:c>
+      <x:c r="C19" s="7" t="str">
+        <x:v>Tesla T4</x:v>
+      </x:c>
+      <x:c r="D19" s="7" t="str">
+        <x:v>amp</x:v>
+      </x:c>
+      <x:c r="E19" s="7" t="n">
+        <x:v>32</x:v>
+      </x:c>
+      <x:c r="F19" s="7" t="n">
+        <x:v>224</x:v>
+      </x:c>
+      <x:c r="G19" s="7" t="n">
+        <x:v>224</x:v>
+      </x:c>
+      <x:c r="H19" s="7" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="I19" s="51" t="b">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="J19" s="42" t="n">
+        <x:v>44.336849000274015</x:v>
+      </x:c>
+      <x:c r="K19" s="42" t="n">
+        <x:v>44.857776350272616</x:v>
+      </x:c>
+      <x:c r="L19" s="42" t="n">
+        <x:v>45.68571830006932</x:v>
+      </x:c>
+      <x:c r="M19" s="42" t="n">
+        <x:v>44.385808240058395</x:v>
+      </x:c>
+      <x:c r="N19" s="44" t="n">
+        <x:v>720.9511613921644</x:v>
+      </x:c>
+      <x:c r="O19" s="7" t="n">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="P19" s="7" t="n">
+        <x:v>100</x:v>
+      </x:c>
+      <x:c r="Q19" s="7" t="str">
+        <x:v>2.8.0+cu128</x:v>
+      </x:c>
+      <x:c r="R19" s="51" t="b">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="S19" s="51" t="b">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="T19" s="12" t="str">
+        <x:v>normalized GPU input; tensor TTA + model + softmax/aggregation/T</x:v>
+      </x:c>
+      <x:c r="U19" s="7" t="str">
+        <x:v>step3/I08/latency_batch32.json</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="22">
+      <x:c r="A22" t="str">
+        <x:v>Raw samples: step3/Ixx/latency_batch1/32.json; batch 1 và 32.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="23">
+      <x:c r="A23" t="str">
         <x:v>10 warmup + 100 lần đo; synchronize trước/sau. Input sẵn trên GPU; gồm TTA/model/softmax/T.</x:v>
       </x:c>
     </x:row>
-    <x:row r="7">
-      <x:c r="A7" t="str">
+    <x:row r="24">
+      <x:c r="A24" t="str">
         <x:v>Không gồm decode/PIL/H2D/D2H. p95≤100 ms là ngưỡng pipeline GPU; chưa phải toàn bộ camera/robot.</x:v>
       </x:c>
     </x:row>
@@ -2623,6 +3986,1016 @@
     <x:mergeCell ref="A5:G5"/>
     <x:mergeCell ref="A6:G6"/>
     <x:mergeCell ref="A7:G7"/>
+    <x:mergeCell ref="A22:G22"/>
+    <x:mergeCell ref="A23:G23"/>
+    <x:mergeCell ref="A24:G24"/>
+  </x:mergeCells>
+  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</x:worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:sheetFormatPr defaultRowHeight="15"/>
+  <x:cols>
+    <x:col min="1" max="1" width="8.130000114440918" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="8.130000114440918" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="8.130000114440918" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="29.3799991607666" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="15" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="15" hidden="0" customWidth="1"/>
+    <x:col min="7" max="7" width="15" hidden="0" customWidth="1"/>
+    <x:col min="8" max="8" width="15" hidden="0" customWidth="1"/>
+    <x:col min="9" max="9" width="8.130000114440918" hidden="0" customWidth="1"/>
+    <x:col min="10" max="10" width="42.5" hidden="0" customWidth="1"/>
+    <x:col min="11" max="11" width="42.5" hidden="0" customWidth="1"/>
+  </x:cols>
+  <x:sheetData>
+    <x:row r="1" ht="44" customHeight="1">
+      <x:c r="A1" s="47" t="str">
+        <x:v>Hạng</x:v>
+      </x:c>
+      <x:c r="B1" s="47" t="str">
+        <x:v>ID</x:v>
+      </x:c>
+      <x:c r="C1" s="47" t="str">
+        <x:v>Bước</x:v>
+      </x:c>
+      <x:c r="D1" s="47" t="str">
+        <x:v>Cấu hình</x:v>
+      </x:c>
+      <x:c r="E1" s="47" t="str">
+        <x:v>Macro-F1 val</x:v>
+      </x:c>
+      <x:c r="F1" s="47" t="str">
+        <x:v>Top-1 val</x:v>
+      </x:c>
+      <x:c r="G1" s="47" t="str">
+        <x:v>ECE val</x:v>
+      </x:c>
+      <x:c r="H1" s="47" t="str">
+        <x:v>p95 (ms)</x:v>
+      </x:c>
+      <x:c r="I1" s="47" t="str">
+        <x:v>Số seed</x:v>
+      </x:c>
+      <x:c r="J1" s="47" t="str">
+        <x:v>Điều kiện đo</x:v>
+      </x:c>
+      <x:c r="K1" s="47" t="str">
+        <x:v>Ghi chú</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="2" ht="35" customHeight="1">
+      <x:c r="A2" s="52" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="B2" s="52" t="str">
+        <x:v>I09</x:v>
+      </x:c>
+      <x:c r="C2" s="52" t="str">
+        <x:v>I</x:v>
+      </x:c>
+      <x:c r="D2" s="53" t="str">
+        <x:v>Resolution 288</x:v>
+      </x:c>
+      <x:c r="E2" s="54" t="n">
+        <x:v>0.9698380941836109</x:v>
+      </x:c>
+      <x:c r="F2" s="54" t="n">
+        <x:v>0.9771493858897458</x:v>
+      </x:c>
+      <x:c r="G2" s="55" t="n">
+        <x:v>0.1038055720536991</x:v>
+      </x:c>
+      <x:c r="H2" s="56" t="n">
+        <x:v>9.068122750227303</x:v>
+      </x:c>
+      <x:c r="I2" s="52" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="J2" s="53" t="str">
+        <x:v>Lightning T4, 100 synchronized GPU pipeline timings</x:v>
+      </x:c>
+      <x:c r="K2" s="53" t="str">
+        <x:v>val only; no multi-seed test results</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="3" ht="35" customHeight="1">
+      <x:c r="A3" s="7" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="B3" s="7" t="str">
+        <x:v>I04</x:v>
+      </x:c>
+      <x:c r="C3" s="7" t="str">
+        <x:v>I</x:v>
+      </x:c>
+      <x:c r="D3" s="12" t="str">
+        <x:v>Resolution 256</x:v>
+      </x:c>
+      <x:c r="E3" s="40" t="n">
+        <x:v>0.9689643072792996</x:v>
+      </x:c>
+      <x:c r="F3" s="40" t="n">
+        <x:v>0.9765781205369894</x:v>
+      </x:c>
+      <x:c r="G3" s="41" t="n">
+        <x:v>0.09549411788631819</x:v>
+      </x:c>
+      <x:c r="H3" s="42" t="n">
+        <x:v>9.138116349868142</x:v>
+      </x:c>
+      <x:c r="I3" s="7" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="J3" s="12" t="str">
+        <x:v>Lightning T4, 100 synchronized GPU pipeline timings</x:v>
+      </x:c>
+      <x:c r="K3" s="12" t="str">
+        <x:v>val only; no multi-seed test results</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="4" ht="35" customHeight="1">
+      <x:c r="A4" s="7" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="B4" s="7" t="str">
+        <x:v>I10</x:v>
+      </x:c>
+      <x:c r="C4" s="7" t="str">
+        <x:v>I</x:v>
+      </x:c>
+      <x:c r="D4" s="12" t="str">
+        <x:v>Resolution 320</x:v>
+      </x:c>
+      <x:c r="E4" s="40" t="n">
+        <x:v>0.968106255766696</x:v>
+      </x:c>
+      <x:c r="F4" s="40" t="n">
+        <x:v>0.9762924878606113</x:v>
+      </x:c>
+      <x:c r="G4" s="41" t="n">
+        <x:v>0.11564186553556126</x:v>
+      </x:c>
+      <x:c r="H4" s="42" t="n">
+        <x:v>9.153301400033342</x:v>
+      </x:c>
+      <x:c r="I4" s="7" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="J4" s="12" t="str">
+        <x:v>Lightning T4, 100 synchronized GPU pipeline timings</x:v>
+      </x:c>
+      <x:c r="K4" s="12" t="str">
+        <x:v>val only; no multi-seed test results</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="5" ht="35" customHeight="1">
+      <x:c r="A5" s="7" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="B5" s="7" t="str">
+        <x:v>I02</x:v>
+      </x:c>
+      <x:c r="C5" s="7" t="str">
+        <x:v>I</x:v>
+      </x:c>
+      <x:c r="D5" s="12" t="str">
+        <x:v>5 crops / probability</x:v>
+      </x:c>
+      <x:c r="E5" s="40" t="n">
+        <x:v>0.9661639604452444</x:v>
+      </x:c>
+      <x:c r="F5" s="40" t="n">
+        <x:v>0.9754355898314767</x:v>
+      </x:c>
+      <x:c r="G5" s="41" t="n">
+        <x:v>0.09960301870037136</x:v>
+      </x:c>
+      <x:c r="H5" s="42" t="n">
+        <x:v>42.252744699828774</x:v>
+      </x:c>
+      <x:c r="I5" s="7" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="J5" s="12" t="str">
+        <x:v>Lightning T4, 100 synchronized GPU pipeline timings</x:v>
+      </x:c>
+      <x:c r="K5" s="12" t="str">
+        <x:v>val only; no multi-seed test results</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="6" ht="35" customHeight="1">
+      <x:c r="A6" s="7" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="B6" s="7" t="str">
+        <x:v>I03</x:v>
+      </x:c>
+      <x:c r="C6" s="7" t="str">
+        <x:v>I</x:v>
+      </x:c>
+      <x:c r="D6" s="12" t="str">
+        <x:v>Hflip TTA / logits</x:v>
+      </x:c>
+      <x:c r="E6" s="40" t="n">
+        <x:v>0.9642724549175057</x:v>
+      </x:c>
+      <x:c r="F6" s="40" t="n">
+        <x:v>0.9734361610968295</x:v>
+      </x:c>
+      <x:c r="G6" s="41" t="n">
+        <x:v>0.09718448681233922</x:v>
+      </x:c>
+      <x:c r="H6" s="42" t="n">
+        <x:v>16.35914885002876</x:v>
+      </x:c>
+      <x:c r="I6" s="7" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="J6" s="12" t="str">
+        <x:v>Lightning T4, 100 synchronized GPU pipeline timings</x:v>
+      </x:c>
+      <x:c r="K6" s="12" t="str">
+        <x:v>val only; no multi-seed test results</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="7" ht="35" customHeight="1">
+      <x:c r="A7" s="7" t="n">
+        <x:v>6</x:v>
+      </x:c>
+      <x:c r="B7" s="7" t="str">
+        <x:v>I01</x:v>
+      </x:c>
+      <x:c r="C7" s="7" t="str">
+        <x:v>I</x:v>
+      </x:c>
+      <x:c r="D7" s="12" t="str">
+        <x:v>Hflip TTA / probability</x:v>
+      </x:c>
+      <x:c r="E7" s="40" t="n">
+        <x:v>0.9642588606265972</x:v>
+      </x:c>
+      <x:c r="F7" s="40" t="n">
+        <x:v>0.9734361610968295</x:v>
+      </x:c>
+      <x:c r="G7" s="41" t="n">
+        <x:v>0.09708798446443855</x:v>
+      </x:c>
+      <x:c r="H7" s="42" t="n">
+        <x:v>18.862193050108544</x:v>
+      </x:c>
+      <x:c r="I7" s="7" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="J7" s="12" t="str">
+        <x:v>Lightning T4, 100 synchronized GPU pipeline timings</x:v>
+      </x:c>
+      <x:c r="K7" s="12" t="str">
+        <x:v>val only; no multi-seed test results</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="8" ht="35" customHeight="1">
+      <x:c r="A8" s="7" t="n">
+        <x:v>7</x:v>
+      </x:c>
+      <x:c r="B8" s="7" t="str">
+        <x:v>I07</x:v>
+      </x:c>
+      <x:c r="C8" s="7" t="str">
+        <x:v>I</x:v>
+      </x:c>
+      <x:c r="D8" s="12" t="str">
+        <x:v>1 view + temperature</x:v>
+      </x:c>
+      <x:c r="E8" s="40" t="n">
+        <x:v>0.9641032435221208</x:v>
+      </x:c>
+      <x:c r="F8" s="40" t="n">
+        <x:v>0.9737217937732077</x:v>
+      </x:c>
+      <x:c r="G8" s="41" t="n">
+        <x:v>0.004736394133104849</x:v>
+      </x:c>
+      <x:c r="H8" s="42" t="n">
+        <x:v>7.490706349949504</x:v>
+      </x:c>
+      <x:c r="I8" s="7" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="J8" s="12" t="str">
+        <x:v>Lightning T4, 100 synchronized GPU pipeline timings</x:v>
+      </x:c>
+      <x:c r="K8" s="12" t="str">
+        <x:v>val only; no multi-seed test results</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="9" ht="35" customHeight="1">
+      <x:c r="A9" s="7" t="n">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="B9" s="7" t="str">
+        <x:v>I08</x:v>
+      </x:c>
+      <x:c r="C9" s="7" t="str">
+        <x:v>I</x:v>
+      </x:c>
+      <x:c r="D9" s="12" t="str">
+        <x:v>1 view AMP FP16</x:v>
+      </x:c>
+      <x:c r="E9" s="40" t="n">
+        <x:v>0.9641032435221208</x:v>
+      </x:c>
+      <x:c r="F9" s="40" t="n">
+        <x:v>0.9737217937732077</x:v>
+      </x:c>
+      <x:c r="G9" s="41" t="n">
+        <x:v>0.09613235726078252</x:v>
+      </x:c>
+      <x:c r="H9" s="42" t="n">
+        <x:v>10.559240600014162</x:v>
+      </x:c>
+      <x:c r="I9" s="7" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="J9" s="12" t="str">
+        <x:v>Lightning T4, 100 synchronized GPU pipeline timings</x:v>
+      </x:c>
+      <x:c r="K9" s="12" t="str">
+        <x:v>val only; no multi-seed test results</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="10" ht="35" customHeight="1">
+      <x:c r="A10" s="7" t="n">
+        <x:v>9</x:v>
+      </x:c>
+      <x:c r="B10" s="7" t="str">
+        <x:v>I00</x:v>
+      </x:c>
+      <x:c r="C10" s="7" t="str">
+        <x:v>I</x:v>
+      </x:c>
+      <x:c r="D10" s="12" t="str">
+        <x:v>1 view FP32</x:v>
+      </x:c>
+      <x:c r="E10" s="40" t="n">
+        <x:v>0.9641032435221208</x:v>
+      </x:c>
+      <x:c r="F10" s="40" t="n">
+        <x:v>0.9737217937732077</x:v>
+      </x:c>
+      <x:c r="G10" s="41" t="n">
+        <x:v>0.09615286034275924</x:v>
+      </x:c>
+      <x:c r="H10" s="42" t="n">
+        <x:v>9.390229150073992</x:v>
+      </x:c>
+      <x:c r="I10" s="7" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="J10" s="12" t="str">
+        <x:v>Lightning T4, 100 synchronized GPU pipeline timings</x:v>
+      </x:c>
+      <x:c r="K10" s="12" t="str">
+        <x:v>val only; no multi-seed test results</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="11" ht="35" customHeight="1">
+      <x:c r="A11" s="7" t="n">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="B11" s="7" t="str">
+        <x:v>T04</x:v>
+      </x:c>
+      <x:c r="C11" s="7" t="str">
+        <x:v>T</x:v>
+      </x:c>
+      <x:c r="D11" s="12" t="str">
+        <x:v>CutMix alpha=1</x:v>
+      </x:c>
+      <x:c r="E11" s="40" t="n">
+        <x:v>0.9630413373883078</x:v>
+      </x:c>
+      <x:c r="F11" s="40" t="n">
+        <x:v>0.9720079977149386</x:v>
+      </x:c>
+      <x:c r="G11" s="41" t="n">
+        <x:v>0.025046328791773743</x:v>
+      </x:c>
+      <x:c r="H11" s="42"/>
+      <x:c r="I11" s="7" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="J11" s="12" t="str">
+        <x:v>No comparable p95; screening timings only</x:v>
+      </x:c>
+      <x:c r="K11" s="12" t="str">
+        <x:v>val only; no multi-seed test results</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="14">
+      <x:c r="A14" t="str">
+        <x:v>Top 10 cấu hình val, một seed. T00=B03 và T05=I00 được bỏ trùng; p95 chỉ so trong Lightning Bước 3.</x:v>
+      </x:c>
+    </x:row>
+  </x:sheetData>
+  <x:mergeCells>
+    <x:mergeCell ref="A14:G14"/>
+  </x:mergeCells>
+  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</x:worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:sheetFormatPr defaultRowHeight="15"/>
+  <x:cols>
+    <x:col min="1" max="1" width="8.130000114440918" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="8.130000114440918" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="15" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="29.3799991607666" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="15" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="15" hidden="0" customWidth="1"/>
+    <x:col min="7" max="7" width="15" hidden="0" customWidth="1"/>
+    <x:col min="8" max="8" width="15" hidden="0" customWidth="1"/>
+    <x:col min="9" max="9" width="15" hidden="0" customWidth="1"/>
+    <x:col min="10" max="10" width="15" hidden="0" customWidth="1"/>
+    <x:col min="11" max="11" width="15" hidden="0" customWidth="1"/>
+    <x:col min="12" max="12" width="15" hidden="0" customWidth="1"/>
+    <x:col min="13" max="13" width="15" hidden="0" customWidth="1"/>
+    <x:col min="14" max="14" width="29.3799991607666" hidden="0" customWidth="1"/>
+  </x:cols>
+  <x:sheetData>
+    <x:row r="1" ht="44" customHeight="1">
+      <x:c r="A1" s="47" t="str">
+        <x:v>ID</x:v>
+      </x:c>
+      <x:c r="B1" s="47" t="str">
+        <x:v>Seed</x:v>
+      </x:c>
+      <x:c r="C1" s="47" t="str">
+        <x:v>Công thức</x:v>
+      </x:c>
+      <x:c r="D1" s="47" t="str">
+        <x:v>Suy luận</x:v>
+      </x:c>
+      <x:c r="E1" s="47" t="str">
+        <x:v>T val</x:v>
+      </x:c>
+      <x:c r="F1" s="47" t="str">
+        <x:v>Macro-F1 val</x:v>
+      </x:c>
+      <x:c r="G1" s="47" t="str">
+        <x:v>Top-1 val</x:v>
+      </x:c>
+      <x:c r="H1" s="47" t="str">
+        <x:v>Macro-F1 test</x:v>
+      </x:c>
+      <x:c r="I1" s="47" t="str">
+        <x:v>Top-1 test</x:v>
+      </x:c>
+      <x:c r="J1" s="47" t="str">
+        <x:v>ECE test</x:v>
+      </x:c>
+      <x:c r="K1" s="47" t="str">
+        <x:v>ECE test chưa T</x:v>
+      </x:c>
+      <x:c r="L1" s="47" t="str">
+        <x:v>p95 (ms)</x:v>
+      </x:c>
+      <x:c r="M1" s="47" t="str">
+        <x:v>Checkpoint epoch</x:v>
+      </x:c>
+      <x:c r="N1" s="47" t="str">
+        <x:v>Trạng thái</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="2" ht="35" customHeight="1">
+      <x:c r="A2" s="7" t="str">
+        <x:v>F00</x:v>
+      </x:c>
+      <x:c r="B2" s="7" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="C2" s="7" t="str">
+        <x:v>T00</x:v>
+      </x:c>
+      <x:c r="D2" s="12" t="str">
+        <x:v>I00</x:v>
+      </x:c>
+      <x:c r="E2" s="39" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="F2" s="40"/>
+      <x:c r="G2" s="40"/>
+      <x:c r="H2" s="40"/>
+      <x:c r="I2" s="40"/>
+      <x:c r="J2" s="41"/>
+      <x:c r="K2" s="41"/>
+      <x:c r="L2" s="42"/>
+      <x:c r="M2" s="7"/>
+      <x:c r="N2" s="12" t="str">
+        <x:v>Chưa train/test</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="3" ht="35" customHeight="1">
+      <x:c r="A3" s="7" t="str">
+        <x:v>F00</x:v>
+      </x:c>
+      <x:c r="B3" s="7" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="C3" s="7" t="str">
+        <x:v>T00</x:v>
+      </x:c>
+      <x:c r="D3" s="12" t="str">
+        <x:v>I00</x:v>
+      </x:c>
+      <x:c r="E3" s="39" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="F3" s="40"/>
+      <x:c r="G3" s="40"/>
+      <x:c r="H3" s="40"/>
+      <x:c r="I3" s="40"/>
+      <x:c r="J3" s="41"/>
+      <x:c r="K3" s="41"/>
+      <x:c r="L3" s="42"/>
+      <x:c r="M3" s="7"/>
+      <x:c r="N3" s="12" t="str">
+        <x:v>Chưa train/test</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="4" ht="35" customHeight="1">
+      <x:c r="A4" s="7" t="str">
+        <x:v>F00</x:v>
+      </x:c>
+      <x:c r="B4" s="7" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="C4" s="7" t="str">
+        <x:v>T00</x:v>
+      </x:c>
+      <x:c r="D4" s="12" t="str">
+        <x:v>I00</x:v>
+      </x:c>
+      <x:c r="E4" s="39" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="F4" s="40"/>
+      <x:c r="G4" s="40"/>
+      <x:c r="H4" s="40"/>
+      <x:c r="I4" s="40"/>
+      <x:c r="J4" s="41"/>
+      <x:c r="K4" s="41"/>
+      <x:c r="L4" s="42"/>
+      <x:c r="M4" s="7"/>
+      <x:c r="N4" s="12" t="str">
+        <x:v>Chưa train/test</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="5" ht="35" customHeight="1">
+      <x:c r="A5" s="7" t="str">
+        <x:v>F01</x:v>
+      </x:c>
+      <x:c r="B5" s="7" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="C5" s="7" t="str">
+        <x:v>T05</x:v>
+      </x:c>
+      <x:c r="D5" s="12" t="str">
+        <x:v>I09 + own val-fit T</x:v>
+      </x:c>
+      <x:c r="E5" s="39"/>
+      <x:c r="F5" s="40"/>
+      <x:c r="G5" s="40"/>
+      <x:c r="H5" s="40"/>
+      <x:c r="I5" s="40"/>
+      <x:c r="J5" s="41"/>
+      <x:c r="K5" s="41"/>
+      <x:c r="L5" s="42"/>
+      <x:c r="M5" s="7"/>
+      <x:c r="N5" s="12" t="str">
+        <x:v>Chưa train/test</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="6" ht="35" customHeight="1">
+      <x:c r="A6" s="7" t="str">
+        <x:v>F01</x:v>
+      </x:c>
+      <x:c r="B6" s="7" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="C6" s="7" t="str">
+        <x:v>T05</x:v>
+      </x:c>
+      <x:c r="D6" s="12" t="str">
+        <x:v>I09 + own val-fit T</x:v>
+      </x:c>
+      <x:c r="E6" s="39"/>
+      <x:c r="F6" s="40"/>
+      <x:c r="G6" s="40"/>
+      <x:c r="H6" s="40"/>
+      <x:c r="I6" s="40"/>
+      <x:c r="J6" s="41"/>
+      <x:c r="K6" s="41"/>
+      <x:c r="L6" s="42"/>
+      <x:c r="M6" s="7"/>
+      <x:c r="N6" s="12" t="str">
+        <x:v>Chưa train/test</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="7" ht="35" customHeight="1">
+      <x:c r="A7" s="7" t="str">
+        <x:v>F01</x:v>
+      </x:c>
+      <x:c r="B7" s="7" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="C7" s="7" t="str">
+        <x:v>T05</x:v>
+      </x:c>
+      <x:c r="D7" s="12" t="str">
+        <x:v>I09 + own val-fit T</x:v>
+      </x:c>
+      <x:c r="E7" s="39"/>
+      <x:c r="F7" s="40"/>
+      <x:c r="G7" s="40"/>
+      <x:c r="H7" s="40"/>
+      <x:c r="I7" s="40"/>
+      <x:c r="J7" s="41"/>
+      <x:c r="K7" s="41"/>
+      <x:c r="L7" s="42"/>
+      <x:c r="M7" s="7"/>
+      <x:c r="N7" s="12" t="str">
+        <x:v>Chưa train/test</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="10">
+      <x:c r="A10" t="str">
+        <x:v>Chờ Bước 4: chưa có mean ± std, metric test hoặc dự đoán test. Không điền số val vào test.</x:v>
+      </x:c>
+    </x:row>
+  </x:sheetData>
+  <x:mergeCells>
+    <x:mergeCell ref="A10:G10"/>
+  </x:mergeCells>
+  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</x:worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:sheetFormatPr defaultRowHeight="15"/>
+  <x:cols>
+    <x:col min="1" max="1" width="8.130000114440918" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="29.3799991607666" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="15" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="15" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="15" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="15" hidden="0" customWidth="1"/>
+    <x:col min="7" max="7" width="29.3799991607666" hidden="0" customWidth="1"/>
+  </x:cols>
+  <x:sheetData>
+    <x:row r="1" ht="44" customHeight="1">
+      <x:c r="A1" s="47" t="str">
+        <x:v>ID</x:v>
+      </x:c>
+      <x:c r="B1" s="47" t="str">
+        <x:v>Lớp</x:v>
+      </x:c>
+      <x:c r="C1" s="47" t="str">
+        <x:v>Số ảnh test/seed</x:v>
+      </x:c>
+      <x:c r="D1" s="47" t="str">
+        <x:v>Precision test</x:v>
+      </x:c>
+      <x:c r="E1" s="47" t="str">
+        <x:v>Recall test</x:v>
+      </x:c>
+      <x:c r="F1" s="47" t="str">
+        <x:v>F1 test</x:v>
+      </x:c>
+      <x:c r="G1" s="47" t="str">
+        <x:v>Trạng thái</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="2" ht="35" customHeight="1">
+      <x:c r="A2" s="7" t="str">
+        <x:v>F00</x:v>
+      </x:c>
+      <x:c r="B2" s="12" t="str">
+        <x:v>Chinee Apple</x:v>
+      </x:c>
+      <x:c r="C2" s="7" t="n">
+        <x:v>226</x:v>
+      </x:c>
+      <x:c r="D2" s="40"/>
+      <x:c r="E2" s="40"/>
+      <x:c r="F2" s="40"/>
+      <x:c r="G2" s="12" t="str">
+        <x:v>Chưa có dự đoán test</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="3" ht="35" customHeight="1">
+      <x:c r="A3" s="7" t="str">
+        <x:v>F00</x:v>
+      </x:c>
+      <x:c r="B3" s="12" t="str">
+        <x:v>Lantana</x:v>
+      </x:c>
+      <x:c r="C3" s="7" t="n">
+        <x:v>213</x:v>
+      </x:c>
+      <x:c r="D3" s="40"/>
+      <x:c r="E3" s="40"/>
+      <x:c r="F3" s="40"/>
+      <x:c r="G3" s="12" t="str">
+        <x:v>Chưa có dự đoán test</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="4" ht="35" customHeight="1">
+      <x:c r="A4" s="7" t="str">
+        <x:v>F00</x:v>
+      </x:c>
+      <x:c r="B4" s="12" t="str">
+        <x:v>Parkinsonia</x:v>
+      </x:c>
+      <x:c r="C4" s="7" t="n">
+        <x:v>207</x:v>
+      </x:c>
+      <x:c r="D4" s="40"/>
+      <x:c r="E4" s="40"/>
+      <x:c r="F4" s="40"/>
+      <x:c r="G4" s="12" t="str">
+        <x:v>Chưa có dự đoán test</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="5" ht="35" customHeight="1">
+      <x:c r="A5" s="7" t="str">
+        <x:v>F00</x:v>
+      </x:c>
+      <x:c r="B5" s="12" t="str">
+        <x:v>Parthenium</x:v>
+      </x:c>
+      <x:c r="C5" s="7" t="n">
+        <x:v>205</x:v>
+      </x:c>
+      <x:c r="D5" s="40"/>
+      <x:c r="E5" s="40"/>
+      <x:c r="F5" s="40"/>
+      <x:c r="G5" s="12" t="str">
+        <x:v>Chưa có dự đoán test</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="6" ht="35" customHeight="1">
+      <x:c r="A6" s="7" t="str">
+        <x:v>F00</x:v>
+      </x:c>
+      <x:c r="B6" s="12" t="str">
+        <x:v>Prickly Acacia</x:v>
+      </x:c>
+      <x:c r="C6" s="7" t="n">
+        <x:v>213</x:v>
+      </x:c>
+      <x:c r="D6" s="40"/>
+      <x:c r="E6" s="40"/>
+      <x:c r="F6" s="40"/>
+      <x:c r="G6" s="12" t="str">
+        <x:v>Chưa có dự đoán test</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="7" ht="35" customHeight="1">
+      <x:c r="A7" s="7" t="str">
+        <x:v>F00</x:v>
+      </x:c>
+      <x:c r="B7" s="12" t="str">
+        <x:v>Rubber Vine</x:v>
+      </x:c>
+      <x:c r="C7" s="7" t="n">
+        <x:v>202</x:v>
+      </x:c>
+      <x:c r="D7" s="40"/>
+      <x:c r="E7" s="40"/>
+      <x:c r="F7" s="40"/>
+      <x:c r="G7" s="12" t="str">
+        <x:v>Chưa có dự đoán test</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="8" ht="35" customHeight="1">
+      <x:c r="A8" s="7" t="str">
+        <x:v>F00</x:v>
+      </x:c>
+      <x:c r="B8" s="12" t="str">
+        <x:v>Siam Weed</x:v>
+      </x:c>
+      <x:c r="C8" s="7" t="n">
+        <x:v>215</x:v>
+      </x:c>
+      <x:c r="D8" s="40"/>
+      <x:c r="E8" s="40"/>
+      <x:c r="F8" s="40"/>
+      <x:c r="G8" s="12" t="str">
+        <x:v>Chưa có dự đoán test</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="9" ht="35" customHeight="1">
+      <x:c r="A9" s="7" t="str">
+        <x:v>F00</x:v>
+      </x:c>
+      <x:c r="B9" s="12" t="str">
+        <x:v>Snake Weed</x:v>
+      </x:c>
+      <x:c r="C9" s="7" t="n">
+        <x:v>204</x:v>
+      </x:c>
+      <x:c r="D9" s="40"/>
+      <x:c r="E9" s="40"/>
+      <x:c r="F9" s="40"/>
+      <x:c r="G9" s="12" t="str">
+        <x:v>Chưa có dự đoán test</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="10" ht="35" customHeight="1">
+      <x:c r="A10" s="7" t="str">
+        <x:v>F00</x:v>
+      </x:c>
+      <x:c r="B10" s="12" t="str">
+        <x:v>Negatives</x:v>
+      </x:c>
+      <x:c r="C10" s="7" t="n">
+        <x:v>1822</x:v>
+      </x:c>
+      <x:c r="D10" s="40"/>
+      <x:c r="E10" s="40"/>
+      <x:c r="F10" s="40"/>
+      <x:c r="G10" s="12" t="str">
+        <x:v>Chưa có dự đoán test</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="11" ht="35" customHeight="1">
+      <x:c r="A11" s="7" t="str">
+        <x:v>F01</x:v>
+      </x:c>
+      <x:c r="B11" s="12" t="str">
+        <x:v>Chinee Apple</x:v>
+      </x:c>
+      <x:c r="C11" s="7" t="n">
+        <x:v>226</x:v>
+      </x:c>
+      <x:c r="D11" s="40"/>
+      <x:c r="E11" s="40"/>
+      <x:c r="F11" s="40"/>
+      <x:c r="G11" s="12" t="str">
+        <x:v>Chưa có dự đoán test</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="12" ht="35" customHeight="1">
+      <x:c r="A12" s="7" t="str">
+        <x:v>F01</x:v>
+      </x:c>
+      <x:c r="B12" s="12" t="str">
+        <x:v>Lantana</x:v>
+      </x:c>
+      <x:c r="C12" s="7" t="n">
+        <x:v>213</x:v>
+      </x:c>
+      <x:c r="D12" s="40"/>
+      <x:c r="E12" s="40"/>
+      <x:c r="F12" s="40"/>
+      <x:c r="G12" s="12" t="str">
+        <x:v>Chưa có dự đoán test</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="13" ht="35" customHeight="1">
+      <x:c r="A13" s="7" t="str">
+        <x:v>F01</x:v>
+      </x:c>
+      <x:c r="B13" s="12" t="str">
+        <x:v>Parkinsonia</x:v>
+      </x:c>
+      <x:c r="C13" s="7" t="n">
+        <x:v>207</x:v>
+      </x:c>
+      <x:c r="D13" s="40"/>
+      <x:c r="E13" s="40"/>
+      <x:c r="F13" s="40"/>
+      <x:c r="G13" s="12" t="str">
+        <x:v>Chưa có dự đoán test</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="14" ht="35" customHeight="1">
+      <x:c r="A14" s="7" t="str">
+        <x:v>F01</x:v>
+      </x:c>
+      <x:c r="B14" s="12" t="str">
+        <x:v>Parthenium</x:v>
+      </x:c>
+      <x:c r="C14" s="7" t="n">
+        <x:v>205</x:v>
+      </x:c>
+      <x:c r="D14" s="40"/>
+      <x:c r="E14" s="40"/>
+      <x:c r="F14" s="40"/>
+      <x:c r="G14" s="12" t="str">
+        <x:v>Chưa có dự đoán test</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="15" ht="35" customHeight="1">
+      <x:c r="A15" s="7" t="str">
+        <x:v>F01</x:v>
+      </x:c>
+      <x:c r="B15" s="12" t="str">
+        <x:v>Prickly Acacia</x:v>
+      </x:c>
+      <x:c r="C15" s="7" t="n">
+        <x:v>213</x:v>
+      </x:c>
+      <x:c r="D15" s="40"/>
+      <x:c r="E15" s="40"/>
+      <x:c r="F15" s="40"/>
+      <x:c r="G15" s="12" t="str">
+        <x:v>Chưa có dự đoán test</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="16" ht="35" customHeight="1">
+      <x:c r="A16" s="7" t="str">
+        <x:v>F01</x:v>
+      </x:c>
+      <x:c r="B16" s="12" t="str">
+        <x:v>Rubber Vine</x:v>
+      </x:c>
+      <x:c r="C16" s="7" t="n">
+        <x:v>202</x:v>
+      </x:c>
+      <x:c r="D16" s="40"/>
+      <x:c r="E16" s="40"/>
+      <x:c r="F16" s="40"/>
+      <x:c r="G16" s="12" t="str">
+        <x:v>Chưa có dự đoán test</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="17" ht="35" customHeight="1">
+      <x:c r="A17" s="7" t="str">
+        <x:v>F01</x:v>
+      </x:c>
+      <x:c r="B17" s="12" t="str">
+        <x:v>Siam Weed</x:v>
+      </x:c>
+      <x:c r="C17" s="7" t="n">
+        <x:v>215</x:v>
+      </x:c>
+      <x:c r="D17" s="40"/>
+      <x:c r="E17" s="40"/>
+      <x:c r="F17" s="40"/>
+      <x:c r="G17" s="12" t="str">
+        <x:v>Chưa có dự đoán test</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="18" ht="35" customHeight="1">
+      <x:c r="A18" s="7" t="str">
+        <x:v>F01</x:v>
+      </x:c>
+      <x:c r="B18" s="12" t="str">
+        <x:v>Snake Weed</x:v>
+      </x:c>
+      <x:c r="C18" s="7" t="n">
+        <x:v>204</x:v>
+      </x:c>
+      <x:c r="D18" s="40"/>
+      <x:c r="E18" s="40"/>
+      <x:c r="F18" s="40"/>
+      <x:c r="G18" s="12" t="str">
+        <x:v>Chưa có dự đoán test</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="19" ht="35" customHeight="1">
+      <x:c r="A19" s="7" t="str">
+        <x:v>F01</x:v>
+      </x:c>
+      <x:c r="B19" s="12" t="str">
+        <x:v>Negatives</x:v>
+      </x:c>
+      <x:c r="C19" s="7" t="n">
+        <x:v>1822</x:v>
+      </x:c>
+      <x:c r="D19" s="40"/>
+      <x:c r="E19" s="40"/>
+      <x:c r="F19" s="40"/>
+      <x:c r="G19" s="12" t="str">
+        <x:v>Chưa có dự đoán test</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="22">
+      <x:c r="A22" t="str">
+        <x:v>Chờ Bước 4: chưa có mean ± std, metric test hoặc dự đoán test. Không điền số val vào test.</x:v>
+      </x:c>
+    </x:row>
+  </x:sheetData>
+  <x:mergeCells>
+    <x:mergeCell ref="A22:G22"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>

</xml_diff>

<commit_message>
Complete paired-seed finals, verified workbook and DeepWeeds report
</commit_message>
<xml_diff>
--- a/results.xlsx
+++ b/results.xlsx
@@ -2,13 +2,13 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Backbones" sheetId="1" r:id="R53d35f168295427e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Training" sheetId="2" r:id="Ra9d2e6141fd643eb"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Inference" sheetId="3" r:id="R5c97a44c9374414f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Latency" sheetId="4" r:id="Rb3fe4bd9c7894eed"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="5" r:id="R5e78d8ee7b494b23"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Final" sheetId="6" r:id="R0a8ccc05fdcd4087"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="PerClass" sheetId="7" r:id="R6505d689bf0e4acb"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Backbones" sheetId="1" r:id="R450f78bbc30d4f4a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Training" sheetId="2" r:id="R5086a451f0384992"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Inference" sheetId="3" r:id="R9682f6a8c1b94d92"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Latency" sheetId="4" r:id="Rd013906bf5814d15"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="5" r:id="R1d32c434c98f429d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Final" sheetId="6" r:id="R2b6ab2d17f8e4c9a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="PerClass" sheetId="7" r:id="R94a4d458884041d2"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -58,7 +58,7 @@
       <x:name val="Arial"/>
     </x:font>
   </x:fonts>
-  <x:fills count="10">
+  <x:fills count="26">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -105,6 +105,86 @@
         <x:fgColor rgb="FFE4F0E9"/>
       </x:patternFill>
     </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF243B53"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFE4F0E9"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFEDF1F5"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFDDEDE4"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF243B53"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFE4F0E9"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFEDF1F5"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFDDEDE4"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF243B53"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFE4F0E9"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFEDF1F5"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFDDEDE4"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF243B53"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFE4F0E9"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFEDF1F5"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFDDEDE4"/>
+      </x:patternFill>
+    </x:fill>
   </x:fills>
   <x:borders count="1">
     <x:border/>
@@ -112,7 +192,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="57">
+  <x:cellXfs count="221">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyAlignment="1">
       <x:alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -292,6 +372,440 @@
     </x:xf>
     <x:xf numFmtId="164" fontId="3" fillId="9" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="10" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="10" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="10" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="11" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="11" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="3" fillId="11" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="205" fontId="3" fillId="11" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="164" fontId="3" fillId="11" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="12" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="12" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="204" fontId="3" fillId="12" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="3" fillId="12" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="205" fontId="3" fillId="12" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="164" fontId="3" fillId="12" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="4" fillId="12" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="4" fillId="12" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="204" fontId="4" fillId="12" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="4" fillId="12" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="205" fontId="4" fillId="12" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="164" fontId="4" fillId="12" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="13" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="13" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="204" fontId="3" fillId="13" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="3" fillId="13" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="205" fontId="3" fillId="13" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="164" fontId="3" fillId="13" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="4" fillId="13" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="4" fillId="13" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="204" fontId="4" fillId="13" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="4" fillId="13" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="205" fontId="4" fillId="13" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="164" fontId="4" fillId="13" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="10" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="1" fillId="10" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="1" fillId="10" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="205" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="164" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="3" fillId="13" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="200" fontId="3" fillId="13" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="205" fontId="3" fillId="13" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="164" fontId="3" fillId="13" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="202" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="3" fillId="14" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="14" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="14" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="15" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="15" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="3" fillId="15" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="205" fontId="3" fillId="15" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="164" fontId="3" fillId="15" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="16" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="16" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="204" fontId="3" fillId="16" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="3" fillId="16" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="205" fontId="3" fillId="16" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="164" fontId="3" fillId="16" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="4" fillId="16" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="4" fillId="16" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="204" fontId="4" fillId="16" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="4" fillId="16" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="205" fontId="4" fillId="16" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="164" fontId="4" fillId="16" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="17" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="17" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="204" fontId="3" fillId="17" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="3" fillId="17" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="205" fontId="3" fillId="17" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="164" fontId="3" fillId="17" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="4" fillId="17" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="4" fillId="17" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="204" fontId="4" fillId="17" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="4" fillId="17" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="205" fontId="4" fillId="17" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="164" fontId="4" fillId="17" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="14" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="1" fillId="14" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="1" fillId="14" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="17" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="200" fontId="3" fillId="17" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="205" fontId="3" fillId="17" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="164" fontId="3" fillId="17" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="3" fillId="18" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="18" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="18" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="19" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="19" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="3" fillId="19" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="205" fontId="3" fillId="19" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="164" fontId="3" fillId="19" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="20" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="20" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="204" fontId="3" fillId="20" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="3" fillId="20" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="205" fontId="3" fillId="20" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="164" fontId="3" fillId="20" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="4" fillId="20" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="4" fillId="20" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="204" fontId="4" fillId="20" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="4" fillId="20" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="205" fontId="4" fillId="20" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="164" fontId="4" fillId="20" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="21" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="21" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="204" fontId="3" fillId="21" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="3" fillId="21" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="205" fontId="3" fillId="21" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="164" fontId="3" fillId="21" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="4" fillId="21" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="4" fillId="21" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="204" fontId="4" fillId="21" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="4" fillId="21" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="205" fontId="4" fillId="21" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="164" fontId="4" fillId="21" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="18" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="1" fillId="18" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="1" fillId="18" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="21" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="200" fontId="3" fillId="21" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="205" fontId="3" fillId="21" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="164" fontId="3" fillId="21" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="202" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="4" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="4" fillId="18" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="22" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="22" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="22" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="23" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="23" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="3" fillId="23" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="205" fontId="3" fillId="23" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="164" fontId="3" fillId="23" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="24" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="24" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="204" fontId="3" fillId="24" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="3" fillId="24" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="205" fontId="3" fillId="24" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="164" fontId="3" fillId="24" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="4" fillId="24" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="4" fillId="24" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="204" fontId="4" fillId="24" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="4" fillId="24" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="205" fontId="4" fillId="24" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="164" fontId="4" fillId="24" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="25" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="25" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="204" fontId="3" fillId="25" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="3" fillId="25" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="205" fontId="3" fillId="25" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="164" fontId="3" fillId="25" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="4" fillId="25" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="4" fillId="25" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="204" fontId="4" fillId="25" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="4" fillId="25" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="205" fontId="4" fillId="25" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="164" fontId="4" fillId="25" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="22" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="1" fillId="22" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="1" fillId="22" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="25" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="200" fontId="3" fillId="25" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="205" fontId="3" fillId="25" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="164" fontId="3" fillId="25" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="4" fillId="22" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
     </x:xf>
   </x:cellXfs>
   <x:cellStyles count="1">
@@ -652,6 +1166,7 @@
     <x:col min="17" max="17" width="22" customWidth="1"/>
     <x:col min="18" max="18" width="48" customWidth="1"/>
     <x:col min="19" max="19" width="48" customWidth="1"/>
+    <x:col min="20" max="20" width="11.25" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="42" customHeight="1">
@@ -750,6 +1265,9 @@
           <x:t xml:space="preserve">curve_path</x:t>
         </x:is>
       </x:c>
+      <x:c r="T1" s="183" t="str">
+        <x:v>Crop size</x:v>
+      </x:c>
     </x:row>
     <x:row r="2">
       <x:c r="A2" s="2" t="inlineStr">
@@ -825,6 +1343,9 @@
           <x:t xml:space="preserve">curves/B01_resnet50_seed0.png</x:t>
         </x:is>
       </x:c>
+      <x:c r="T2" s="7" t="n">
+        <x:v>224</x:v>
+      </x:c>
     </x:row>
     <x:row r="3">
       <x:c r="A3" s="2" t="inlineStr">
@@ -900,6 +1421,9 @@
           <x:t xml:space="preserve">curves/B02_resnext50_32x4d_seed0.png</x:t>
         </x:is>
       </x:c>
+      <x:c r="T3" s="7" t="n">
+        <x:v>224</x:v>
+      </x:c>
     </x:row>
     <x:row r="4">
       <x:c r="A4" s="2" t="inlineStr">
@@ -975,6 +1499,9 @@
           <x:t xml:space="preserve">curves/B03_convnext_tiny_seed0.png</x:t>
         </x:is>
       </x:c>
+      <x:c r="T4" s="7" t="n">
+        <x:v>224</x:v>
+      </x:c>
     </x:row>
     <x:row r="5">
       <x:c r="A5" s="2" t="inlineStr">
@@ -1050,6 +1577,9 @@
           <x:t xml:space="preserve">curves/B04_deit_small_patch16_224_seed0.png</x:t>
         </x:is>
       </x:c>
+      <x:c r="T5" s="7" t="n">
+        <x:v>224</x:v>
+      </x:c>
     </x:row>
     <x:row r="6">
       <x:c r="A6" s="2" t="inlineStr">
@@ -1124,6 +1654,9 @@
         <x:is>
           <x:t xml:space="preserve">curves/B05_efficientnet_b0_seed0.png</x:t>
         </x:is>
+      </x:c>
+      <x:c r="T6" s="7" t="n">
+        <x:v>224</x:v>
       </x:c>
     </x:row>
     <x:row r="9">
@@ -2708,8 +3241,8 @@
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
-    <x:col min="1" max="1" width="8.130000114440918" hidden="0" customWidth="1"/>
-    <x:col min="2" max="2" width="28.1299991607666" hidden="0" customWidth="1"/>
+    <x:col min="1" max="1" width="14.380000114440918" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="30" hidden="0" customWidth="1"/>
     <x:col min="3" max="3" width="14.380000114440918" hidden="0" customWidth="1"/>
     <x:col min="4" max="4" width="14.380000114440918" hidden="0" customWidth="1"/>
     <x:col min="5" max="5" width="14.380000114440918" hidden="0" customWidth="1"/>
@@ -2727,80 +3260,88 @@
     <x:col min="17" max="17" width="14.380000114440918" hidden="0" customWidth="1"/>
     <x:col min="18" max="18" width="14.380000114440918" hidden="0" customWidth="1"/>
     <x:col min="19" max="19" width="14.380000114440918" hidden="0" customWidth="1"/>
-    <x:col min="20" max="20" width="56.25" hidden="0" customWidth="1"/>
-    <x:col min="21" max="21" width="41.880001068115234" hidden="0" customWidth="1"/>
+    <x:col min="20" max="20" width="52.5" hidden="0" customWidth="1"/>
+    <x:col min="21" max="21" width="52.5" hidden="0" customWidth="1"/>
+    <x:col min="22" max="22" width="8.130000114440918" hidden="0" customWidth="1"/>
+    <x:col min="23" max="23" width="14.380000114440918" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
-    <x:row r="1" ht="45" customHeight="1">
-      <x:c r="A1" s="48" t="str">
-        <x:v>exp_id</x:v>
-      </x:c>
-      <x:c r="B1" s="48" t="str">
+    <x:row r="1" ht="44" customHeight="1">
+      <x:c r="A1" s="183" t="str">
+        <x:v>ID</x:v>
+      </x:c>
+      <x:c r="B1" s="183" t="str">
         <x:v>Phương pháp</x:v>
       </x:c>
-      <x:c r="C1" s="48" t="str">
-        <x:v>gpu</x:v>
-      </x:c>
-      <x:c r="D1" s="48" t="str">
+      <x:c r="C1" s="183" t="str">
+        <x:v>GPU</x:v>
+      </x:c>
+      <x:c r="D1" s="183" t="str">
         <x:v>dtype</x:v>
       </x:c>
-      <x:c r="E1" s="48" t="str">
-        <x:v>batch</x:v>
-      </x:c>
-      <x:c r="F1" s="48" t="str">
+      <x:c r="E1" s="183" t="str">
+        <x:v>Batch</x:v>
+      </x:c>
+      <x:c r="F1" s="183" t="str">
         <x:v>Crop size</x:v>
       </x:c>
-      <x:c r="G1" s="48" t="str">
+      <x:c r="G1" s="183" t="str">
         <x:v>Input size</x:v>
       </x:c>
-      <x:c r="H1" s="48" t="str">
+      <x:c r="H1" s="183" t="str">
         <x:v>K</x:v>
       </x:c>
-      <x:c r="I1" s="48" t="str">
-        <x:v>fused_bn</x:v>
-      </x:c>
-      <x:c r="J1" s="48" t="str">
+      <x:c r="I1" s="183" t="str">
+        <x:v>Gộp BN</x:v>
+      </x:c>
+      <x:c r="J1" s="183" t="str">
         <x:v>p50 (ms)</x:v>
       </x:c>
-      <x:c r="K1" s="48" t="str">
+      <x:c r="K1" s="183" t="str">
         <x:v>p95 (ms)</x:v>
       </x:c>
-      <x:c r="L1" s="48" t="str">
+      <x:c r="L1" s="183" t="str">
         <x:v>p99 (ms)</x:v>
       </x:c>
-      <x:c r="M1" s="48" t="str">
+      <x:c r="M1" s="183" t="str">
         <x:v>Mean (ms)</x:v>
       </x:c>
-      <x:c r="N1" s="48" t="str">
+      <x:c r="N1" s="183" t="str">
         <x:v>Ảnh/s</x:v>
       </x:c>
-      <x:c r="O1" s="48" t="str">
-        <x:v>warmup</x:v>
-      </x:c>
-      <x:c r="P1" s="48" t="str">
+      <x:c r="O1" s="183" t="str">
+        <x:v>Warmup</x:v>
+      </x:c>
+      <x:c r="P1" s="183" t="str">
         <x:v>Lần đo</x:v>
       </x:c>
-      <x:c r="Q1" s="48" t="str">
+      <x:c r="Q1" s="183" t="str">
         <x:v>torch</x:v>
       </x:c>
-      <x:c r="R1" s="48" t="str">
+      <x:c r="R1" s="183" t="str">
         <x:v>Gồm tiền xử lý</x:v>
       </x:c>
-      <x:c r="S1" s="48" t="str">
+      <x:c r="S1" s="183" t="str">
         <x:v>Gồm transfer</x:v>
       </x:c>
-      <x:c r="T1" s="48" t="str">
+      <x:c r="T1" s="183" t="str">
         <x:v>Phạm vi đo</x:v>
       </x:c>
-      <x:c r="U1" s="48" t="str">
+      <x:c r="U1" s="183" t="str">
         <x:v>Nguồn số đo</x:v>
       </x:c>
-    </x:row>
-    <x:row r="2" ht="36" customHeight="1">
+      <x:c r="V1" s="183" t="str">
+        <x:v>Seed</x:v>
+      </x:c>
+      <x:c r="W1" s="183" t="str">
+        <x:v>T val</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="2" ht="30" customHeight="1">
       <x:c r="A2" s="7" t="str">
         <x:v>I00</x:v>
       </x:c>
-      <x:c r="B2" s="12" t="str">
+      <x:c r="B2" s="7" t="str">
         <x:v>1 view FP32</x:v>
       </x:c>
       <x:c r="C2" s="7" t="str">
@@ -2854,18 +3395,24 @@
       <x:c r="S2" s="51" t="b">
         <x:v>0</x:v>
       </x:c>
-      <x:c r="T2" s="12" t="str">
+      <x:c r="T2" s="7" t="str">
         <x:v>normalized GPU input; tensor TTA + model + softmax/aggregation/T</x:v>
       </x:c>
       <x:c r="U2" s="7" t="str">
         <x:v>step3/I00/latency_batch1.json</x:v>
       </x:c>
-    </x:row>
-    <x:row r="3" ht="36" customHeight="1">
+      <x:c r="V2" s="7" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="W2" s="39" t="n">
+        <x:v>1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="3" ht="30" customHeight="1">
       <x:c r="A3" s="7" t="str">
         <x:v>I00</x:v>
       </x:c>
-      <x:c r="B3" s="12" t="str">
+      <x:c r="B3" s="7" t="str">
         <x:v>1 view FP32</x:v>
       </x:c>
       <x:c r="C3" s="7" t="str">
@@ -2919,18 +3466,24 @@
       <x:c r="S3" s="51" t="b">
         <x:v>0</x:v>
       </x:c>
-      <x:c r="T3" s="12" t="str">
+      <x:c r="T3" s="7" t="str">
         <x:v>normalized GPU input; tensor TTA + model + softmax/aggregation/T</x:v>
       </x:c>
       <x:c r="U3" s="7" t="str">
         <x:v>step3/I00/latency_batch32.json</x:v>
       </x:c>
-    </x:row>
-    <x:row r="4" ht="36" customHeight="1">
+      <x:c r="V3" s="7" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="W3" s="39" t="n">
+        <x:v>1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="4" ht="30" customHeight="1">
       <x:c r="A4" s="7" t="str">
         <x:v>I01</x:v>
       </x:c>
-      <x:c r="B4" s="12" t="str">
+      <x:c r="B4" s="7" t="str">
         <x:v>Hflip TTA / probability</x:v>
       </x:c>
       <x:c r="C4" s="7" t="str">
@@ -2984,18 +3537,24 @@
       <x:c r="S4" s="51" t="b">
         <x:v>0</x:v>
       </x:c>
-      <x:c r="T4" s="12" t="str">
+      <x:c r="T4" s="7" t="str">
         <x:v>normalized GPU input; tensor TTA + model + softmax/aggregation/T</x:v>
       </x:c>
       <x:c r="U4" s="7" t="str">
         <x:v>step3/I01/latency_batch1.json</x:v>
       </x:c>
-    </x:row>
-    <x:row r="5" ht="36" customHeight="1">
+      <x:c r="V4" s="7" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="W4" s="39" t="n">
+        <x:v>1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="5" ht="30" customHeight="1">
       <x:c r="A5" s="7" t="str">
         <x:v>I01</x:v>
       </x:c>
-      <x:c r="B5" s="12" t="str">
+      <x:c r="B5" s="7" t="str">
         <x:v>Hflip TTA / probability</x:v>
       </x:c>
       <x:c r="C5" s="7" t="str">
@@ -3049,18 +3608,24 @@
       <x:c r="S5" s="51" t="b">
         <x:v>0</x:v>
       </x:c>
-      <x:c r="T5" s="12" t="str">
+      <x:c r="T5" s="7" t="str">
         <x:v>normalized GPU input; tensor TTA + model + softmax/aggregation/T</x:v>
       </x:c>
       <x:c r="U5" s="7" t="str">
         <x:v>step3/I01/latency_batch32.json</x:v>
       </x:c>
-    </x:row>
-    <x:row r="6" ht="36" customHeight="1">
+      <x:c r="V5" s="7" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="W5" s="39" t="n">
+        <x:v>1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="6" ht="30" customHeight="1">
       <x:c r="A6" s="7" t="str">
         <x:v>I02</x:v>
       </x:c>
-      <x:c r="B6" s="12" t="str">
+      <x:c r="B6" s="7" t="str">
         <x:v>5 crops / probability</x:v>
       </x:c>
       <x:c r="C6" s="7" t="str">
@@ -3114,18 +3679,24 @@
       <x:c r="S6" s="51" t="b">
         <x:v>0</x:v>
       </x:c>
-      <x:c r="T6" s="12" t="str">
+      <x:c r="T6" s="7" t="str">
         <x:v>normalized GPU input; tensor TTA + model + softmax/aggregation/T</x:v>
       </x:c>
       <x:c r="U6" s="7" t="str">
         <x:v>step3/I02/latency_batch1.json</x:v>
       </x:c>
-    </x:row>
-    <x:row r="7" ht="36" customHeight="1">
+      <x:c r="V6" s="7" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="W6" s="39" t="n">
+        <x:v>1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="7" ht="30" customHeight="1">
       <x:c r="A7" s="7" t="str">
         <x:v>I02</x:v>
       </x:c>
-      <x:c r="B7" s="12" t="str">
+      <x:c r="B7" s="7" t="str">
         <x:v>5 crops / probability</x:v>
       </x:c>
       <x:c r="C7" s="7" t="str">
@@ -3179,18 +3750,24 @@
       <x:c r="S7" s="51" t="b">
         <x:v>0</x:v>
       </x:c>
-      <x:c r="T7" s="12" t="str">
+      <x:c r="T7" s="7" t="str">
         <x:v>normalized GPU input; tensor TTA + model + softmax/aggregation/T</x:v>
       </x:c>
       <x:c r="U7" s="7" t="str">
         <x:v>step3/I02/latency_batch32.json</x:v>
       </x:c>
-    </x:row>
-    <x:row r="8" ht="36" customHeight="1">
+      <x:c r="V7" s="7" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="W7" s="39" t="n">
+        <x:v>1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="8" ht="30" customHeight="1">
       <x:c r="A8" s="7" t="str">
         <x:v>I03</x:v>
       </x:c>
-      <x:c r="B8" s="12" t="str">
+      <x:c r="B8" s="7" t="str">
         <x:v>Hflip TTA / logits</x:v>
       </x:c>
       <x:c r="C8" s="7" t="str">
@@ -3244,18 +3821,24 @@
       <x:c r="S8" s="51" t="b">
         <x:v>0</x:v>
       </x:c>
-      <x:c r="T8" s="12" t="str">
+      <x:c r="T8" s="7" t="str">
         <x:v>normalized GPU input; tensor TTA + model + softmax/aggregation/T</x:v>
       </x:c>
       <x:c r="U8" s="7" t="str">
         <x:v>step3/I03/latency_batch1.json</x:v>
       </x:c>
-    </x:row>
-    <x:row r="9" ht="36" customHeight="1">
+      <x:c r="V8" s="7" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="W8" s="39" t="n">
+        <x:v>1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="9" ht="30" customHeight="1">
       <x:c r="A9" s="7" t="str">
         <x:v>I03</x:v>
       </x:c>
-      <x:c r="B9" s="12" t="str">
+      <x:c r="B9" s="7" t="str">
         <x:v>Hflip TTA / logits</x:v>
       </x:c>
       <x:c r="C9" s="7" t="str">
@@ -3309,18 +3892,24 @@
       <x:c r="S9" s="51" t="b">
         <x:v>0</x:v>
       </x:c>
-      <x:c r="T9" s="12" t="str">
+      <x:c r="T9" s="7" t="str">
         <x:v>normalized GPU input; tensor TTA + model + softmax/aggregation/T</x:v>
       </x:c>
       <x:c r="U9" s="7" t="str">
         <x:v>step3/I03/latency_batch32.json</x:v>
       </x:c>
-    </x:row>
-    <x:row r="10" ht="36" customHeight="1">
+      <x:c r="V9" s="7" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="W9" s="39" t="n">
+        <x:v>1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="10" ht="30" customHeight="1">
       <x:c r="A10" s="7" t="str">
         <x:v>I04</x:v>
       </x:c>
-      <x:c r="B10" s="12" t="str">
+      <x:c r="B10" s="7" t="str">
         <x:v>Resolution 256</x:v>
       </x:c>
       <x:c r="C10" s="7" t="str">
@@ -3374,18 +3963,24 @@
       <x:c r="S10" s="51" t="b">
         <x:v>0</x:v>
       </x:c>
-      <x:c r="T10" s="12" t="str">
+      <x:c r="T10" s="7" t="str">
         <x:v>normalized GPU input; tensor TTA + model + softmax/aggregation/T</x:v>
       </x:c>
       <x:c r="U10" s="7" t="str">
         <x:v>step3/I04/latency_batch1.json</x:v>
       </x:c>
-    </x:row>
-    <x:row r="11" ht="36" customHeight="1">
+      <x:c r="V10" s="7" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="W10" s="39" t="n">
+        <x:v>1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="11" ht="30" customHeight="1">
       <x:c r="A11" s="7" t="str">
         <x:v>I04</x:v>
       </x:c>
-      <x:c r="B11" s="12" t="str">
+      <x:c r="B11" s="7" t="str">
         <x:v>Resolution 256</x:v>
       </x:c>
       <x:c r="C11" s="7" t="str">
@@ -3439,18 +4034,24 @@
       <x:c r="S11" s="51" t="b">
         <x:v>0</x:v>
       </x:c>
-      <x:c r="T11" s="12" t="str">
+      <x:c r="T11" s="7" t="str">
         <x:v>normalized GPU input; tensor TTA + model + softmax/aggregation/T</x:v>
       </x:c>
       <x:c r="U11" s="7" t="str">
         <x:v>step3/I04/latency_batch32.json</x:v>
       </x:c>
-    </x:row>
-    <x:row r="12" ht="36" customHeight="1">
+      <x:c r="V11" s="7" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="W11" s="39" t="n">
+        <x:v>1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="12" ht="30" customHeight="1">
       <x:c r="A12" s="7" t="str">
         <x:v>I09</x:v>
       </x:c>
-      <x:c r="B12" s="12" t="str">
+      <x:c r="B12" s="7" t="str">
         <x:v>Resolution 288</x:v>
       </x:c>
       <x:c r="C12" s="7" t="str">
@@ -3504,18 +4105,24 @@
       <x:c r="S12" s="51" t="b">
         <x:v>0</x:v>
       </x:c>
-      <x:c r="T12" s="12" t="str">
+      <x:c r="T12" s="7" t="str">
         <x:v>normalized GPU input; tensor TTA + model + softmax/aggregation/T</x:v>
       </x:c>
       <x:c r="U12" s="7" t="str">
         <x:v>step3/I09/latency_batch1.json</x:v>
       </x:c>
-    </x:row>
-    <x:row r="13" ht="36" customHeight="1">
+      <x:c r="V12" s="7" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="W12" s="39" t="n">
+        <x:v>1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="13" ht="30" customHeight="1">
       <x:c r="A13" s="7" t="str">
         <x:v>I09</x:v>
       </x:c>
-      <x:c r="B13" s="12" t="str">
+      <x:c r="B13" s="7" t="str">
         <x:v>Resolution 288</x:v>
       </x:c>
       <x:c r="C13" s="7" t="str">
@@ -3569,18 +4176,24 @@
       <x:c r="S13" s="51" t="b">
         <x:v>0</x:v>
       </x:c>
-      <x:c r="T13" s="12" t="str">
+      <x:c r="T13" s="7" t="str">
         <x:v>normalized GPU input; tensor TTA + model + softmax/aggregation/T</x:v>
       </x:c>
       <x:c r="U13" s="7" t="str">
         <x:v>step3/I09/latency_batch32.json</x:v>
       </x:c>
-    </x:row>
-    <x:row r="14" ht="36" customHeight="1">
+      <x:c r="V13" s="7" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="W13" s="39" t="n">
+        <x:v>1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="14" ht="30" customHeight="1">
       <x:c r="A14" s="7" t="str">
         <x:v>I10</x:v>
       </x:c>
-      <x:c r="B14" s="12" t="str">
+      <x:c r="B14" s="7" t="str">
         <x:v>Resolution 320</x:v>
       </x:c>
       <x:c r="C14" s="7" t="str">
@@ -3634,18 +4247,24 @@
       <x:c r="S14" s="51" t="b">
         <x:v>0</x:v>
       </x:c>
-      <x:c r="T14" s="12" t="str">
+      <x:c r="T14" s="7" t="str">
         <x:v>normalized GPU input; tensor TTA + model + softmax/aggregation/T</x:v>
       </x:c>
       <x:c r="U14" s="7" t="str">
         <x:v>step3/I10/latency_batch1.json</x:v>
       </x:c>
-    </x:row>
-    <x:row r="15" ht="36" customHeight="1">
+      <x:c r="V14" s="7" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="W14" s="39" t="n">
+        <x:v>1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="15" ht="30" customHeight="1">
       <x:c r="A15" s="7" t="str">
         <x:v>I10</x:v>
       </x:c>
-      <x:c r="B15" s="12" t="str">
+      <x:c r="B15" s="7" t="str">
         <x:v>Resolution 320</x:v>
       </x:c>
       <x:c r="C15" s="7" t="str">
@@ -3699,18 +4318,24 @@
       <x:c r="S15" s="51" t="b">
         <x:v>0</x:v>
       </x:c>
-      <x:c r="T15" s="12" t="str">
+      <x:c r="T15" s="7" t="str">
         <x:v>normalized GPU input; tensor TTA + model + softmax/aggregation/T</x:v>
       </x:c>
       <x:c r="U15" s="7" t="str">
         <x:v>step3/I10/latency_batch32.json</x:v>
       </x:c>
-    </x:row>
-    <x:row r="16" ht="36" customHeight="1">
+      <x:c r="V15" s="7" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="W15" s="39" t="n">
+        <x:v>1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="16" ht="30" customHeight="1">
       <x:c r="A16" s="7" t="str">
         <x:v>I07</x:v>
       </x:c>
-      <x:c r="B16" s="12" t="str">
+      <x:c r="B16" s="7" t="str">
         <x:v>1 view + temperature</x:v>
       </x:c>
       <x:c r="C16" s="7" t="str">
@@ -3764,18 +4389,24 @@
       <x:c r="S16" s="51" t="b">
         <x:v>0</x:v>
       </x:c>
-      <x:c r="T16" s="12" t="str">
+      <x:c r="T16" s="7" t="str">
         <x:v>normalized GPU input; tensor TTA + model + softmax/aggregation/T</x:v>
       </x:c>
       <x:c r="U16" s="7" t="str">
         <x:v>step3/I07/latency_batch1.json</x:v>
       </x:c>
-    </x:row>
-    <x:row r="17" ht="36" customHeight="1">
+      <x:c r="V16" s="7" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="W16" s="39" t="n">
+        <x:v>0.6106658951607421</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="17" ht="30" customHeight="1">
       <x:c r="A17" s="7" t="str">
         <x:v>I07</x:v>
       </x:c>
-      <x:c r="B17" s="12" t="str">
+      <x:c r="B17" s="7" t="str">
         <x:v>1 view + temperature</x:v>
       </x:c>
       <x:c r="C17" s="7" t="str">
@@ -3829,18 +4460,24 @@
       <x:c r="S17" s="51" t="b">
         <x:v>0</x:v>
       </x:c>
-      <x:c r="T17" s="12" t="str">
+      <x:c r="T17" s="7" t="str">
         <x:v>normalized GPU input; tensor TTA + model + softmax/aggregation/T</x:v>
       </x:c>
       <x:c r="U17" s="7" t="str">
         <x:v>step3/I07/latency_batch32.json</x:v>
       </x:c>
-    </x:row>
-    <x:row r="18" ht="36" customHeight="1">
+      <x:c r="V17" s="7" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="W17" s="39" t="n">
+        <x:v>0.6106658951607421</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="18" ht="30" customHeight="1">
       <x:c r="A18" s="7" t="str">
         <x:v>I08</x:v>
       </x:c>
-      <x:c r="B18" s="12" t="str">
+      <x:c r="B18" s="7" t="str">
         <x:v>1 view AMP FP16</x:v>
       </x:c>
       <x:c r="C18" s="7" t="str">
@@ -3894,18 +4531,24 @@
       <x:c r="S18" s="51" t="b">
         <x:v>0</x:v>
       </x:c>
-      <x:c r="T18" s="12" t="str">
+      <x:c r="T18" s="7" t="str">
         <x:v>normalized GPU input; tensor TTA + model + softmax/aggregation/T</x:v>
       </x:c>
       <x:c r="U18" s="7" t="str">
         <x:v>step3/I08/latency_batch1.json</x:v>
       </x:c>
-    </x:row>
-    <x:row r="19" ht="36" customHeight="1">
+      <x:c r="V18" s="7" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="W18" s="39" t="n">
+        <x:v>1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="19" ht="30" customHeight="1">
       <x:c r="A19" s="7" t="str">
         <x:v>I08</x:v>
       </x:c>
-      <x:c r="B19" s="12" t="str">
+      <x:c r="B19" s="7" t="str">
         <x:v>1 view AMP FP16</x:v>
       </x:c>
       <x:c r="C19" s="7" t="str">
@@ -3959,37 +4602,446 @@
       <x:c r="S19" s="51" t="b">
         <x:v>0</x:v>
       </x:c>
-      <x:c r="T19" s="12" t="str">
+      <x:c r="T19" s="7" t="str">
         <x:v>normalized GPU input; tensor TTA + model + softmax/aggregation/T</x:v>
       </x:c>
       <x:c r="U19" s="7" t="str">
         <x:v>step3/I08/latency_batch32.json</x:v>
       </x:c>
-    </x:row>
-    <x:row r="22">
-      <x:c r="A22" t="str">
-        <x:v>Raw samples: step3/Ixx/latency_batch1/32.json; batch 1 và 32.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="23">
-      <x:c r="A23" t="str">
-        <x:v>10 warmup + 100 lần đo; synchronize trước/sau. Input sẵn trên GPU; gồm TTA/model/softmax/T.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="24">
-      <x:c r="A24" t="str">
-        <x:v>Không gồm decode/PIL/H2D/D2H. p95≤100 ms là ngưỡng pipeline GPU; chưa phải toàn bộ camera/robot.</x:v>
+      <x:c r="V19" s="7" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="W19" s="39" t="n">
+        <x:v>1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="20" ht="30" customHeight="1">
+      <x:c r="A20" s="7" t="str">
+        <x:v>F00</x:v>
+      </x:c>
+      <x:c r="B20" s="7" t="str">
+        <x:v>T00/I00</x:v>
+      </x:c>
+      <x:c r="C20" s="7" t="str">
+        <x:v>Tesla T4</x:v>
+      </x:c>
+      <x:c r="D20" s="7" t="str">
+        <x:v>fp32</x:v>
+      </x:c>
+      <x:c r="E20" s="7" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="F20" s="7" t="n">
+        <x:v>224</x:v>
+      </x:c>
+      <x:c r="G20" s="7" t="n">
+        <x:v>224</x:v>
+      </x:c>
+      <x:c r="H20" s="7" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="I20" s="51" t="b">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="J20" s="42" t="n">
+        <x:v>5.157577999966634</x:v>
+      </x:c>
+      <x:c r="K20" s="42" t="n">
+        <x:v>9.054779199891527</x:v>
+      </x:c>
+      <x:c r="L20" s="42" t="n">
+        <x:v>9.25613158003216</x:v>
+      </x:c>
+      <x:c r="M20" s="42" t="n">
+        <x:v>6.028892839997297</x:v>
+      </x:c>
+      <x:c r="N20" s="44" t="n">
+        <x:v>165.86793405345188</x:v>
+      </x:c>
+      <x:c r="O20" s="7" t="n">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="P20" s="7" t="n">
+        <x:v>100</x:v>
+      </x:c>
+      <x:c r="Q20" s="7" t="str">
+        <x:v>2.8.0+cu128</x:v>
+      </x:c>
+      <x:c r="R20" s="51" t="b">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="S20" s="51" t="b">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="T20" s="7" t="str">
+        <x:v>normalized GPU input; tensor TTA + model + softmax/aggregation/T</x:v>
+      </x:c>
+      <x:c r="U20" s="7" t="str">
+        <x:v>step4/F00/seed0/latency_batch1.json</x:v>
+      </x:c>
+      <x:c r="V20" s="7" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="W20" s="39" t="n">
+        <x:v>1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="21" ht="30" customHeight="1">
+      <x:c r="A21" s="7" t="str">
+        <x:v>F00</x:v>
+      </x:c>
+      <x:c r="B21" s="7" t="str">
+        <x:v>T00/I00</x:v>
+      </x:c>
+      <x:c r="C21" s="7" t="str">
+        <x:v>Tesla T4</x:v>
+      </x:c>
+      <x:c r="D21" s="7" t="str">
+        <x:v>fp32</x:v>
+      </x:c>
+      <x:c r="E21" s="7" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="F21" s="7" t="n">
+        <x:v>224</x:v>
+      </x:c>
+      <x:c r="G21" s="7" t="n">
+        <x:v>224</x:v>
+      </x:c>
+      <x:c r="H21" s="7" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="I21" s="51" t="b">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="J21" s="42" t="n">
+        <x:v>5.1001264998831175</x:v>
+      </x:c>
+      <x:c r="K21" s="42" t="n">
+        <x:v>7.994760450105787</x:v>
+      </x:c>
+      <x:c r="L21" s="42" t="n">
+        <x:v>8.134175540217258</x:v>
+      </x:c>
+      <x:c r="M21" s="42" t="n">
+        <x:v>5.7852694799794335</x:v>
+      </x:c>
+      <x:c r="N21" s="44" t="n">
+        <x:v>172.85279509634094</x:v>
+      </x:c>
+      <x:c r="O21" s="7" t="n">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="P21" s="7" t="n">
+        <x:v>100</x:v>
+      </x:c>
+      <x:c r="Q21" s="7" t="str">
+        <x:v>2.8.0+cu128</x:v>
+      </x:c>
+      <x:c r="R21" s="51" t="b">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="S21" s="51" t="b">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="T21" s="7" t="str">
+        <x:v>normalized GPU input; tensor TTA + model + softmax/aggregation/T</x:v>
+      </x:c>
+      <x:c r="U21" s="7" t="str">
+        <x:v>step4/F00/seed1/latency_batch1.json</x:v>
+      </x:c>
+      <x:c r="V21" s="7" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="W21" s="39" t="n">
+        <x:v>1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="22" ht="30" customHeight="1">
+      <x:c r="A22" s="7" t="str">
+        <x:v>F00</x:v>
+      </x:c>
+      <x:c r="B22" s="7" t="str">
+        <x:v>T00/I00</x:v>
+      </x:c>
+      <x:c r="C22" s="7" t="str">
+        <x:v>Tesla T4</x:v>
+      </x:c>
+      <x:c r="D22" s="7" t="str">
+        <x:v>fp32</x:v>
+      </x:c>
+      <x:c r="E22" s="7" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="F22" s="7" t="n">
+        <x:v>224</x:v>
+      </x:c>
+      <x:c r="G22" s="7" t="n">
+        <x:v>224</x:v>
+      </x:c>
+      <x:c r="H22" s="7" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="I22" s="51" t="b">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="J22" s="42" t="n">
+        <x:v>4.9598479997712275</x:v>
+      </x:c>
+      <x:c r="K22" s="42" t="n">
+        <x:v>6.590184450055857</x:v>
+      </x:c>
+      <x:c r="L22" s="42" t="n">
+        <x:v>7.931422750116327</x:v>
+      </x:c>
+      <x:c r="M22" s="42" t="n">
+        <x:v>5.142020369999045</x:v>
+      </x:c>
+      <x:c r="N22" s="44" t="n">
+        <x:v>194.47608683825297</x:v>
+      </x:c>
+      <x:c r="O22" s="7" t="n">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="P22" s="7" t="n">
+        <x:v>100</x:v>
+      </x:c>
+      <x:c r="Q22" s="7" t="str">
+        <x:v>2.8.0+cu128</x:v>
+      </x:c>
+      <x:c r="R22" s="51" t="b">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="S22" s="51" t="b">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="T22" s="7" t="str">
+        <x:v>normalized GPU input; tensor TTA + model + softmax/aggregation/T</x:v>
+      </x:c>
+      <x:c r="U22" s="7" t="str">
+        <x:v>step4/F00/seed2/latency_batch1.json</x:v>
+      </x:c>
+      <x:c r="V22" s="7" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="W22" s="39" t="n">
+        <x:v>1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="23" ht="30" customHeight="1">
+      <x:c r="A23" s="7" t="str">
+        <x:v>F01</x:v>
+      </x:c>
+      <x:c r="B23" s="7" t="str">
+        <x:v>T05/I09 + val-fit T</x:v>
+      </x:c>
+      <x:c r="C23" s="7" t="str">
+        <x:v>Tesla T4</x:v>
+      </x:c>
+      <x:c r="D23" s="7" t="str">
+        <x:v>fp32</x:v>
+      </x:c>
+      <x:c r="E23" s="7" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="F23" s="7" t="n">
+        <x:v>288</x:v>
+      </x:c>
+      <x:c r="G23" s="7" t="n">
+        <x:v>288</x:v>
+      </x:c>
+      <x:c r="H23" s="7" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="I23" s="51" t="b">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="J23" s="42" t="n">
+        <x:v>6.897031499875084</x:v>
+      </x:c>
+      <x:c r="K23" s="42" t="n">
+        <x:v>8.59377480007879</x:v>
+      </x:c>
+      <x:c r="L23" s="42" t="n">
+        <x:v>9.167404129789249</x:v>
+      </x:c>
+      <x:c r="M23" s="42" t="n">
+        <x:v>7.101249600004849</x:v>
+      </x:c>
+      <x:c r="N23" s="44" t="n">
+        <x:v>140.82028605209388</x:v>
+      </x:c>
+      <x:c r="O23" s="7" t="n">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="P23" s="7" t="n">
+        <x:v>100</x:v>
+      </x:c>
+      <x:c r="Q23" s="7" t="str">
+        <x:v>2.8.0+cu128</x:v>
+      </x:c>
+      <x:c r="R23" s="51" t="b">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="S23" s="51" t="b">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="T23" s="7" t="str">
+        <x:v>normalized GPU input; tensor TTA + model + softmax/aggregation/T</x:v>
+      </x:c>
+      <x:c r="U23" s="7" t="str">
+        <x:v>step4/F01/seed0/latency_batch1.json</x:v>
+      </x:c>
+      <x:c r="V23" s="7" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="W23" s="39" t="n">
+        <x:v>0.5893082440670381</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="24" ht="30" customHeight="1">
+      <x:c r="A24" s="7" t="str">
+        <x:v>F01</x:v>
+      </x:c>
+      <x:c r="B24" s="7" t="str">
+        <x:v>T05/I09 + val-fit T</x:v>
+      </x:c>
+      <x:c r="C24" s="7" t="str">
+        <x:v>Tesla T4</x:v>
+      </x:c>
+      <x:c r="D24" s="7" t="str">
+        <x:v>fp32</x:v>
+      </x:c>
+      <x:c r="E24" s="7" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="F24" s="7" t="n">
+        <x:v>288</x:v>
+      </x:c>
+      <x:c r="G24" s="7" t="n">
+        <x:v>288</x:v>
+      </x:c>
+      <x:c r="H24" s="7" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="I24" s="51" t="b">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="J24" s="42" t="n">
+        <x:v>6.682051500092712</x:v>
+      </x:c>
+      <x:c r="K24" s="42" t="n">
+        <x:v>6.966536250092759</x:v>
+      </x:c>
+      <x:c r="L24" s="42" t="n">
+        <x:v>8.879824999748964</x:v>
+      </x:c>
+      <x:c r="M24" s="42" t="n">
+        <x:v>6.73522807001973</x:v>
+      </x:c>
+      <x:c r="N24" s="44" t="n">
+        <x:v>148.47307167685423</x:v>
+      </x:c>
+      <x:c r="O24" s="7" t="n">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="P24" s="7" t="n">
+        <x:v>100</x:v>
+      </x:c>
+      <x:c r="Q24" s="7" t="str">
+        <x:v>2.8.0+cu128</x:v>
+      </x:c>
+      <x:c r="R24" s="51" t="b">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="S24" s="51" t="b">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="T24" s="7" t="str">
+        <x:v>normalized GPU input; tensor TTA + model + softmax/aggregation/T</x:v>
+      </x:c>
+      <x:c r="U24" s="7" t="str">
+        <x:v>step4/F01/seed1/latency_batch1.json</x:v>
+      </x:c>
+      <x:c r="V24" s="7" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="W24" s="39" t="n">
+        <x:v>0.616111856771697</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="25" ht="30" customHeight="1">
+      <x:c r="A25" s="7" t="str">
+        <x:v>F01</x:v>
+      </x:c>
+      <x:c r="B25" s="7" t="str">
+        <x:v>T05/I09 + val-fit T</x:v>
+      </x:c>
+      <x:c r="C25" s="7" t="str">
+        <x:v>Tesla T4</x:v>
+      </x:c>
+      <x:c r="D25" s="7" t="str">
+        <x:v>fp32</x:v>
+      </x:c>
+      <x:c r="E25" s="7" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="F25" s="7" t="n">
+        <x:v>288</x:v>
+      </x:c>
+      <x:c r="G25" s="7" t="n">
+        <x:v>288</x:v>
+      </x:c>
+      <x:c r="H25" s="7" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="I25" s="51" t="b">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="J25" s="42" t="n">
+        <x:v>6.69605250004679</x:v>
+      </x:c>
+      <x:c r="K25" s="42" t="n">
+        <x:v>8.79023894965485</x:v>
+      </x:c>
+      <x:c r="L25" s="42" t="n">
+        <x:v>9.171601190041656</x:v>
+      </x:c>
+      <x:c r="M25" s="42" t="n">
+        <x:v>6.859637240017946</x:v>
+      </x:c>
+      <x:c r="N25" s="44" t="n">
+        <x:v>145.7803036822664</x:v>
+      </x:c>
+      <x:c r="O25" s="7" t="n">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="P25" s="7" t="n">
+        <x:v>100</x:v>
+      </x:c>
+      <x:c r="Q25" s="7" t="str">
+        <x:v>2.8.0+cu128</x:v>
+      </x:c>
+      <x:c r="R25" s="51" t="b">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="S25" s="51" t="b">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="T25" s="7" t="str">
+        <x:v>normalized GPU input; tensor TTA + model + softmax/aggregation/T</x:v>
+      </x:c>
+      <x:c r="U25" s="7" t="str">
+        <x:v>step4/F01/seed2/latency_batch1.json</x:v>
+      </x:c>
+      <x:c r="V25" s="7" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="W25" s="39" t="n">
+        <x:v>0.6125404440631913</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
-  <x:mergeCells>
-    <x:mergeCell ref="A5:G5"/>
-    <x:mergeCell ref="A6:G6"/>
-    <x:mergeCell ref="A7:G7"/>
-    <x:mergeCell ref="A22:G22"/>
-    <x:mergeCell ref="A23:G23"/>
-    <x:mergeCell ref="A24:G24"/>
-  </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>
 </file>
@@ -4012,73 +5064,73 @@
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="44" customHeight="1">
-      <x:c r="A1" s="47" t="str">
+      <x:c r="A1" s="183" t="str">
         <x:v>Hạng</x:v>
       </x:c>
-      <x:c r="B1" s="47" t="str">
+      <x:c r="B1" s="183" t="str">
         <x:v>ID</x:v>
       </x:c>
-      <x:c r="C1" s="47" t="str">
+      <x:c r="C1" s="183" t="str">
         <x:v>Bước</x:v>
       </x:c>
-      <x:c r="D1" s="47" t="str">
+      <x:c r="D1" s="183" t="str">
         <x:v>Cấu hình</x:v>
       </x:c>
-      <x:c r="E1" s="47" t="str">
+      <x:c r="E1" s="183" t="str">
         <x:v>Macro-F1 val</x:v>
       </x:c>
-      <x:c r="F1" s="47" t="str">
+      <x:c r="F1" s="183" t="str">
         <x:v>Top-1 val</x:v>
       </x:c>
-      <x:c r="G1" s="47" t="str">
+      <x:c r="G1" s="183" t="str">
         <x:v>ECE val</x:v>
       </x:c>
-      <x:c r="H1" s="47" t="str">
+      <x:c r="H1" s="183" t="str">
         <x:v>p95 (ms)</x:v>
       </x:c>
-      <x:c r="I1" s="47" t="str">
+      <x:c r="I1" s="183" t="str">
         <x:v>Số seed</x:v>
       </x:c>
-      <x:c r="J1" s="47" t="str">
+      <x:c r="J1" s="183" t="str">
         <x:v>Điều kiện đo</x:v>
       </x:c>
-      <x:c r="K1" s="47" t="str">
+      <x:c r="K1" s="183" t="str">
         <x:v>Ghi chú</x:v>
       </x:c>
     </x:row>
     <x:row r="2" ht="35" customHeight="1">
-      <x:c r="A2" s="52" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="B2" s="52" t="str">
+      <x:c r="A2" s="184" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="B2" s="184" t="str">
         <x:v>I09</x:v>
       </x:c>
-      <x:c r="C2" s="52" t="str">
+      <x:c r="C2" s="184" t="str">
         <x:v>I</x:v>
       </x:c>
-      <x:c r="D2" s="53" t="str">
+      <x:c r="D2" s="185" t="str">
         <x:v>Resolution 288</x:v>
       </x:c>
-      <x:c r="E2" s="54" t="n">
+      <x:c r="E2" s="186" t="n">
         <x:v>0.9698380941836109</x:v>
       </x:c>
-      <x:c r="F2" s="54" t="n">
+      <x:c r="F2" s="186" t="n">
         <x:v>0.9771493858897458</x:v>
       </x:c>
-      <x:c r="G2" s="55" t="n">
+      <x:c r="G2" s="187" t="n">
         <x:v>0.1038055720536991</x:v>
       </x:c>
-      <x:c r="H2" s="56" t="n">
+      <x:c r="H2" s="188" t="n">
         <x:v>9.068122750227303</x:v>
       </x:c>
-      <x:c r="I2" s="52" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="J2" s="53" t="str">
-        <x:v>Lightning T4, 100 synchronized GPU pipeline timings</x:v>
-      </x:c>
-      <x:c r="K2" s="53" t="str">
-        <x:v>val only; no multi-seed test results</x:v>
+      <x:c r="I2" s="184" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="J2" s="185" t="str">
+        <x:v>Lightning T4 GPU pipeline</x:v>
+      </x:c>
+      <x:c r="K2" s="185" t="str">
+        <x:v>Một seed; T00=B03 và T05=I00 bỏ trùng</x:v>
       </x:c>
     </x:row>
     <x:row r="3" ht="35" customHeight="1">
@@ -4110,10 +5162,10 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="J3" s="12" t="str">
-        <x:v>Lightning T4, 100 synchronized GPU pipeline timings</x:v>
+        <x:v>Lightning T4 GPU pipeline</x:v>
       </x:c>
       <x:c r="K3" s="12" t="str">
-        <x:v>val only; no multi-seed test results</x:v>
+        <x:v>Một seed; T00=B03 và T05=I00 bỏ trùng</x:v>
       </x:c>
     </x:row>
     <x:row r="4" ht="35" customHeight="1">
@@ -4145,10 +5197,10 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="J4" s="12" t="str">
-        <x:v>Lightning T4, 100 synchronized GPU pipeline timings</x:v>
+        <x:v>Lightning T4 GPU pipeline</x:v>
       </x:c>
       <x:c r="K4" s="12" t="str">
-        <x:v>val only; no multi-seed test results</x:v>
+        <x:v>Một seed; T00=B03 và T05=I00 bỏ trùng</x:v>
       </x:c>
     </x:row>
     <x:row r="5" ht="35" customHeight="1">
@@ -4156,34 +5208,34 @@
         <x:v>4</x:v>
       </x:c>
       <x:c r="B5" s="7" t="str">
-        <x:v>I02</x:v>
+        <x:v>F01</x:v>
       </x:c>
       <x:c r="C5" s="7" t="str">
-        <x:v>I</x:v>
+        <x:v>F</x:v>
       </x:c>
       <x:c r="D5" s="12" t="str">
-        <x:v>5 crops / probability</x:v>
+        <x:v>ConvNeXt / T05 / I09 + val-fit T</x:v>
       </x:c>
       <x:c r="E5" s="40" t="n">
-        <x:v>0.9661639604452444</x:v>
+        <x:v>0.9677329532976656</x:v>
       </x:c>
       <x:c r="F5" s="40" t="n">
-        <x:v>0.9754355898314767</x:v>
+        <x:v>0.9755308007236027</x:v>
       </x:c>
       <x:c r="G5" s="41" t="n">
-        <x:v>0.09960301870037136</x:v>
+        <x:v>0.006190727482624035</x:v>
       </x:c>
       <x:c r="H5" s="42" t="n">
-        <x:v>42.252744699828774</x:v>
+        <x:v>8.79023894965485</x:v>
       </x:c>
       <x:c r="I5" s="7" t="n">
-        <x:v>1</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="J5" s="12" t="str">
-        <x:v>Lightning T4, 100 synchronized GPU pipeline timings</x:v>
+        <x:v>Lightning T4; maximum seed p95</x:v>
       </x:c>
       <x:c r="K5" s="12" t="str">
-        <x:v>val only; no multi-seed test results</x:v>
+        <x:v>Mean val 3 seed; công thức khóa trước test</x:v>
       </x:c>
     </x:row>
     <x:row r="6" ht="35" customHeight="1">
@@ -4191,34 +5243,34 @@
         <x:v>5</x:v>
       </x:c>
       <x:c r="B6" s="7" t="str">
-        <x:v>I03</x:v>
+        <x:v>I02</x:v>
       </x:c>
       <x:c r="C6" s="7" t="str">
         <x:v>I</x:v>
       </x:c>
       <x:c r="D6" s="12" t="str">
-        <x:v>Hflip TTA / logits</x:v>
+        <x:v>5 crops / probability</x:v>
       </x:c>
       <x:c r="E6" s="40" t="n">
-        <x:v>0.9642724549175057</x:v>
+        <x:v>0.9661639604452444</x:v>
       </x:c>
       <x:c r="F6" s="40" t="n">
-        <x:v>0.9734361610968295</x:v>
+        <x:v>0.9754355898314767</x:v>
       </x:c>
       <x:c r="G6" s="41" t="n">
-        <x:v>0.09718448681233922</x:v>
+        <x:v>0.09960301870037136</x:v>
       </x:c>
       <x:c r="H6" s="42" t="n">
-        <x:v>16.35914885002876</x:v>
+        <x:v>42.252744699828774</x:v>
       </x:c>
       <x:c r="I6" s="7" t="n">
         <x:v>1</x:v>
       </x:c>
       <x:c r="J6" s="12" t="str">
-        <x:v>Lightning T4, 100 synchronized GPU pipeline timings</x:v>
+        <x:v>Lightning T4 GPU pipeline</x:v>
       </x:c>
       <x:c r="K6" s="12" t="str">
-        <x:v>val only; no multi-seed test results</x:v>
+        <x:v>Một seed; T00=B03 và T05=I00 bỏ trùng</x:v>
       </x:c>
     </x:row>
     <x:row r="7" ht="35" customHeight="1">
@@ -4226,34 +5278,34 @@
         <x:v>6</x:v>
       </x:c>
       <x:c r="B7" s="7" t="str">
-        <x:v>I01</x:v>
+        <x:v>I03</x:v>
       </x:c>
       <x:c r="C7" s="7" t="str">
         <x:v>I</x:v>
       </x:c>
       <x:c r="D7" s="12" t="str">
-        <x:v>Hflip TTA / probability</x:v>
+        <x:v>Hflip TTA / logits</x:v>
       </x:c>
       <x:c r="E7" s="40" t="n">
-        <x:v>0.9642588606265972</x:v>
+        <x:v>0.9642724549175057</x:v>
       </x:c>
       <x:c r="F7" s="40" t="n">
         <x:v>0.9734361610968295</x:v>
       </x:c>
       <x:c r="G7" s="41" t="n">
-        <x:v>0.09708798446443855</x:v>
+        <x:v>0.09718448681233922</x:v>
       </x:c>
       <x:c r="H7" s="42" t="n">
-        <x:v>18.862193050108544</x:v>
+        <x:v>16.35914885002876</x:v>
       </x:c>
       <x:c r="I7" s="7" t="n">
         <x:v>1</x:v>
       </x:c>
       <x:c r="J7" s="12" t="str">
-        <x:v>Lightning T4, 100 synchronized GPU pipeline timings</x:v>
+        <x:v>Lightning T4 GPU pipeline</x:v>
       </x:c>
       <x:c r="K7" s="12" t="str">
-        <x:v>val only; no multi-seed test results</x:v>
+        <x:v>Một seed; T00=B03 và T05=I00 bỏ trùng</x:v>
       </x:c>
     </x:row>
     <x:row r="8" ht="35" customHeight="1">
@@ -4261,34 +5313,34 @@
         <x:v>7</x:v>
       </x:c>
       <x:c r="B8" s="7" t="str">
-        <x:v>I07</x:v>
+        <x:v>I01</x:v>
       </x:c>
       <x:c r="C8" s="7" t="str">
         <x:v>I</x:v>
       </x:c>
       <x:c r="D8" s="12" t="str">
-        <x:v>1 view + temperature</x:v>
+        <x:v>Hflip TTA / probability</x:v>
       </x:c>
       <x:c r="E8" s="40" t="n">
-        <x:v>0.9641032435221208</x:v>
+        <x:v>0.9642588606265972</x:v>
       </x:c>
       <x:c r="F8" s="40" t="n">
-        <x:v>0.9737217937732077</x:v>
+        <x:v>0.9734361610968295</x:v>
       </x:c>
       <x:c r="G8" s="41" t="n">
-        <x:v>0.004736394133104849</x:v>
+        <x:v>0.09708798446443855</x:v>
       </x:c>
       <x:c r="H8" s="42" t="n">
-        <x:v>7.490706349949504</x:v>
+        <x:v>18.862193050108544</x:v>
       </x:c>
       <x:c r="I8" s="7" t="n">
         <x:v>1</x:v>
       </x:c>
       <x:c r="J8" s="12" t="str">
-        <x:v>Lightning T4, 100 synchronized GPU pipeline timings</x:v>
+        <x:v>Lightning T4 GPU pipeline</x:v>
       </x:c>
       <x:c r="K8" s="12" t="str">
-        <x:v>val only; no multi-seed test results</x:v>
+        <x:v>Một seed; T00=B03 và T05=I00 bỏ trùng</x:v>
       </x:c>
     </x:row>
     <x:row r="9" ht="35" customHeight="1">
@@ -4296,13 +5348,13 @@
         <x:v>8</x:v>
       </x:c>
       <x:c r="B9" s="7" t="str">
-        <x:v>I08</x:v>
+        <x:v>I07</x:v>
       </x:c>
       <x:c r="C9" s="7" t="str">
         <x:v>I</x:v>
       </x:c>
       <x:c r="D9" s="12" t="str">
-        <x:v>1 view AMP FP16</x:v>
+        <x:v>1 view + temperature</x:v>
       </x:c>
       <x:c r="E9" s="40" t="n">
         <x:v>0.9641032435221208</x:v>
@@ -4311,19 +5363,19 @@
         <x:v>0.9737217937732077</x:v>
       </x:c>
       <x:c r="G9" s="41" t="n">
-        <x:v>0.09613235726078252</x:v>
+        <x:v>0.004736394133104849</x:v>
       </x:c>
       <x:c r="H9" s="42" t="n">
-        <x:v>10.559240600014162</x:v>
+        <x:v>7.490706349949504</x:v>
       </x:c>
       <x:c r="I9" s="7" t="n">
         <x:v>1</x:v>
       </x:c>
       <x:c r="J9" s="12" t="str">
-        <x:v>Lightning T4, 100 synchronized GPU pipeline timings</x:v>
+        <x:v>Lightning T4 GPU pipeline</x:v>
       </x:c>
       <x:c r="K9" s="12" t="str">
-        <x:v>val only; no multi-seed test results</x:v>
+        <x:v>Một seed; T00=B03 và T05=I00 bỏ trùng</x:v>
       </x:c>
     </x:row>
     <x:row r="10" ht="35" customHeight="1">
@@ -4331,13 +5383,13 @@
         <x:v>9</x:v>
       </x:c>
       <x:c r="B10" s="7" t="str">
-        <x:v>I00</x:v>
+        <x:v>I08</x:v>
       </x:c>
       <x:c r="C10" s="7" t="str">
         <x:v>I</x:v>
       </x:c>
       <x:c r="D10" s="12" t="str">
-        <x:v>1 view FP32</x:v>
+        <x:v>1 view AMP FP16</x:v>
       </x:c>
       <x:c r="E10" s="40" t="n">
         <x:v>0.9641032435221208</x:v>
@@ -4346,19 +5398,19 @@
         <x:v>0.9737217937732077</x:v>
       </x:c>
       <x:c r="G10" s="41" t="n">
-        <x:v>0.09615286034275924</x:v>
+        <x:v>0.09613235726078252</x:v>
       </x:c>
       <x:c r="H10" s="42" t="n">
-        <x:v>9.390229150073992</x:v>
+        <x:v>10.559240600014162</x:v>
       </x:c>
       <x:c r="I10" s="7" t="n">
         <x:v>1</x:v>
       </x:c>
       <x:c r="J10" s="12" t="str">
-        <x:v>Lightning T4, 100 synchronized GPU pipeline timings</x:v>
+        <x:v>Lightning T4 GPU pipeline</x:v>
       </x:c>
       <x:c r="K10" s="12" t="str">
-        <x:v>val only; no multi-seed test results</x:v>
+        <x:v>Một seed; T00=B03 và T05=I00 bỏ trùng</x:v>
       </x:c>
     </x:row>
     <x:row r="11" ht="35" customHeight="1">
@@ -4366,42 +5418,173 @@
         <x:v>10</x:v>
       </x:c>
       <x:c r="B11" s="7" t="str">
-        <x:v>T04</x:v>
+        <x:v>I00</x:v>
       </x:c>
       <x:c r="C11" s="7" t="str">
-        <x:v>T</x:v>
+        <x:v>I</x:v>
       </x:c>
       <x:c r="D11" s="12" t="str">
-        <x:v>CutMix alpha=1</x:v>
+        <x:v>1 view FP32</x:v>
       </x:c>
       <x:c r="E11" s="40" t="n">
-        <x:v>0.9630413373883078</x:v>
+        <x:v>0.9641032435221208</x:v>
       </x:c>
       <x:c r="F11" s="40" t="n">
-        <x:v>0.9720079977149386</x:v>
+        <x:v>0.9737217937732077</x:v>
       </x:c>
       <x:c r="G11" s="41" t="n">
-        <x:v>0.025046328791773743</x:v>
-      </x:c>
-      <x:c r="H11" s="42"/>
+        <x:v>0.09615286034275924</x:v>
+      </x:c>
+      <x:c r="H11" s="42" t="n">
+        <x:v>9.390229150073992</x:v>
+      </x:c>
       <x:c r="I11" s="7" t="n">
         <x:v>1</x:v>
       </x:c>
       <x:c r="J11" s="12" t="str">
-        <x:v>No comparable p95; screening timings only</x:v>
+        <x:v>Lightning T4 GPU pipeline</x:v>
       </x:c>
       <x:c r="K11" s="12" t="str">
-        <x:v>val only; no multi-seed test results</x:v>
+        <x:v>Một seed; T00=B03 và T05=I00 bỏ trùng</x:v>
       </x:c>
     </x:row>
     <x:row r="14">
       <x:c r="A14" t="str">
-        <x:v>Top 10 cấu hình val, một seed. T00=B03 và T05=I00 được bỏ trùng; p95 chỉ so trong Lightning Bước 3.</x:v>
-      </x:c>
+        <x:v>Top 10 theo val; B/T/I một seed, F mean ba seed. T00=B03 và T05=I00 bỏ trùng.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="15" ht="44" customHeight="1">
+      <x:c r="A15" s="183" t="str">
+        <x:v>Nhóm</x:v>
+      </x:c>
+      <x:c r="B15" s="183" t="str">
+        <x:v>F1 test mean</x:v>
+      </x:c>
+      <x:c r="C15" s="183" t="str">
+        <x:v>Std F1 test</x:v>
+      </x:c>
+      <x:c r="D15" s="183" t="str">
+        <x:v>Top-1 mean</x:v>
+      </x:c>
+      <x:c r="E15" s="183" t="str">
+        <x:v>Std top-1</x:v>
+      </x:c>
+      <x:c r="F15" s="183" t="str">
+        <x:v>ECE test</x:v>
+      </x:c>
+      <x:c r="G15" s="183" t="str">
+        <x:v>p95 cao nhất (ms)</x:v>
+      </x:c>
+      <x:c r="H15" s="183" t="str">
+        <x:v>Số seed</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="16" ht="30" customHeight="1">
+      <x:c r="A16" s="6" t="str">
+        <x:v>F00</x:v>
+      </x:c>
+      <x:c r="B16" s="92" t="n">
+        <x:f>'Final'!K8</x:f>
+        <x:v>0.9582598428151718</x:v>
+      </x:c>
+      <x:c r="C16" s="92" t="n">
+        <x:f>'Final'!L8</x:f>
+        <x:v>0.003775840468897587</x:v>
+      </x:c>
+      <x:c r="D16" s="92" t="n">
+        <x:f>'Final'!M8</x:f>
+        <x:v>0.9672084402623325</x:v>
+      </x:c>
+      <x:c r="E16" s="92" t="n">
+        <x:f>'Final'!N8</x:f>
+        <x:v>0.002534415288655702</x:v>
+      </x:c>
+      <x:c r="F16" s="93" t="n">
+        <x:f>'Final'!O8</x:f>
+        <x:v>0.010145725543199298</x:v>
+      </x:c>
+      <x:c r="G16" s="94" t="n">
+        <x:f>'Final'!S8</x:f>
+        <x:v>9.054779199891527</x:v>
+      </x:c>
+      <x:c r="H16" s="6" t="n">
+        <x:v>3</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="17" ht="30" customHeight="1">
+      <x:c r="A17" s="216" t="str">
+        <x:v>F01</x:v>
+      </x:c>
+      <x:c r="B17" s="217" t="n">
+        <x:f>'Final'!K9</x:f>
+        <x:v>0.9685776546225721</x:v>
+      </x:c>
+      <x:c r="C17" s="217" t="n">
+        <x:f>'Final'!L9</x:f>
+        <x:v>0.0027479284561232153</x:v>
+      </x:c>
+      <x:c r="D17" s="217" t="n">
+        <x:f>'Final'!M9</x:f>
+        <x:v>0.975762760193898</x:v>
+      </x:c>
+      <x:c r="E17" s="217" t="n">
+        <x:f>'Final'!N9</x:f>
+        <x:v>0.001869814235615052</x:v>
+      </x:c>
+      <x:c r="F17" s="218" t="n">
+        <x:f>'Final'!O9</x:f>
+        <x:v>0.0070808355774166325</x:v>
+      </x:c>
+      <x:c r="G17" s="219" t="n">
+        <x:f>'Final'!S9</x:f>
+        <x:v>8.79023894965485</x:v>
+      </x:c>
+      <x:c r="H17" s="216" t="n">
+        <x:v>3</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="19" ht="28" customHeight="1">
+      <x:c r="A19" s="6" t="str">
+        <x:v>Δ F1 test (pp)</x:v>
+      </x:c>
+      <x:c r="B19" s="6"/>
+      <x:c r="C19" s="6"/>
+      <x:c r="D19" s="178" t="n">
+        <x:f>100*(B17-B16)</x:f>
+        <x:v>1.0317811807400212</x:v>
+      </x:c>
+      <x:c r="E19" s="6"/>
+      <x:c r="F19" s="6" t="str">
+        <x:v>F01 đã chốt trên val trước test.</x:v>
+      </x:c>
+      <x:c r="G19" s="6"/>
+      <x:c r="H19" s="6"/>
+    </x:row>
+    <x:row r="20" ht="28" customHeight="1">
+      <x:c r="A20" s="6" t="str">
+        <x:v>Std lớn hơn (pp)</x:v>
+      </x:c>
+      <x:c r="B20" s="6"/>
+      <x:c r="C20" s="6"/>
+      <x:c r="D20" s="178" t="n">
+        <x:f>100*MAX(C16:C17)</x:f>
+        <x:v>0.3775840468897587</x:v>
+      </x:c>
+      <x:c r="E20" s="6"/>
+      <x:c r="F20" s="6" t="str">
+        <x:f>IF(D19&gt;D20,"Δ vượt std lớn hơn","Δ chưa vượt std lớn hơn")</x:f>
+        <x:v>Δ vượt std lớn hơn</x:v>
+      </x:c>
+      <x:c r="G20" s="6"/>
+      <x:c r="H20" s="6"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
     <x:mergeCell ref="A14:G14"/>
+    <x:mergeCell ref="A19:C19"/>
+    <x:mergeCell ref="A20:C20"/>
+    <x:mergeCell ref="F19:H19"/>
+    <x:mergeCell ref="F20:H20"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>
@@ -4413,9 +5596,9 @@
   <x:cols>
     <x:col min="1" max="1" width="8.130000114440918" hidden="0" customWidth="1"/>
     <x:col min="2" max="2" width="8.130000114440918" hidden="0" customWidth="1"/>
-    <x:col min="3" max="3" width="15" hidden="0" customWidth="1"/>
-    <x:col min="4" max="4" width="29.3799991607666" hidden="0" customWidth="1"/>
-    <x:col min="5" max="5" width="15" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="29.3799991607666" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="15" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="29.3799991607666" hidden="0" customWidth="1"/>
     <x:col min="6" max="6" width="15" hidden="0" customWidth="1"/>
     <x:col min="7" max="7" width="15" hidden="0" customWidth="1"/>
     <x:col min="8" max="8" width="15" hidden="0" customWidth="1"/>
@@ -4424,50 +5607,78 @@
     <x:col min="11" max="11" width="15" hidden="0" customWidth="1"/>
     <x:col min="12" max="12" width="15" hidden="0" customWidth="1"/>
     <x:col min="13" max="13" width="15" hidden="0" customWidth="1"/>
-    <x:col min="14" max="14" width="29.3799991607666" hidden="0" customWidth="1"/>
+    <x:col min="14" max="14" width="15" hidden="0" customWidth="1"/>
+    <x:col min="15" max="15" width="15" hidden="0" customWidth="1"/>
+    <x:col min="16" max="16" width="15" hidden="0" customWidth="1"/>
+    <x:col min="17" max="17" width="15" hidden="0" customWidth="1"/>
+    <x:col min="18" max="18" width="15" hidden="0" customWidth="1"/>
+    <x:col min="19" max="19" width="15" hidden="0" customWidth="1"/>
+    <x:col min="20" max="20" width="18.75" hidden="0" customWidth="1"/>
+    <x:col min="21" max="21" width="29.3799991607666" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="44" customHeight="1">
-      <x:c r="A1" s="47" t="str">
+      <x:c r="A1" s="183" t="str">
         <x:v>ID</x:v>
       </x:c>
-      <x:c r="B1" s="47" t="str">
+      <x:c r="B1" s="183" t="str">
         <x:v>Seed</x:v>
       </x:c>
-      <x:c r="C1" s="47" t="str">
+      <x:c r="C1" s="183" t="str">
+        <x:v>Backbone / tag</x:v>
+      </x:c>
+      <x:c r="D1" s="183" t="str">
         <x:v>Công thức</x:v>
       </x:c>
-      <x:c r="D1" s="47" t="str">
+      <x:c r="E1" s="183" t="str">
         <x:v>Suy luận</x:v>
       </x:c>
-      <x:c r="E1" s="47" t="str">
+      <x:c r="F1" s="183" t="str">
         <x:v>T val</x:v>
       </x:c>
-      <x:c r="F1" s="47" t="str">
+      <x:c r="G1" s="183" t="str">
         <x:v>Macro-F1 val</x:v>
       </x:c>
-      <x:c r="G1" s="47" t="str">
+      <x:c r="H1" s="183" t="str">
+        <x:v>Std F1 val</x:v>
+      </x:c>
+      <x:c r="I1" s="183" t="str">
         <x:v>Top-1 val</x:v>
       </x:c>
-      <x:c r="H1" s="47" t="str">
+      <x:c r="J1" s="183" t="str">
+        <x:v>Std top-1 val</x:v>
+      </x:c>
+      <x:c r="K1" s="183" t="str">
         <x:v>Macro-F1 test</x:v>
       </x:c>
-      <x:c r="I1" s="47" t="str">
+      <x:c r="L1" s="183" t="str">
+        <x:v>Std F1 test</x:v>
+      </x:c>
+      <x:c r="M1" s="183" t="str">
         <x:v>Top-1 test</x:v>
       </x:c>
-      <x:c r="J1" s="47" t="str">
+      <x:c r="N1" s="183" t="str">
+        <x:v>Std top-1 test</x:v>
+      </x:c>
+      <x:c r="O1" s="183" t="str">
         <x:v>ECE test</x:v>
       </x:c>
-      <x:c r="K1" s="47" t="str">
+      <x:c r="P1" s="183" t="str">
+        <x:v>Std ECE test</x:v>
+      </x:c>
+      <x:c r="Q1" s="183" t="str">
         <x:v>ECE test chưa T</x:v>
       </x:c>
-      <x:c r="L1" s="47" t="str">
+      <x:c r="R1" s="183" t="str">
+        <x:v>Std ECE chưa T</x:v>
+      </x:c>
+      <x:c r="S1" s="183" t="str">
         <x:v>p95 (ms)</x:v>
       </x:c>
-      <x:c r="M1" s="47" t="str">
+      <x:c r="T1" s="183" t="str">
         <x:v>Checkpoint epoch</x:v>
       </x:c>
-      <x:c r="N1" s="47" t="str">
+      <x:c r="U1" s="183" t="str">
         <x:v>Trạng thái</x:v>
       </x:c>
     </x:row>
@@ -4478,25 +5689,50 @@
       <x:c r="B2" s="7" t="n">
         <x:v>0</x:v>
       </x:c>
-      <x:c r="C2" s="7" t="str">
+      <x:c r="C2" s="12" t="str">
+        <x:v>convnext_tiny.fb_in1k</x:v>
+      </x:c>
+      <x:c r="D2" s="7" t="str">
         <x:v>T00</x:v>
       </x:c>
-      <x:c r="D2" s="12" t="str">
+      <x:c r="E2" s="12" t="str">
         <x:v>I00</x:v>
       </x:c>
-      <x:c r="E2" s="39" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="F2" s="40"/>
-      <x:c r="G2" s="40"/>
+      <x:c r="F2" s="39" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G2" s="40" t="n">
+        <x:v>0.9625123132868771</x:v>
+      </x:c>
       <x:c r="H2" s="40"/>
-      <x:c r="I2" s="40"/>
-      <x:c r="J2" s="41"/>
-      <x:c r="K2" s="41"/>
-      <x:c r="L2" s="42"/>
-      <x:c r="M2" s="7"/>
-      <x:c r="N2" s="12" t="str">
-        <x:v>Chưa train/test</x:v>
+      <x:c r="I2" s="40" t="n">
+        <x:v>0.9734361610968295</x:v>
+      </x:c>
+      <x:c r="J2" s="40"/>
+      <x:c r="K2" s="40" t="n">
+        <x:v>0.9571840317127569</x:v>
+      </x:c>
+      <x:c r="L2" s="40"/>
+      <x:c r="M2" s="40" t="n">
+        <x:v>0.9663530082691759</x:v>
+      </x:c>
+      <x:c r="N2" s="40"/>
+      <x:c r="O2" s="41" t="n">
+        <x:v>0.009163650048474442</x:v>
+      </x:c>
+      <x:c r="P2" s="41"/>
+      <x:c r="Q2" s="41" t="n">
+        <x:v>0.009163650048474442</x:v>
+      </x:c>
+      <x:c r="R2" s="41"/>
+      <x:c r="S2" s="42" t="n">
+        <x:v>9.054779199891527</x:v>
+      </x:c>
+      <x:c r="T2" s="7" t="n">
+        <x:v>9</x:v>
+      </x:c>
+      <x:c r="U2" s="12" t="str">
+        <x:v>Đủ kết quả</x:v>
       </x:c>
     </x:row>
     <x:row r="3" ht="35" customHeight="1">
@@ -4506,25 +5742,50 @@
       <x:c r="B3" s="7" t="n">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="C3" s="7" t="str">
+      <x:c r="C3" s="12" t="str">
+        <x:v>convnext_tiny.fb_in1k</x:v>
+      </x:c>
+      <x:c r="D3" s="7" t="str">
         <x:v>T00</x:v>
       </x:c>
-      <x:c r="D3" s="12" t="str">
+      <x:c r="E3" s="12" t="str">
         <x:v>I00</x:v>
       </x:c>
-      <x:c r="E3" s="39" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="F3" s="40"/>
-      <x:c r="G3" s="40"/>
+      <x:c r="F3" s="39" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G3" s="40" t="n">
+        <x:v>0.9602874885880599</x:v>
+      </x:c>
       <x:c r="H3" s="40"/>
-      <x:c r="I3" s="40"/>
-      <x:c r="J3" s="41"/>
-      <x:c r="K3" s="41"/>
-      <x:c r="L3" s="42"/>
-      <x:c r="M3" s="7"/>
-      <x:c r="N3" s="12" t="str">
-        <x:v>Chưa train/test</x:v>
+      <x:c r="I3" s="40" t="n">
+        <x:v>0.9700085689802913</x:v>
+      </x:c>
+      <x:c r="J3" s="40"/>
+      <x:c r="K3" s="40" t="n">
+        <x:v>0.9624568389775155</x:v>
+      </x:c>
+      <x:c r="L3" s="40"/>
+      <x:c r="M3" s="40" t="n">
+        <x:v>0.9700598802395209</x:v>
+      </x:c>
+      <x:c r="N3" s="40"/>
+      <x:c r="O3" s="41" t="n">
+        <x:v>0.009922613284858873</x:v>
+      </x:c>
+      <x:c r="P3" s="41"/>
+      <x:c r="Q3" s="41" t="n">
+        <x:v>0.009922613284858873</x:v>
+      </x:c>
+      <x:c r="R3" s="41"/>
+      <x:c r="S3" s="42" t="n">
+        <x:v>7.994760450105787</x:v>
+      </x:c>
+      <x:c r="T3" s="7" t="n">
+        <x:v>7</x:v>
+      </x:c>
+      <x:c r="U3" s="12" t="str">
+        <x:v>Đủ kết quả</x:v>
       </x:c>
     </x:row>
     <x:row r="4" ht="35" customHeight="1">
@@ -4534,25 +5795,50 @@
       <x:c r="B4" s="7" t="n">
         <x:v>2</x:v>
       </x:c>
-      <x:c r="C4" s="7" t="str">
+      <x:c r="C4" s="12" t="str">
+        <x:v>convnext_tiny.fb_in1k</x:v>
+      </x:c>
+      <x:c r="D4" s="7" t="str">
         <x:v>T00</x:v>
       </x:c>
-      <x:c r="D4" s="12" t="str">
+      <x:c r="E4" s="12" t="str">
         <x:v>I00</x:v>
       </x:c>
-      <x:c r="E4" s="39" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="F4" s="40"/>
-      <x:c r="G4" s="40"/>
+      <x:c r="F4" s="39" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G4" s="40" t="n">
+        <x:v>0.9643185836720115</x:v>
+      </x:c>
       <x:c r="H4" s="40"/>
-      <x:c r="I4" s="40"/>
-      <x:c r="J4" s="41"/>
-      <x:c r="K4" s="41"/>
-      <x:c r="L4" s="42"/>
-      <x:c r="M4" s="7"/>
-      <x:c r="N4" s="12" t="str">
-        <x:v>Chưa train/test</x:v>
+      <x:c r="I4" s="40" t="n">
+        <x:v>0.9728648957440731</x:v>
+      </x:c>
+      <x:c r="J4" s="40"/>
+      <x:c r="K4" s="40" t="n">
+        <x:v>0.9551386577552431</x:v>
+      </x:c>
+      <x:c r="L4" s="40"/>
+      <x:c r="M4" s="40" t="n">
+        <x:v>0.9652124322783006</x:v>
+      </x:c>
+      <x:c r="N4" s="40"/>
+      <x:c r="O4" s="41" t="n">
+        <x:v>0.01135091329626458</x:v>
+      </x:c>
+      <x:c r="P4" s="41"/>
+      <x:c r="Q4" s="41" t="n">
+        <x:v>0.01135091329626458</x:v>
+      </x:c>
+      <x:c r="R4" s="41"/>
+      <x:c r="S4" s="42" t="n">
+        <x:v>6.590184450055857</x:v>
+      </x:c>
+      <x:c r="T4" s="7" t="n">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="U4" s="12" t="str">
+        <x:v>Đủ kết quả</x:v>
       </x:c>
     </x:row>
     <x:row r="5" ht="35" customHeight="1">
@@ -4562,23 +5848,50 @@
       <x:c r="B5" s="7" t="n">
         <x:v>0</x:v>
       </x:c>
-      <x:c r="C5" s="7" t="str">
+      <x:c r="C5" s="12" t="str">
+        <x:v>convnext_tiny.fb_in1k</x:v>
+      </x:c>
+      <x:c r="D5" s="7" t="str">
         <x:v>T05</x:v>
       </x:c>
-      <x:c r="D5" s="12" t="str">
-        <x:v>I09 + own val-fit T</x:v>
-      </x:c>
-      <x:c r="E5" s="39"/>
-      <x:c r="F5" s="40"/>
-      <x:c r="G5" s="40"/>
+      <x:c r="E5" s="12" t="str">
+        <x:v>I09 + val-fit T</x:v>
+      </x:c>
+      <x:c r="F5" s="39" t="n">
+        <x:v>0.5893082440670381</x:v>
+      </x:c>
+      <x:c r="G5" s="40" t="n">
+        <x:v>0.970150583894313</x:v>
+      </x:c>
       <x:c r="H5" s="40"/>
-      <x:c r="I5" s="40"/>
-      <x:c r="J5" s="41"/>
-      <x:c r="K5" s="41"/>
-      <x:c r="L5" s="42"/>
-      <x:c r="M5" s="7"/>
-      <x:c r="N5" s="12" t="str">
-        <x:v>Chưa train/test</x:v>
+      <x:c r="I5" s="40" t="n">
+        <x:v>0.9774350185661239</x:v>
+      </x:c>
+      <x:c r="J5" s="40"/>
+      <x:c r="K5" s="40" t="n">
+        <x:v>0.9664794913707</x:v>
+      </x:c>
+      <x:c r="L5" s="40"/>
+      <x:c r="M5" s="40" t="n">
+        <x:v>0.9740518962075848</x:v>
+      </x:c>
+      <x:c r="N5" s="40"/>
+      <x:c r="O5" s="41" t="n">
+        <x:v>0.008380899435414948</x:v>
+      </x:c>
+      <x:c r="P5" s="41"/>
+      <x:c r="Q5" s="41" t="n">
+        <x:v>0.10358777279155981</x:v>
+      </x:c>
+      <x:c r="R5" s="41"/>
+      <x:c r="S5" s="42" t="n">
+        <x:v>8.59377480007879</x:v>
+      </x:c>
+      <x:c r="T5" s="7" t="n">
+        <x:v>9</x:v>
+      </x:c>
+      <x:c r="U5" s="12" t="str">
+        <x:v>Đủ kết quả</x:v>
       </x:c>
     </x:row>
     <x:row r="6" ht="35" customHeight="1">
@@ -4588,23 +5901,50 @@
       <x:c r="B6" s="7" t="n">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="C6" s="7" t="str">
+      <x:c r="C6" s="12" t="str">
+        <x:v>convnext_tiny.fb_in1k</x:v>
+      </x:c>
+      <x:c r="D6" s="7" t="str">
         <x:v>T05</x:v>
       </x:c>
-      <x:c r="D6" s="12" t="str">
-        <x:v>I09 + own val-fit T</x:v>
-      </x:c>
-      <x:c r="E6" s="39"/>
-      <x:c r="F6" s="40"/>
-      <x:c r="G6" s="40"/>
+      <x:c r="E6" s="12" t="str">
+        <x:v>I09 + val-fit T</x:v>
+      </x:c>
+      <x:c r="F6" s="39" t="n">
+        <x:v>0.616111856771697</x:v>
+      </x:c>
+      <x:c r="G6" s="40" t="n">
+        <x:v>0.9678452999693072</x:v>
+      </x:c>
       <x:c r="H6" s="40"/>
-      <x:c r="I6" s="40"/>
-      <x:c r="J6" s="41"/>
-      <x:c r="K6" s="41"/>
-      <x:c r="L6" s="42"/>
-      <x:c r="M6" s="7"/>
-      <x:c r="N6" s="12" t="str">
-        <x:v>Chưa train/test</x:v>
+      <x:c r="I6" s="40" t="n">
+        <x:v>0.9762924878606113</x:v>
+      </x:c>
+      <x:c r="J6" s="40"/>
+      <x:c r="K6" s="40" t="n">
+        <x:v>0.9716881420858778</x:v>
+      </x:c>
+      <x:c r="L6" s="40"/>
+      <x:c r="M6" s="40" t="n">
+        <x:v>0.9777587681779298</x:v>
+      </x:c>
+      <x:c r="N6" s="40"/>
+      <x:c r="O6" s="41" t="n">
+        <x:v>0.008441545648702673</x:v>
+      </x:c>
+      <x:c r="P6" s="41"/>
+      <x:c r="Q6" s="41" t="n">
+        <x:v>0.0934120020901055</x:v>
+      </x:c>
+      <x:c r="R6" s="41"/>
+      <x:c r="S6" s="42" t="n">
+        <x:v>6.966536250092759</x:v>
+      </x:c>
+      <x:c r="T6" s="7" t="n">
+        <x:v>9</x:v>
+      </x:c>
+      <x:c r="U6" s="12" t="str">
+        <x:v>Đủ kết quả</x:v>
       </x:c>
     </x:row>
     <x:row r="7" ht="35" customHeight="1">
@@ -4614,33 +5954,211 @@
       <x:c r="B7" s="7" t="n">
         <x:v>2</x:v>
       </x:c>
-      <x:c r="C7" s="7" t="str">
+      <x:c r="C7" s="12" t="str">
+        <x:v>convnext_tiny.fb_in1k</x:v>
+      </x:c>
+      <x:c r="D7" s="7" t="str">
         <x:v>T05</x:v>
       </x:c>
-      <x:c r="D7" s="12" t="str">
-        <x:v>I09 + own val-fit T</x:v>
-      </x:c>
-      <x:c r="E7" s="39"/>
-      <x:c r="F7" s="40"/>
-      <x:c r="G7" s="40"/>
+      <x:c r="E7" s="12" t="str">
+        <x:v>I09 + val-fit T</x:v>
+      </x:c>
+      <x:c r="F7" s="39" t="n">
+        <x:v>0.6125404440631913</x:v>
+      </x:c>
+      <x:c r="G7" s="40" t="n">
+        <x:v>0.9652029760293767</x:v>
+      </x:c>
       <x:c r="H7" s="40"/>
-      <x:c r="I7" s="40"/>
-      <x:c r="J7" s="41"/>
-      <x:c r="K7" s="41"/>
-      <x:c r="L7" s="42"/>
-      <x:c r="M7" s="7"/>
-      <x:c r="N7" s="12" t="str">
-        <x:v>Chưa train/test</x:v>
+      <x:c r="I7" s="40" t="n">
+        <x:v>0.9728648957440731</x:v>
+      </x:c>
+      <x:c r="J7" s="40"/>
+      <x:c r="K7" s="40" t="n">
+        <x:v>0.9675653304111385</x:v>
+      </x:c>
+      <x:c r="L7" s="40"/>
+      <x:c r="M7" s="40" t="n">
+        <x:v>0.9754776161961791</x:v>
+      </x:c>
+      <x:c r="N7" s="40"/>
+      <x:c r="O7" s="41" t="n">
+        <x:v>0.004420061648132276</x:v>
+      </x:c>
+      <x:c r="P7" s="41"/>
+      <x:c r="Q7" s="41" t="n">
+        <x:v>0.10288207345594523</x:v>
+      </x:c>
+      <x:c r="R7" s="41"/>
+      <x:c r="S7" s="42" t="n">
+        <x:v>8.79023894965485</x:v>
+      </x:c>
+      <x:c r="T7" s="7" t="n">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="U7" s="12" t="str">
+        <x:v>Đủ kết quả</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="8" ht="35" customHeight="1">
+      <x:c r="A8" s="195" t="str">
+        <x:v>F00</x:v>
+      </x:c>
+      <x:c r="B8" s="195" t="str">
+        <x:v>0/1/2</x:v>
+      </x:c>
+      <x:c r="C8" s="196" t="str">
+        <x:v>convnext_tiny.fb_in1k</x:v>
+      </x:c>
+      <x:c r="D8" s="195" t="str">
+        <x:v>T00</x:v>
+      </x:c>
+      <x:c r="E8" s="196" t="str">
+        <x:v>I00</x:v>
+      </x:c>
+      <x:c r="F8" s="197"/>
+      <x:c r="G8" s="198" t="n">
+        <x:f>AVERAGE(G2:G4)</x:f>
+        <x:v>0.9623727951823162</x:v>
+      </x:c>
+      <x:c r="H8" s="198" t="n">
+        <x:f>STDEV.S(G2:G4)</x:f>
+        <x:v>0.0020191658847380314</x:v>
+      </x:c>
+      <x:c r="I8" s="198" t="n">
+        <x:f>AVERAGE(I2:I4)</x:f>
+        <x:v>0.9721032086070647</x:v>
+      </x:c>
+      <x:c r="J8" s="198" t="n">
+        <x:f>STDEV.S(I2:I4)</x:f>
+        <x:v>0.0018363611846126046</x:v>
+      </x:c>
+      <x:c r="K8" s="198" t="n">
+        <x:f>AVERAGE(K2:K4)</x:f>
+        <x:v>0.9582598428151718</x:v>
+      </x:c>
+      <x:c r="L8" s="198" t="n">
+        <x:f>STDEV.S(K2:K4)</x:f>
+        <x:v>0.003775840468897587</x:v>
+      </x:c>
+      <x:c r="M8" s="198" t="n">
+        <x:f>AVERAGE(M2:M4)</x:f>
+        <x:v>0.9672084402623325</x:v>
+      </x:c>
+      <x:c r="N8" s="198" t="n">
+        <x:f>STDEV.S(M2:M4)</x:f>
+        <x:v>0.002534415288655702</x:v>
+      </x:c>
+      <x:c r="O8" s="199" t="n">
+        <x:f>AVERAGE(O2:O4)</x:f>
+        <x:v>0.010145725543199298</x:v>
+      </x:c>
+      <x:c r="P8" s="199" t="n">
+        <x:f>STDEV.S(O2:O4)</x:f>
+        <x:v>0.0011105694209051897</x:v>
+      </x:c>
+      <x:c r="Q8" s="199" t="n">
+        <x:f>AVERAGE(Q2:Q4)</x:f>
+        <x:v>0.010145725543199298</x:v>
+      </x:c>
+      <x:c r="R8" s="199" t="n">
+        <x:f>STDEV.S(Q2:Q4)</x:f>
+        <x:v>0.0011105694209051897</x:v>
+      </x:c>
+      <x:c r="S8" s="200" t="n">
+        <x:f>MAX(S2:S4)</x:f>
+        <x:v>9.054779199891527</x:v>
+      </x:c>
+      <x:c r="T8" s="195"/>
+      <x:c r="U8" s="196" t="str">
+        <x:v>Mean ± std; 3 seed</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="9" ht="35" customHeight="1">
+      <x:c r="A9" s="207" t="str">
+        <x:v>F01</x:v>
+      </x:c>
+      <x:c r="B9" s="207" t="str">
+        <x:v>0/1/2</x:v>
+      </x:c>
+      <x:c r="C9" s="208" t="str">
+        <x:v>convnext_tiny.fb_in1k</x:v>
+      </x:c>
+      <x:c r="D9" s="207" t="str">
+        <x:v>T05</x:v>
+      </x:c>
+      <x:c r="E9" s="208" t="str">
+        <x:v>I09 + val-fit T</x:v>
+      </x:c>
+      <x:c r="F9" s="209"/>
+      <x:c r="G9" s="210" t="n">
+        <x:f>AVERAGE(G5:G7)</x:f>
+        <x:v>0.9677329532976656</x:v>
+      </x:c>
+      <x:c r="H9" s="210" t="n">
+        <x:f>STDEV.S(G5:G7)</x:f>
+        <x:v>0.0024757165078551743</x:v>
+      </x:c>
+      <x:c r="I9" s="210" t="n">
+        <x:f>AVERAGE(I5:I7)</x:f>
+        <x:v>0.9755308007236027</x:v>
+      </x:c>
+      <x:c r="J9" s="210" t="n">
+        <x:f>STDEV.S(I5:I7)</x:f>
+        <x:v>0.0023783673230118674</x:v>
+      </x:c>
+      <x:c r="K9" s="210" t="n">
+        <x:f>AVERAGE(K5:K7)</x:f>
+        <x:v>0.9685776546225721</x:v>
+      </x:c>
+      <x:c r="L9" s="210" t="n">
+        <x:f>STDEV.S(K5:K7)</x:f>
+        <x:v>0.0027479284561232153</x:v>
+      </x:c>
+      <x:c r="M9" s="210" t="n">
+        <x:f>AVERAGE(M5:M7)</x:f>
+        <x:v>0.975762760193898</x:v>
+      </x:c>
+      <x:c r="N9" s="210" t="n">
+        <x:f>STDEV.S(M5:M7)</x:f>
+        <x:v>0.001869814235615052</x:v>
+      </x:c>
+      <x:c r="O9" s="211" t="n">
+        <x:f>AVERAGE(O5:O7)</x:f>
+        <x:v>0.0070808355774166325</x:v>
+      </x:c>
+      <x:c r="P9" s="211" t="n">
+        <x:f>STDEV.S(O5:O7)</x:f>
+        <x:v>0.0023044973243347496</x:v>
+      </x:c>
+      <x:c r="Q9" s="211" t="n">
+        <x:f>AVERAGE(Q5:Q7)</x:f>
+        <x:v>0.09996061611253686</x:v>
+      </x:c>
+      <x:c r="R9" s="211" t="n">
+        <x:f>STDEV.S(Q5:Q7)</x:f>
+        <x:v>0.005682232140555335</x:v>
+      </x:c>
+      <x:c r="S9" s="212" t="n">
+        <x:f>MAX(S5:S7)</x:f>
+        <x:v>8.79023894965485</x:v>
+      </x:c>
+      <x:c r="T9" s="207"/>
+      <x:c r="U9" s="208" t="str">
+        <x:v>Mean ± std; 3 seed</x:v>
       </x:c>
     </x:row>
     <x:row r="10">
-      <x:c r="A10" t="str">
-        <x:v>Chờ Bước 4: chưa có mean ± std, metric test hoặc dự đoán test. Không điền số val vào test.</x:v>
+      <x:c r="A10"/>
+    </x:row>
+    <x:row r="12">
+      <x:c r="A12" t="str">
+        <x:v>Kết quả chung kết tính từ dự đoán test; mọi lựa chọn đã khóa trên val trước test.</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
-    <x:mergeCell ref="A10:G10"/>
+    <x:mergeCell ref="A12:G12"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>
@@ -4656,30 +6174,38 @@
     <x:col min="4" max="4" width="15" hidden="0" customWidth="1"/>
     <x:col min="5" max="5" width="15" hidden="0" customWidth="1"/>
     <x:col min="6" max="6" width="15" hidden="0" customWidth="1"/>
-    <x:col min="7" max="7" width="29.3799991607666" hidden="0" customWidth="1"/>
+    <x:col min="7" max="7" width="15" hidden="0" customWidth="1"/>
+    <x:col min="8" max="8" width="15" hidden="0" customWidth="1"/>
+    <x:col min="9" max="9" width="15" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="44" customHeight="1">
-      <x:c r="A1" s="47" t="str">
+      <x:c r="A1" s="183" t="str">
         <x:v>ID</x:v>
       </x:c>
-      <x:c r="B1" s="47" t="str">
+      <x:c r="B1" s="183" t="str">
         <x:v>Lớp</x:v>
       </x:c>
-      <x:c r="C1" s="47" t="str">
+      <x:c r="C1" s="183" t="str">
+        <x:v>Precision mean</x:v>
+      </x:c>
+      <x:c r="D1" s="183" t="str">
+        <x:v>Std precision</x:v>
+      </x:c>
+      <x:c r="E1" s="183" t="str">
+        <x:v>Recall mean</x:v>
+      </x:c>
+      <x:c r="F1" s="183" t="str">
+        <x:v>Std recall</x:v>
+      </x:c>
+      <x:c r="G1" s="183" t="str">
+        <x:v>F1 mean</x:v>
+      </x:c>
+      <x:c r="H1" s="183" t="str">
+        <x:v>Std F1</x:v>
+      </x:c>
+      <x:c r="I1" s="183" t="str">
         <x:v>Số ảnh test/seed</x:v>
-      </x:c>
-      <x:c r="D1" s="47" t="str">
-        <x:v>Precision test</x:v>
-      </x:c>
-      <x:c r="E1" s="47" t="str">
-        <x:v>Recall test</x:v>
-      </x:c>
-      <x:c r="F1" s="47" t="str">
-        <x:v>F1 test</x:v>
-      </x:c>
-      <x:c r="G1" s="47" t="str">
-        <x:v>Trạng thái</x:v>
       </x:c>
     </x:row>
     <x:row r="2" ht="35" customHeight="1">
@@ -4687,16 +6213,28 @@
         <x:v>F00</x:v>
       </x:c>
       <x:c r="B2" s="12" t="str">
-        <x:v>Chinee Apple</x:v>
-      </x:c>
-      <x:c r="C2" s="7" t="n">
+        <x:v>Chinee apple</x:v>
+      </x:c>
+      <x:c r="C2" s="40" t="n">
+        <x:v>0.9533771498405316</x:v>
+      </x:c>
+      <x:c r="D2" s="40" t="n">
+        <x:v>0.0077698903010514</x:v>
+      </x:c>
+      <x:c r="E2" s="40" t="n">
+        <x:v>0.9041297935103244</x:v>
+      </x:c>
+      <x:c r="F2" s="40" t="n">
+        <x:v>0.0199524325346145</x:v>
+      </x:c>
+      <x:c r="G2" s="40" t="n">
+        <x:v>0.9280194626790308</x:v>
+      </x:c>
+      <x:c r="H2" s="40" t="n">
+        <x:v>0.0113530477952647</x:v>
+      </x:c>
+      <x:c r="I2" s="7" t="n">
         <x:v>226</x:v>
-      </x:c>
-      <x:c r="D2" s="40"/>
-      <x:c r="E2" s="40"/>
-      <x:c r="F2" s="40"/>
-      <x:c r="G2" s="12" t="str">
-        <x:v>Chưa có dự đoán test</x:v>
       </x:c>
     </x:row>
     <x:row r="3" ht="35" customHeight="1">
@@ -4706,14 +6244,26 @@
       <x:c r="B3" s="12" t="str">
         <x:v>Lantana</x:v>
       </x:c>
-      <x:c r="C3" s="7" t="n">
+      <x:c r="C3" s="40" t="n">
+        <x:v>0.9570938335543908</x:v>
+      </x:c>
+      <x:c r="D3" s="40" t="n">
+        <x:v>0.0135330992381525</x:v>
+      </x:c>
+      <x:c r="E3" s="40" t="n">
+        <x:v>0.971830985915493</x:v>
+      </x:c>
+      <x:c r="F3" s="40" t="n">
+        <x:v>0.0124213676575802</x:v>
+      </x:c>
+      <x:c r="G3" s="40" t="n">
+        <x:v>0.9642934056941034</x:v>
+      </x:c>
+      <x:c r="H3" s="40" t="n">
+        <x:v>0.0024992831246765</x:v>
+      </x:c>
+      <x:c r="I3" s="7" t="n">
         <x:v>213</x:v>
-      </x:c>
-      <x:c r="D3" s="40"/>
-      <x:c r="E3" s="40"/>
-      <x:c r="F3" s="40"/>
-      <x:c r="G3" s="12" t="str">
-        <x:v>Chưa có dự đoán test</x:v>
       </x:c>
     </x:row>
     <x:row r="4" ht="35" customHeight="1">
@@ -4723,14 +6273,26 @@
       <x:c r="B4" s="12" t="str">
         <x:v>Parkinsonia</x:v>
       </x:c>
-      <x:c r="C4" s="7" t="n">
+      <x:c r="C4" s="40" t="n">
+        <x:v>0.9684475047092258</x:v>
+      </x:c>
+      <x:c r="D4" s="40" t="n">
+        <x:v>0.0069609770859486</x:v>
+      </x:c>
+      <x:c r="E4" s="40" t="n">
+        <x:v>0.9871175523349436</x:v>
+      </x:c>
+      <x:c r="F4" s="40" t="n">
+        <x:v>0.0027891317352155</x:v>
+      </x:c>
+      <x:c r="G4" s="40" t="n">
+        <x:v>0.9776787539945434</x:v>
+      </x:c>
+      <x:c r="H4" s="40" t="n">
+        <x:v>0.0026770374538299</x:v>
+      </x:c>
+      <x:c r="I4" s="7" t="n">
         <x:v>207</x:v>
-      </x:c>
-      <x:c r="D4" s="40"/>
-      <x:c r="E4" s="40"/>
-      <x:c r="F4" s="40"/>
-      <x:c r="G4" s="12" t="str">
-        <x:v>Chưa có dự đoán test</x:v>
       </x:c>
     </x:row>
     <x:row r="5" ht="35" customHeight="1">
@@ -4740,14 +6302,26 @@
       <x:c r="B5" s="12" t="str">
         <x:v>Parthenium</x:v>
       </x:c>
-      <x:c r="C5" s="7" t="n">
+      <x:c r="C5" s="40" t="n">
+        <x:v>0.9931348743848744</x:v>
+      </x:c>
+      <x:c r="D5" s="40" t="n">
+        <x:v>0.0030759701243842</x:v>
+      </x:c>
+      <x:c r="E5" s="40" t="n">
+        <x:v>0.9447154471544716</x:v>
+      </x:c>
+      <x:c r="F5" s="40" t="n">
+        <x:v>0.0171311443135816</x:v>
+      </x:c>
+      <x:c r="G5" s="40" t="n">
+        <x:v>0.9682821117021166</x:v>
+      </x:c>
+      <x:c r="H5" s="40" t="n">
+        <x:v>0.0103517909239521</x:v>
+      </x:c>
+      <x:c r="I5" s="7" t="n">
         <x:v>205</x:v>
-      </x:c>
-      <x:c r="D5" s="40"/>
-      <x:c r="E5" s="40"/>
-      <x:c r="F5" s="40"/>
-      <x:c r="G5" s="12" t="str">
-        <x:v>Chưa có dự đoán test</x:v>
       </x:c>
     </x:row>
     <x:row r="6" ht="35" customHeight="1">
@@ -4755,16 +6329,28 @@
         <x:v>F00</x:v>
       </x:c>
       <x:c r="B6" s="12" t="str">
-        <x:v>Prickly Acacia</x:v>
-      </x:c>
-      <x:c r="C6" s="7" t="n">
+        <x:v>Prickly acacia</x:v>
+      </x:c>
+      <x:c r="C6" s="40" t="n">
+        <x:v>0.9234774170543512</x:v>
+      </x:c>
+      <x:c r="D6" s="40" t="n">
+        <x:v>0.0210256576899015</x:v>
+      </x:c>
+      <x:c r="E6" s="40" t="n">
+        <x:v>0.9593114241001564</x:v>
+      </x:c>
+      <x:c r="F6" s="40" t="n">
+        <x:v>0.0027105646440827</x:v>
+      </x:c>
+      <x:c r="G6" s="40" t="n">
+        <x:v>0.9409885012743584</x:v>
+      </x:c>
+      <x:c r="H6" s="40" t="n">
+        <x:v>0.0120766763301061</x:v>
+      </x:c>
+      <x:c r="I6" s="7" t="n">
         <x:v>213</x:v>
-      </x:c>
-      <x:c r="D6" s="40"/>
-      <x:c r="E6" s="40"/>
-      <x:c r="F6" s="40"/>
-      <x:c r="G6" s="12" t="str">
-        <x:v>Chưa có dự đoán test</x:v>
       </x:c>
     </x:row>
     <x:row r="7" ht="35" customHeight="1">
@@ -4772,16 +6358,28 @@
         <x:v>F00</x:v>
       </x:c>
       <x:c r="B7" s="12" t="str">
-        <x:v>Rubber Vine</x:v>
-      </x:c>
-      <x:c r="C7" s="7" t="n">
+        <x:v>Rubber vine</x:v>
+      </x:c>
+      <x:c r="C7" s="40" t="n">
+        <x:v>0.9605305536848886</x:v>
+      </x:c>
+      <x:c r="D7" s="40" t="n">
+        <x:v>0.0123118176462888</x:v>
+      </x:c>
+      <x:c r="E7" s="40" t="n">
+        <x:v>0.9587458745874587</x:v>
+      </x:c>
+      <x:c r="F7" s="40" t="n">
+        <x:v>0.0114326785978143</x:v>
+      </x:c>
+      <x:c r="G7" s="40" t="n">
+        <x:v>0.9595403620702528</x:v>
+      </x:c>
+      <x:c r="H7" s="40" t="n">
+        <x:v>0.0012011554751293</x:v>
+      </x:c>
+      <x:c r="I7" s="7" t="n">
         <x:v>202</x:v>
-      </x:c>
-      <x:c r="D7" s="40"/>
-      <x:c r="E7" s="40"/>
-      <x:c r="F7" s="40"/>
-      <x:c r="G7" s="12" t="str">
-        <x:v>Chưa có dự đoán test</x:v>
       </x:c>
     </x:row>
     <x:row r="8" ht="35" customHeight="1">
@@ -4789,16 +6387,28 @@
         <x:v>F00</x:v>
       </x:c>
       <x:c r="B8" s="12" t="str">
-        <x:v>Siam Weed</x:v>
-      </x:c>
-      <x:c r="C8" s="7" t="n">
+        <x:v>Siam weed</x:v>
+      </x:c>
+      <x:c r="C8" s="40" t="n">
+        <x:v>0.9594589719886476</x:v>
+      </x:c>
+      <x:c r="D8" s="40" t="n">
+        <x:v>0.0078032970939469</x:v>
+      </x:c>
+      <x:c r="E8" s="40" t="n">
+        <x:v>0.9906976744186048</x:v>
+      </x:c>
+      <x:c r="F8" s="40" t="n">
+        <x:v>0.0093023255813953</x:v>
+      </x:c>
+      <x:c r="G8" s="40" t="n">
+        <x:v>0.9748248124030252</x:v>
+      </x:c>
+      <x:c r="H8" s="40" t="n">
+        <x:v>0.0082609281778264</x:v>
+      </x:c>
+      <x:c r="I8" s="7" t="n">
         <x:v>215</x:v>
-      </x:c>
-      <x:c r="D8" s="40"/>
-      <x:c r="E8" s="40"/>
-      <x:c r="F8" s="40"/>
-      <x:c r="G8" s="12" t="str">
-        <x:v>Chưa có dự đoán test</x:v>
       </x:c>
     </x:row>
     <x:row r="9" ht="35" customHeight="1">
@@ -4806,16 +6416,28 @@
         <x:v>F00</x:v>
       </x:c>
       <x:c r="B9" s="12" t="str">
-        <x:v>Snake Weed</x:v>
-      </x:c>
-      <x:c r="C9" s="7" t="n">
+        <x:v>Snake weed</x:v>
+      </x:c>
+      <x:c r="C9" s="40" t="n">
+        <x:v>0.9463247863247864</x:v>
+      </x:c>
+      <x:c r="D9" s="40" t="n">
+        <x:v>0.0120419585683813</x:v>
+      </x:c>
+      <x:c r="E9" s="40" t="n">
+        <x:v>0.9199346405228758</x:v>
+      </x:c>
+      <x:c r="F9" s="40" t="n">
+        <x:v>0.005660296756761</x:v>
+      </x:c>
+      <x:c r="G9" s="40" t="n">
+        <x:v>0.9329098323366172</x:v>
+      </x:c>
+      <x:c r="H9" s="40" t="n">
+        <x:v>0.0062649434334657</x:v>
+      </x:c>
+      <x:c r="I9" s="7" t="n">
         <x:v>204</x:v>
-      </x:c>
-      <x:c r="D9" s="40"/>
-      <x:c r="E9" s="40"/>
-      <x:c r="F9" s="40"/>
-      <x:c r="G9" s="12" t="str">
-        <x:v>Chưa có dự đoán test</x:v>
       </x:c>
     </x:row>
     <x:row r="10" ht="35" customHeight="1">
@@ -4823,16 +6445,28 @@
         <x:v>F00</x:v>
       </x:c>
       <x:c r="B10" s="12" t="str">
-        <x:v>Negatives</x:v>
-      </x:c>
-      <x:c r="C10" s="7" t="n">
+        <x:v>Negative</x:v>
+      </x:c>
+      <x:c r="C10" s="40" t="n">
+        <x:v>0.9764837898344766</x:v>
+      </x:c>
+      <x:c r="D10" s="40" t="n">
+        <x:v>0.0037777462981321</x:v>
+      </x:c>
+      <x:c r="E10" s="40" t="n">
+        <x:v>0.9791437980241492</x:v>
+      </x:c>
+      <x:c r="F10" s="40" t="n">
+        <x:v>0.0043563413464291</x:v>
+      </x:c>
+      <x:c r="G10" s="40" t="n">
+        <x:v>0.977801343182498</x:v>
+      </x:c>
+      <x:c r="H10" s="40" t="n">
+        <x:v>0.0010086578698155</x:v>
+      </x:c>
+      <x:c r="I10" s="7" t="n">
         <x:v>1822</x:v>
-      </x:c>
-      <x:c r="D10" s="40"/>
-      <x:c r="E10" s="40"/>
-      <x:c r="F10" s="40"/>
-      <x:c r="G10" s="12" t="str">
-        <x:v>Chưa có dự đoán test</x:v>
       </x:c>
     </x:row>
     <x:row r="11" ht="35" customHeight="1">
@@ -4840,16 +6474,28 @@
         <x:v>F01</x:v>
       </x:c>
       <x:c r="B11" s="12" t="str">
-        <x:v>Chinee Apple</x:v>
-      </x:c>
-      <x:c r="C11" s="7" t="n">
+        <x:v>Chinee apple</x:v>
+      </x:c>
+      <x:c r="C11" s="40" t="n">
+        <x:v>0.9509418913166962</x:v>
+      </x:c>
+      <x:c r="D11" s="40" t="n">
+        <x:v>0.0085334325222566</x:v>
+      </x:c>
+      <x:c r="E11" s="40" t="n">
+        <x:v>0.9424778761061946</x:v>
+      </x:c>
+      <x:c r="F11" s="40" t="n">
+        <x:v>0.0076639416264109</x:v>
+      </x:c>
+      <x:c r="G11" s="40" t="n">
+        <x:v>0.946668777539957</x:v>
+      </x:c>
+      <x:c r="H11" s="40" t="n">
+        <x:v>0.005828482448994</x:v>
+      </x:c>
+      <x:c r="I11" s="7" t="n">
         <x:v>226</x:v>
-      </x:c>
-      <x:c r="D11" s="40"/>
-      <x:c r="E11" s="40"/>
-      <x:c r="F11" s="40"/>
-      <x:c r="G11" s="12" t="str">
-        <x:v>Chưa có dự đoán test</x:v>
       </x:c>
     </x:row>
     <x:row r="12" ht="35" customHeight="1">
@@ -4859,14 +6505,26 @@
       <x:c r="B12" s="12" t="str">
         <x:v>Lantana</x:v>
       </x:c>
-      <x:c r="C12" s="7" t="n">
+      <x:c r="C12" s="40" t="n">
+        <x:v>0.9840178458878588</x:v>
+      </x:c>
+      <x:c r="D12" s="40" t="n">
+        <x:v>0.0098212991373658</x:v>
+      </x:c>
+      <x:c r="E12" s="40" t="n">
+        <x:v>0.9561815336463224</x:v>
+      </x:c>
+      <x:c r="F12" s="40" t="n">
+        <x:v>0.0097730798097001</x:v>
+      </x:c>
+      <x:c r="G12" s="40" t="n">
+        <x:v>0.9698395420093532</x:v>
+      </x:c>
+      <x:c r="H12" s="40" t="n">
+        <x:v>0.0027612334402595</x:v>
+      </x:c>
+      <x:c r="I12" s="7" t="n">
         <x:v>213</x:v>
-      </x:c>
-      <x:c r="D12" s="40"/>
-      <x:c r="E12" s="40"/>
-      <x:c r="F12" s="40"/>
-      <x:c r="G12" s="12" t="str">
-        <x:v>Chưa có dự đoán test</x:v>
       </x:c>
     </x:row>
     <x:row r="13" ht="35" customHeight="1">
@@ -4876,14 +6534,26 @@
       <x:c r="B13" s="12" t="str">
         <x:v>Parkinsonia</x:v>
       </x:c>
-      <x:c r="C13" s="7" t="n">
+      <x:c r="C13" s="40" t="n">
+        <x:v>0.9686789718385296</x:v>
+      </x:c>
+      <x:c r="D13" s="40" t="n">
+        <x:v>0.013761473301017</x:v>
+      </x:c>
+      <x:c r="E13" s="40" t="n">
+        <x:v>0.9903381642512076</x:v>
+      </x:c>
+      <x:c r="F13" s="40" t="n">
+        <x:v>0.0048309178743961</x:v>
+      </x:c>
+      <x:c r="G13" s="40" t="n">
+        <x:v>0.979329682002411</x:v>
+      </x:c>
+      <x:c r="H13" s="40" t="n">
+        <x:v>0.00475727167116</x:v>
+      </x:c>
+      <x:c r="I13" s="7" t="n">
         <x:v>207</x:v>
-      </x:c>
-      <x:c r="D13" s="40"/>
-      <x:c r="E13" s="40"/>
-      <x:c r="F13" s="40"/>
-      <x:c r="G13" s="12" t="str">
-        <x:v>Chưa có dự đoán test</x:v>
       </x:c>
     </x:row>
     <x:row r="14" ht="35" customHeight="1">
@@ -4893,14 +6563,26 @@
       <x:c r="B14" s="12" t="str">
         <x:v>Parthenium</x:v>
       </x:c>
-      <x:c r="C14" s="7" t="n">
+      <x:c r="C14" s="40" t="n">
+        <x:v>0.9899412043381892</x:v>
+      </x:c>
+      <x:c r="D14" s="40" t="n">
+        <x:v>0.0050378210949719</x:v>
+      </x:c>
+      <x:c r="E14" s="40" t="n">
+        <x:v>0.9609756097560976</x:v>
+      </x:c>
+      <x:c r="F14" s="40" t="n">
+        <x:v>0.0084490283296042</x:v>
+      </x:c>
+      <x:c r="G14" s="40" t="n">
+        <x:v>0.9752392645752948</x:v>
+      </x:c>
+      <x:c r="H14" s="40" t="n">
+        <x:v>0.0065860435757441</x:v>
+      </x:c>
+      <x:c r="I14" s="7" t="n">
         <x:v>205</x:v>
-      </x:c>
-      <x:c r="D14" s="40"/>
-      <x:c r="E14" s="40"/>
-      <x:c r="F14" s="40"/>
-      <x:c r="G14" s="12" t="str">
-        <x:v>Chưa có dự đoán test</x:v>
       </x:c>
     </x:row>
     <x:row r="15" ht="35" customHeight="1">
@@ -4908,16 +6590,28 @@
         <x:v>F01</x:v>
       </x:c>
       <x:c r="B15" s="12" t="str">
-        <x:v>Prickly Acacia</x:v>
-      </x:c>
-      <x:c r="C15" s="7" t="n">
+        <x:v>Prickly acacia</x:v>
+      </x:c>
+      <x:c r="C15" s="40" t="n">
+        <x:v>0.958138544222742</x:v>
+      </x:c>
+      <x:c r="D15" s="40" t="n">
+        <x:v>0.0161770482645161</x:v>
+      </x:c>
+      <x:c r="E15" s="40" t="n">
+        <x:v>0.9624413145539906</x:v>
+      </x:c>
+      <x:c r="F15" s="40" t="n">
+        <x:v>0.0046948356807511</x:v>
+      </x:c>
+      <x:c r="G15" s="40" t="n">
+        <x:v>0.9602290418927776</x:v>
+      </x:c>
+      <x:c r="H15" s="40" t="n">
+        <x:v>0.0078299450877083</x:v>
+      </x:c>
+      <x:c r="I15" s="7" t="n">
         <x:v>213</x:v>
-      </x:c>
-      <x:c r="D15" s="40"/>
-      <x:c r="E15" s="40"/>
-      <x:c r="F15" s="40"/>
-      <x:c r="G15" s="12" t="str">
-        <x:v>Chưa có dự đoán test</x:v>
       </x:c>
     </x:row>
     <x:row r="16" ht="35" customHeight="1">
@@ -4925,16 +6619,28 @@
         <x:v>F01</x:v>
       </x:c>
       <x:c r="B16" s="12" t="str">
-        <x:v>Rubber Vine</x:v>
-      </x:c>
-      <x:c r="C16" s="7" t="n">
+        <x:v>Rubber vine</x:v>
+      </x:c>
+      <x:c r="C16" s="40" t="n">
+        <x:v>0.983211964582725</x:v>
+      </x:c>
+      <x:c r="D16" s="40" t="n">
+        <x:v>0.0113127617175234</x:v>
+      </x:c>
+      <x:c r="E16" s="40" t="n">
+        <x:v>0.9587458745874587</x:v>
+      </x:c>
+      <x:c r="F16" s="40" t="n">
+        <x:v>0.0075620060972868</x:v>
+      </x:c>
+      <x:c r="G16" s="40" t="n">
+        <x:v>0.9707710923467124</x:v>
+      </x:c>
+      <x:c r="H16" s="40" t="n">
+        <x:v>0.0036855415833213</x:v>
+      </x:c>
+      <x:c r="I16" s="7" t="n">
         <x:v>202</x:v>
-      </x:c>
-      <x:c r="D16" s="40"/>
-      <x:c r="E16" s="40"/>
-      <x:c r="F16" s="40"/>
-      <x:c r="G16" s="12" t="str">
-        <x:v>Chưa có dự đoán test</x:v>
       </x:c>
     </x:row>
     <x:row r="17" ht="35" customHeight="1">
@@ -4942,16 +6648,28 @@
         <x:v>F01</x:v>
       </x:c>
       <x:c r="B17" s="12" t="str">
-        <x:v>Siam Weed</x:v>
-      </x:c>
-      <x:c r="C17" s="7" t="n">
+        <x:v>Siam weed</x:v>
+      </x:c>
+      <x:c r="C17" s="40" t="n">
+        <x:v>0.9845597320619704</x:v>
+      </x:c>
+      <x:c r="D17" s="40" t="n">
+        <x:v>0.0025189210908431</x:v>
+      </x:c>
+      <x:c r="E17" s="40" t="n">
+        <x:v>0.9875968992248062</x:v>
+      </x:c>
+      <x:c r="F17" s="40" t="n">
+        <x:v>0.0071047685193114</x:v>
+      </x:c>
+      <x:c r="G17" s="40" t="n">
+        <x:v>0.9860607170666786</x:v>
+      </x:c>
+      <x:c r="H17" s="40" t="n">
+        <x:v>0.0023848678337439</x:v>
+      </x:c>
+      <x:c r="I17" s="7" t="n">
         <x:v>215</x:v>
-      </x:c>
-      <x:c r="D17" s="40"/>
-      <x:c r="E17" s="40"/>
-      <x:c r="F17" s="40"/>
-      <x:c r="G17" s="12" t="str">
-        <x:v>Chưa có dự đoán test</x:v>
       </x:c>
     </x:row>
     <x:row r="18" ht="35" customHeight="1">
@@ -4959,16 +6677,28 @@
         <x:v>F01</x:v>
       </x:c>
       <x:c r="B18" s="12" t="str">
-        <x:v>Snake Weed</x:v>
-      </x:c>
-      <x:c r="C18" s="7" t="n">
+        <x:v>Snake weed</x:v>
+      </x:c>
+      <x:c r="C18" s="40" t="n">
+        <x:v>0.9519976015639116</x:v>
+      </x:c>
+      <x:c r="D18" s="40" t="n">
+        <x:v>0.0066243441448381</x:v>
+      </x:c>
+      <x:c r="E18" s="40" t="n">
+        <x:v>0.937908496732026</x:v>
+      </x:c>
+      <x:c r="F18" s="40" t="n">
+        <x:v>0.0157575992826682</x:v>
+      </x:c>
+      <x:c r="G18" s="40" t="n">
+        <x:v>0.94481898770742</x:v>
+      </x:c>
+      <x:c r="H18" s="40" t="n">
+        <x:v>0.005636929644577</x:v>
+      </x:c>
+      <x:c r="I18" s="7" t="n">
         <x:v>204</x:v>
-      </x:c>
-      <x:c r="D18" s="40"/>
-      <x:c r="E18" s="40"/>
-      <x:c r="F18" s="40"/>
-      <x:c r="G18" s="12" t="str">
-        <x:v>Chưa có dự đoán test</x:v>
       </x:c>
     </x:row>
     <x:row r="19" ht="35" customHeight="1">
@@ -4976,21 +6706,33 @@
         <x:v>F01</x:v>
       </x:c>
       <x:c r="B19" s="12" t="str">
-        <x:v>Negatives</x:v>
-      </x:c>
-      <x:c r="C19" s="7" t="n">
+        <x:v>Negative</x:v>
+      </x:c>
+      <x:c r="C19" s="40" t="n">
+        <x:v>0.9800489556246116</x:v>
+      </x:c>
+      <x:c r="D19" s="40" t="n">
+        <x:v>0.0010802279683081</x:v>
+      </x:c>
+      <x:c r="E19" s="40" t="n">
+        <x:v>0.9884742041712404</x:v>
+      </x:c>
+      <x:c r="F19" s="40" t="n">
+        <x:v>0.0025151348490427</x:v>
+      </x:c>
+      <x:c r="G19" s="40" t="n">
+        <x:v>0.984241786462544</x:v>
+      </x:c>
+      <x:c r="H19" s="40" t="n">
+        <x:v>0.001054537021134</x:v>
+      </x:c>
+      <x:c r="I19" s="7" t="n">
         <x:v>1822</x:v>
-      </x:c>
-      <x:c r="D19" s="40"/>
-      <x:c r="E19" s="40"/>
-      <x:c r="F19" s="40"/>
-      <x:c r="G19" s="12" t="str">
-        <x:v>Chưa có dự đoán test</x:v>
       </x:c>
     </x:row>
     <x:row r="22">
       <x:c r="A22" t="str">
-        <x:v>Chờ Bước 4: chưa có mean ± std, metric test hoặc dự đoán test. Không điền số val vào test.</x:v>
+        <x:v>Kết quả chung kết tính từ dự đoán test; mọi lựa chọn đã khóa trên val trước test.</x:v>
       </x:c>
     </x:row>
   </x:sheetData>

</xml_diff>